<commit_message>
Version 2.4.0: Weighted certification scoring with cap at 10.0
</commit_message>
<xml_diff>
--- a/comprehensive_grocery_certifications_COMPLETE.xlsx
+++ b/comprehensive_grocery_certifications_COMPLETE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StardogChampion\TBL-Grocery-Scanner---DEVELOPMENT-VERSION-Active-development-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429D31D4-4820-4825-A360-FB0BEA294B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389D842D-EDA8-46C5-B9F4-7C740FEAA84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3578,15 +3578,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -3612,7 +3606,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -31962,970 +31956,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="B7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="B12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="B13" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="B14" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B15" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B16" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B18" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B19" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B22" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B24" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="B25" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="B26" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="B27" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="B28" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="B29" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="B30" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="B31" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="B32" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="B33" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="B34" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="B35" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="B36" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="B37" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="B38" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="B39" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="B40" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="B41" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="B42" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="B43" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="B44" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="B45" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="B46" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="B47" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="B48" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="B49" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="B50" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="B51" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="B52" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="B53" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="B54" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="B55" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="B56" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="B57" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="B58" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="B59" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="B60" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="B61" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="B62" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="B63" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="B64" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="B65" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="B66" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="B67" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="B68" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="B69" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="B70" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="B71" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="B72" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="B73" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="B74" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="B75" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="B76" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="B77" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="B78" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="B79" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="B80" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="B81" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="B82" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="B83" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="B84" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="B85" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="B86" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="B87" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="B88" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="B89" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="B90" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="B91" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="B92" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="B93" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="B94" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="B95" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="B96" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="B97" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="B98" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="B99" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="B100" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="B101" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="B102" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="B103" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="B104" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="B105" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="B106" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
-    <hyperlink ref="B107" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="B108" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
-    <hyperlink ref="B109" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="B110" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
-    <hyperlink ref="B111" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="B112" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="B113" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="B114" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
-    <hyperlink ref="B115" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="B116" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
-    <hyperlink ref="B117" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="B118" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
-    <hyperlink ref="B119" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
-    <hyperlink ref="B120" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
-    <hyperlink ref="B121" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
-    <hyperlink ref="B122" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
-    <hyperlink ref="B123" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
-    <hyperlink ref="B124" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
-    <hyperlink ref="B125" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
-    <hyperlink ref="B126" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
-    <hyperlink ref="B127" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
-    <hyperlink ref="B128" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
-    <hyperlink ref="B129" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
-    <hyperlink ref="B130" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
-    <hyperlink ref="B131" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
-    <hyperlink ref="B132" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
-    <hyperlink ref="B133" r:id="rId131" xr:uid="{00000000-0004-0000-0000-000082000000}"/>
-    <hyperlink ref="B134" r:id="rId132" xr:uid="{00000000-0004-0000-0000-000083000000}"/>
-    <hyperlink ref="B135" r:id="rId133" xr:uid="{00000000-0004-0000-0000-000084000000}"/>
-    <hyperlink ref="B136" r:id="rId134" xr:uid="{00000000-0004-0000-0000-000085000000}"/>
-    <hyperlink ref="B137" r:id="rId135" xr:uid="{00000000-0004-0000-0000-000086000000}"/>
-    <hyperlink ref="B138" r:id="rId136" xr:uid="{00000000-0004-0000-0000-000087000000}"/>
-    <hyperlink ref="B139" r:id="rId137" xr:uid="{00000000-0004-0000-0000-000088000000}"/>
-    <hyperlink ref="B140" r:id="rId138" xr:uid="{00000000-0004-0000-0000-000089000000}"/>
-    <hyperlink ref="B141" r:id="rId139" xr:uid="{00000000-0004-0000-0000-00008A000000}"/>
-    <hyperlink ref="B142" r:id="rId140" xr:uid="{00000000-0004-0000-0000-00008B000000}"/>
-    <hyperlink ref="B143" r:id="rId141" xr:uid="{00000000-0004-0000-0000-00008C000000}"/>
-    <hyperlink ref="B144" r:id="rId142" xr:uid="{00000000-0004-0000-0000-00008D000000}"/>
-    <hyperlink ref="B145" r:id="rId143" xr:uid="{00000000-0004-0000-0000-00008E000000}"/>
-    <hyperlink ref="B146" r:id="rId144" xr:uid="{00000000-0004-0000-0000-00008F000000}"/>
-    <hyperlink ref="B147" r:id="rId145" xr:uid="{00000000-0004-0000-0000-000090000000}"/>
-    <hyperlink ref="B148" r:id="rId146" xr:uid="{00000000-0004-0000-0000-000091000000}"/>
-    <hyperlink ref="B149" r:id="rId147" xr:uid="{00000000-0004-0000-0000-000092000000}"/>
-    <hyperlink ref="B150" r:id="rId148" xr:uid="{00000000-0004-0000-0000-000093000000}"/>
-    <hyperlink ref="B151" r:id="rId149" xr:uid="{00000000-0004-0000-0000-000094000000}"/>
-    <hyperlink ref="B152" r:id="rId150" xr:uid="{00000000-0004-0000-0000-000095000000}"/>
-    <hyperlink ref="B153" r:id="rId151" xr:uid="{00000000-0004-0000-0000-000096000000}"/>
-    <hyperlink ref="B154" r:id="rId152" xr:uid="{00000000-0004-0000-0000-000097000000}"/>
-    <hyperlink ref="B155" r:id="rId153" xr:uid="{00000000-0004-0000-0000-000098000000}"/>
-    <hyperlink ref="B156" r:id="rId154" xr:uid="{00000000-0004-0000-0000-000099000000}"/>
-    <hyperlink ref="B157" r:id="rId155" xr:uid="{00000000-0004-0000-0000-00009A000000}"/>
-    <hyperlink ref="B158" r:id="rId156" xr:uid="{00000000-0004-0000-0000-00009B000000}"/>
-    <hyperlink ref="B159" r:id="rId157" xr:uid="{00000000-0004-0000-0000-00009C000000}"/>
-    <hyperlink ref="B160" r:id="rId158" xr:uid="{00000000-0004-0000-0000-00009D000000}"/>
-    <hyperlink ref="B161" r:id="rId159" xr:uid="{00000000-0004-0000-0000-00009E000000}"/>
-    <hyperlink ref="B162" r:id="rId160" xr:uid="{00000000-0004-0000-0000-00009F000000}"/>
-    <hyperlink ref="B163" r:id="rId161" xr:uid="{00000000-0004-0000-0000-0000A0000000}"/>
-    <hyperlink ref="B164" r:id="rId162" xr:uid="{00000000-0004-0000-0000-0000A1000000}"/>
-    <hyperlink ref="B165" r:id="rId163" xr:uid="{00000000-0004-0000-0000-0000A2000000}"/>
-    <hyperlink ref="B166" r:id="rId164" xr:uid="{00000000-0004-0000-0000-0000A3000000}"/>
-    <hyperlink ref="B167" r:id="rId165" xr:uid="{00000000-0004-0000-0000-0000A4000000}"/>
-    <hyperlink ref="B168" r:id="rId166" xr:uid="{00000000-0004-0000-0000-0000A5000000}"/>
-    <hyperlink ref="B169" r:id="rId167" xr:uid="{00000000-0004-0000-0000-0000A6000000}"/>
-    <hyperlink ref="B170" r:id="rId168" xr:uid="{00000000-0004-0000-0000-0000A7000000}"/>
-    <hyperlink ref="B171" r:id="rId169" xr:uid="{00000000-0004-0000-0000-0000A8000000}"/>
-    <hyperlink ref="B172" r:id="rId170" xr:uid="{00000000-0004-0000-0000-0000A9000000}"/>
-    <hyperlink ref="B173" r:id="rId171" xr:uid="{00000000-0004-0000-0000-0000AA000000}"/>
-    <hyperlink ref="B174" r:id="rId172" xr:uid="{00000000-0004-0000-0000-0000AB000000}"/>
-    <hyperlink ref="B175" r:id="rId173" xr:uid="{00000000-0004-0000-0000-0000AC000000}"/>
-    <hyperlink ref="B176" r:id="rId174" xr:uid="{00000000-0004-0000-0000-0000AD000000}"/>
-    <hyperlink ref="B177" r:id="rId175" xr:uid="{00000000-0004-0000-0000-0000AE000000}"/>
-    <hyperlink ref="B178" r:id="rId176" xr:uid="{00000000-0004-0000-0000-0000AF000000}"/>
-    <hyperlink ref="B179" r:id="rId177" xr:uid="{00000000-0004-0000-0000-0000B0000000}"/>
-    <hyperlink ref="B180" r:id="rId178" xr:uid="{00000000-0004-0000-0000-0000B1000000}"/>
-    <hyperlink ref="B181" r:id="rId179" xr:uid="{00000000-0004-0000-0000-0000B2000000}"/>
-    <hyperlink ref="B182" r:id="rId180" xr:uid="{00000000-0004-0000-0000-0000B3000000}"/>
-    <hyperlink ref="B183" r:id="rId181" xr:uid="{00000000-0004-0000-0000-0000B4000000}"/>
-    <hyperlink ref="B184" r:id="rId182" xr:uid="{00000000-0004-0000-0000-0000B5000000}"/>
-    <hyperlink ref="B185" r:id="rId183" xr:uid="{00000000-0004-0000-0000-0000B6000000}"/>
-    <hyperlink ref="B186" r:id="rId184" xr:uid="{00000000-0004-0000-0000-0000B7000000}"/>
-    <hyperlink ref="B187" r:id="rId185" xr:uid="{00000000-0004-0000-0000-0000B8000000}"/>
-    <hyperlink ref="B188" r:id="rId186" xr:uid="{00000000-0004-0000-0000-0000B9000000}"/>
-    <hyperlink ref="B189" r:id="rId187" xr:uid="{00000000-0004-0000-0000-0000BA000000}"/>
-    <hyperlink ref="B190" r:id="rId188" xr:uid="{00000000-0004-0000-0000-0000BB000000}"/>
-    <hyperlink ref="B191" r:id="rId189" xr:uid="{00000000-0004-0000-0000-0000BC000000}"/>
-    <hyperlink ref="B192" r:id="rId190" xr:uid="{00000000-0004-0000-0000-0000BD000000}"/>
-    <hyperlink ref="B193" r:id="rId191" xr:uid="{00000000-0004-0000-0000-0000BE000000}"/>
-    <hyperlink ref="B194" r:id="rId192" xr:uid="{00000000-0004-0000-0000-0000BF000000}"/>
-    <hyperlink ref="B195" r:id="rId193" xr:uid="{00000000-0004-0000-0000-0000C0000000}"/>
-    <hyperlink ref="B196" r:id="rId194" xr:uid="{00000000-0004-0000-0000-0000C1000000}"/>
-    <hyperlink ref="B197" r:id="rId195" xr:uid="{00000000-0004-0000-0000-0000C2000000}"/>
-    <hyperlink ref="B198" r:id="rId196" xr:uid="{00000000-0004-0000-0000-0000C3000000}"/>
-    <hyperlink ref="B199" r:id="rId197" xr:uid="{00000000-0004-0000-0000-0000C4000000}"/>
-    <hyperlink ref="B200" r:id="rId198" xr:uid="{00000000-0004-0000-0000-0000C5000000}"/>
-    <hyperlink ref="B201" r:id="rId199" xr:uid="{00000000-0004-0000-0000-0000C6000000}"/>
-    <hyperlink ref="B202" r:id="rId200" xr:uid="{00000000-0004-0000-0000-0000C7000000}"/>
-    <hyperlink ref="B203" r:id="rId201" xr:uid="{00000000-0004-0000-0000-0000C8000000}"/>
-    <hyperlink ref="B204" r:id="rId202" xr:uid="{00000000-0004-0000-0000-0000C9000000}"/>
-    <hyperlink ref="B205" r:id="rId203" xr:uid="{00000000-0004-0000-0000-0000CA000000}"/>
-    <hyperlink ref="B206" r:id="rId204" xr:uid="{00000000-0004-0000-0000-0000CB000000}"/>
-    <hyperlink ref="B207" r:id="rId205" xr:uid="{00000000-0004-0000-0000-0000CC000000}"/>
-    <hyperlink ref="B208" r:id="rId206" xr:uid="{00000000-0004-0000-0000-0000CD000000}"/>
-    <hyperlink ref="B209" r:id="rId207" xr:uid="{00000000-0004-0000-0000-0000CE000000}"/>
-    <hyperlink ref="B210" r:id="rId208" xr:uid="{00000000-0004-0000-0000-0000CF000000}"/>
-    <hyperlink ref="B211" r:id="rId209" xr:uid="{00000000-0004-0000-0000-0000D0000000}"/>
-    <hyperlink ref="B212" r:id="rId210" xr:uid="{00000000-0004-0000-0000-0000D1000000}"/>
-    <hyperlink ref="B213" r:id="rId211" xr:uid="{00000000-0004-0000-0000-0000D2000000}"/>
-    <hyperlink ref="B214" r:id="rId212" xr:uid="{00000000-0004-0000-0000-0000D3000000}"/>
-    <hyperlink ref="B215" r:id="rId213" xr:uid="{00000000-0004-0000-0000-0000D4000000}"/>
-    <hyperlink ref="B216" r:id="rId214" xr:uid="{00000000-0004-0000-0000-0000D5000000}"/>
-    <hyperlink ref="B217" r:id="rId215" xr:uid="{00000000-0004-0000-0000-0000D6000000}"/>
-    <hyperlink ref="B218" r:id="rId216" xr:uid="{00000000-0004-0000-0000-0000D7000000}"/>
-    <hyperlink ref="B219" r:id="rId217" xr:uid="{00000000-0004-0000-0000-0000D8000000}"/>
-    <hyperlink ref="B220" r:id="rId218" xr:uid="{00000000-0004-0000-0000-0000D9000000}"/>
-    <hyperlink ref="B221" r:id="rId219" xr:uid="{00000000-0004-0000-0000-0000DA000000}"/>
-    <hyperlink ref="B222" r:id="rId220" xr:uid="{00000000-0004-0000-0000-0000DB000000}"/>
-    <hyperlink ref="B223" r:id="rId221" xr:uid="{00000000-0004-0000-0000-0000DC000000}"/>
-    <hyperlink ref="B224" r:id="rId222" xr:uid="{00000000-0004-0000-0000-0000DD000000}"/>
-    <hyperlink ref="B225" r:id="rId223" xr:uid="{00000000-0004-0000-0000-0000DE000000}"/>
-    <hyperlink ref="B226" r:id="rId224" xr:uid="{00000000-0004-0000-0000-0000DF000000}"/>
-    <hyperlink ref="B227" r:id="rId225" xr:uid="{00000000-0004-0000-0000-0000E0000000}"/>
-    <hyperlink ref="B228" r:id="rId226" xr:uid="{00000000-0004-0000-0000-0000E1000000}"/>
-    <hyperlink ref="B229" r:id="rId227" xr:uid="{00000000-0004-0000-0000-0000E2000000}"/>
-    <hyperlink ref="B230" r:id="rId228" xr:uid="{00000000-0004-0000-0000-0000E3000000}"/>
-    <hyperlink ref="B231" r:id="rId229" xr:uid="{00000000-0004-0000-0000-0000E4000000}"/>
-    <hyperlink ref="B232" r:id="rId230" xr:uid="{00000000-0004-0000-0000-0000E5000000}"/>
-    <hyperlink ref="B233" r:id="rId231" xr:uid="{00000000-0004-0000-0000-0000E6000000}"/>
-    <hyperlink ref="B234" r:id="rId232" xr:uid="{00000000-0004-0000-0000-0000E7000000}"/>
-    <hyperlink ref="B235" r:id="rId233" xr:uid="{00000000-0004-0000-0000-0000E8000000}"/>
-    <hyperlink ref="B236" r:id="rId234" xr:uid="{00000000-0004-0000-0000-0000E9000000}"/>
-    <hyperlink ref="B237" r:id="rId235" xr:uid="{00000000-0004-0000-0000-0000EA000000}"/>
-    <hyperlink ref="B238" r:id="rId236" xr:uid="{00000000-0004-0000-0000-0000EB000000}"/>
-    <hyperlink ref="B239" r:id="rId237" xr:uid="{00000000-0004-0000-0000-0000EC000000}"/>
-    <hyperlink ref="B240" r:id="rId238" xr:uid="{00000000-0004-0000-0000-0000ED000000}"/>
-    <hyperlink ref="B241" r:id="rId239" xr:uid="{00000000-0004-0000-0000-0000EE000000}"/>
-    <hyperlink ref="B242" r:id="rId240" xr:uid="{00000000-0004-0000-0000-0000EF000000}"/>
-    <hyperlink ref="B243" r:id="rId241" xr:uid="{00000000-0004-0000-0000-0000F0000000}"/>
-    <hyperlink ref="B244" r:id="rId242" xr:uid="{00000000-0004-0000-0000-0000F1000000}"/>
-    <hyperlink ref="B245" r:id="rId243" xr:uid="{00000000-0004-0000-0000-0000F2000000}"/>
-    <hyperlink ref="B246" r:id="rId244" xr:uid="{00000000-0004-0000-0000-0000F3000000}"/>
-    <hyperlink ref="B247" r:id="rId245" xr:uid="{00000000-0004-0000-0000-0000F4000000}"/>
-    <hyperlink ref="B248" r:id="rId246" xr:uid="{00000000-0004-0000-0000-0000F5000000}"/>
-    <hyperlink ref="B249" r:id="rId247" xr:uid="{00000000-0004-0000-0000-0000F6000000}"/>
-    <hyperlink ref="B250" r:id="rId248" xr:uid="{00000000-0004-0000-0000-0000F7000000}"/>
-    <hyperlink ref="B251" r:id="rId249" xr:uid="{00000000-0004-0000-0000-0000F8000000}"/>
-    <hyperlink ref="B252" r:id="rId250" xr:uid="{00000000-0004-0000-0000-0000F9000000}"/>
-    <hyperlink ref="B253" r:id="rId251" xr:uid="{00000000-0004-0000-0000-0000FA000000}"/>
-    <hyperlink ref="B254" r:id="rId252" xr:uid="{00000000-0004-0000-0000-0000FB000000}"/>
-    <hyperlink ref="B255" r:id="rId253" xr:uid="{00000000-0004-0000-0000-0000FC000000}"/>
-    <hyperlink ref="B256" r:id="rId254" xr:uid="{00000000-0004-0000-0000-0000FD000000}"/>
-    <hyperlink ref="B257" r:id="rId255" xr:uid="{00000000-0004-0000-0000-0000FE000000}"/>
-    <hyperlink ref="B258" r:id="rId256" xr:uid="{00000000-0004-0000-0000-0000FF000000}"/>
-    <hyperlink ref="B259" r:id="rId257" xr:uid="{00000000-0004-0000-0000-000000010000}"/>
-    <hyperlink ref="B260" r:id="rId258" xr:uid="{00000000-0004-0000-0000-000001010000}"/>
-    <hyperlink ref="B261" r:id="rId259" xr:uid="{00000000-0004-0000-0000-000002010000}"/>
-    <hyperlink ref="B262" r:id="rId260" xr:uid="{00000000-0004-0000-0000-000003010000}"/>
-    <hyperlink ref="B263" r:id="rId261" xr:uid="{00000000-0004-0000-0000-000004010000}"/>
-    <hyperlink ref="B264" r:id="rId262" xr:uid="{00000000-0004-0000-0000-000005010000}"/>
-    <hyperlink ref="B265" r:id="rId263" xr:uid="{00000000-0004-0000-0000-000006010000}"/>
-    <hyperlink ref="B266" r:id="rId264" xr:uid="{00000000-0004-0000-0000-000007010000}"/>
-    <hyperlink ref="B267" r:id="rId265" xr:uid="{00000000-0004-0000-0000-000008010000}"/>
-    <hyperlink ref="B268" r:id="rId266" xr:uid="{00000000-0004-0000-0000-000009010000}"/>
-    <hyperlink ref="B269" r:id="rId267" xr:uid="{00000000-0004-0000-0000-00000A010000}"/>
-    <hyperlink ref="B270" r:id="rId268" xr:uid="{00000000-0004-0000-0000-00000B010000}"/>
-    <hyperlink ref="B271" r:id="rId269" xr:uid="{00000000-0004-0000-0000-00000C010000}"/>
-    <hyperlink ref="B272" r:id="rId270" xr:uid="{00000000-0004-0000-0000-00000D010000}"/>
-    <hyperlink ref="B273" r:id="rId271" xr:uid="{00000000-0004-0000-0000-00000E010000}"/>
-    <hyperlink ref="B274" r:id="rId272" xr:uid="{00000000-0004-0000-0000-00000F010000}"/>
-    <hyperlink ref="B275" r:id="rId273" xr:uid="{00000000-0004-0000-0000-000010010000}"/>
-    <hyperlink ref="B276" r:id="rId274" xr:uid="{00000000-0004-0000-0000-000011010000}"/>
-    <hyperlink ref="B277" r:id="rId275" xr:uid="{00000000-0004-0000-0000-000012010000}"/>
-    <hyperlink ref="B278" r:id="rId276" xr:uid="{00000000-0004-0000-0000-000013010000}"/>
-    <hyperlink ref="B279" r:id="rId277" xr:uid="{00000000-0004-0000-0000-000014010000}"/>
-    <hyperlink ref="B280" r:id="rId278" xr:uid="{00000000-0004-0000-0000-000015010000}"/>
-    <hyperlink ref="B281" r:id="rId279" xr:uid="{00000000-0004-0000-0000-000016010000}"/>
-    <hyperlink ref="B282" r:id="rId280" xr:uid="{00000000-0004-0000-0000-000017010000}"/>
-    <hyperlink ref="B283" r:id="rId281" xr:uid="{00000000-0004-0000-0000-000018010000}"/>
-    <hyperlink ref="B284" r:id="rId282" xr:uid="{00000000-0004-0000-0000-000019010000}"/>
-    <hyperlink ref="B285" r:id="rId283" xr:uid="{00000000-0004-0000-0000-00001A010000}"/>
-    <hyperlink ref="B286" r:id="rId284" xr:uid="{00000000-0004-0000-0000-00001B010000}"/>
-    <hyperlink ref="B287" r:id="rId285" xr:uid="{00000000-0004-0000-0000-00001C010000}"/>
-    <hyperlink ref="B288" r:id="rId286" xr:uid="{00000000-0004-0000-0000-00001D010000}"/>
-    <hyperlink ref="B289" r:id="rId287" xr:uid="{00000000-0004-0000-0000-00001E010000}"/>
-    <hyperlink ref="B290" r:id="rId288" xr:uid="{00000000-0004-0000-0000-00001F010000}"/>
-    <hyperlink ref="B291" r:id="rId289" xr:uid="{00000000-0004-0000-0000-000020010000}"/>
-    <hyperlink ref="B292" r:id="rId290" xr:uid="{00000000-0004-0000-0000-000021010000}"/>
-    <hyperlink ref="B293" r:id="rId291" xr:uid="{00000000-0004-0000-0000-000022010000}"/>
-    <hyperlink ref="B294" r:id="rId292" xr:uid="{00000000-0004-0000-0000-000023010000}"/>
-    <hyperlink ref="B295" r:id="rId293" xr:uid="{00000000-0004-0000-0000-000024010000}"/>
-    <hyperlink ref="B296" r:id="rId294" xr:uid="{00000000-0004-0000-0000-000025010000}"/>
-    <hyperlink ref="B297" r:id="rId295" xr:uid="{00000000-0004-0000-0000-000026010000}"/>
-    <hyperlink ref="B298" r:id="rId296" xr:uid="{00000000-0004-0000-0000-000027010000}"/>
-    <hyperlink ref="B299" r:id="rId297" xr:uid="{00000000-0004-0000-0000-000028010000}"/>
-    <hyperlink ref="B300" r:id="rId298" xr:uid="{00000000-0004-0000-0000-000029010000}"/>
-    <hyperlink ref="B301" r:id="rId299" xr:uid="{00000000-0004-0000-0000-00002A010000}"/>
-    <hyperlink ref="B302" r:id="rId300" xr:uid="{00000000-0004-0000-0000-00002B010000}"/>
-    <hyperlink ref="B303" r:id="rId301" xr:uid="{00000000-0004-0000-0000-00002C010000}"/>
-    <hyperlink ref="B304" r:id="rId302" xr:uid="{00000000-0004-0000-0000-00002D010000}"/>
-    <hyperlink ref="B305" r:id="rId303" xr:uid="{00000000-0004-0000-0000-00002E010000}"/>
-    <hyperlink ref="B306" r:id="rId304" xr:uid="{00000000-0004-0000-0000-00002F010000}"/>
-    <hyperlink ref="B307" r:id="rId305" xr:uid="{00000000-0004-0000-0000-000030010000}"/>
-    <hyperlink ref="B308" r:id="rId306" xr:uid="{00000000-0004-0000-0000-000031010000}"/>
-    <hyperlink ref="B309" r:id="rId307" xr:uid="{00000000-0004-0000-0000-000032010000}"/>
-    <hyperlink ref="B310" r:id="rId308" xr:uid="{00000000-0004-0000-0000-000033010000}"/>
-    <hyperlink ref="B311" r:id="rId309" xr:uid="{00000000-0004-0000-0000-000034010000}"/>
-    <hyperlink ref="B312" r:id="rId310" xr:uid="{00000000-0004-0000-0000-000035010000}"/>
-    <hyperlink ref="B313" r:id="rId311" xr:uid="{00000000-0004-0000-0000-000036010000}"/>
-    <hyperlink ref="B314" r:id="rId312" xr:uid="{00000000-0004-0000-0000-000037010000}"/>
-    <hyperlink ref="B315" r:id="rId313" xr:uid="{00000000-0004-0000-0000-000038010000}"/>
-    <hyperlink ref="B316" r:id="rId314" xr:uid="{00000000-0004-0000-0000-000039010000}"/>
-    <hyperlink ref="B317" r:id="rId315" xr:uid="{00000000-0004-0000-0000-00003A010000}"/>
-    <hyperlink ref="B318" r:id="rId316" xr:uid="{00000000-0004-0000-0000-00003B010000}"/>
-    <hyperlink ref="B319" r:id="rId317" xr:uid="{00000000-0004-0000-0000-00003C010000}"/>
-    <hyperlink ref="B320" r:id="rId318" xr:uid="{00000000-0004-0000-0000-00003D010000}"/>
-    <hyperlink ref="B321" r:id="rId319" xr:uid="{00000000-0004-0000-0000-00003E010000}"/>
-    <hyperlink ref="B322" r:id="rId320" xr:uid="{00000000-0004-0000-0000-00003F010000}"/>
-    <hyperlink ref="B323" r:id="rId321" xr:uid="{00000000-0004-0000-0000-000040010000}"/>
-    <hyperlink ref="B324" r:id="rId322" xr:uid="{00000000-0004-0000-0000-000041010000}"/>
-    <hyperlink ref="B325" r:id="rId323" xr:uid="{00000000-0004-0000-0000-000042010000}"/>
-    <hyperlink ref="B326" r:id="rId324" xr:uid="{00000000-0004-0000-0000-000043010000}"/>
-    <hyperlink ref="B327" r:id="rId325" xr:uid="{00000000-0004-0000-0000-000044010000}"/>
-    <hyperlink ref="B328" r:id="rId326" xr:uid="{00000000-0004-0000-0000-000045010000}"/>
-    <hyperlink ref="B329" r:id="rId327" xr:uid="{00000000-0004-0000-0000-000046010000}"/>
-    <hyperlink ref="B330" r:id="rId328" xr:uid="{00000000-0004-0000-0000-000047010000}"/>
-    <hyperlink ref="B331" r:id="rId329" xr:uid="{00000000-0004-0000-0000-000048010000}"/>
-    <hyperlink ref="B332" r:id="rId330" xr:uid="{00000000-0004-0000-0000-000049010000}"/>
-    <hyperlink ref="B333" r:id="rId331" xr:uid="{00000000-0004-0000-0000-00004A010000}"/>
-    <hyperlink ref="B334" r:id="rId332" xr:uid="{00000000-0004-0000-0000-00004B010000}"/>
-    <hyperlink ref="B335" r:id="rId333" xr:uid="{00000000-0004-0000-0000-00004C010000}"/>
-    <hyperlink ref="B336" r:id="rId334" xr:uid="{00000000-0004-0000-0000-00004D010000}"/>
-    <hyperlink ref="B337" r:id="rId335" xr:uid="{00000000-0004-0000-0000-00004E010000}"/>
-    <hyperlink ref="B338" r:id="rId336" xr:uid="{00000000-0004-0000-0000-00004F010000}"/>
-    <hyperlink ref="B339" r:id="rId337" xr:uid="{00000000-0004-0000-0000-000050010000}"/>
-    <hyperlink ref="B340" r:id="rId338" xr:uid="{00000000-0004-0000-0000-000051010000}"/>
-    <hyperlink ref="B341" r:id="rId339" xr:uid="{00000000-0004-0000-0000-000052010000}"/>
-    <hyperlink ref="B342" r:id="rId340" xr:uid="{00000000-0004-0000-0000-000053010000}"/>
-    <hyperlink ref="B343" r:id="rId341" xr:uid="{00000000-0004-0000-0000-000054010000}"/>
-    <hyperlink ref="B344" r:id="rId342" xr:uid="{00000000-0004-0000-0000-000055010000}"/>
-    <hyperlink ref="B345" r:id="rId343" xr:uid="{00000000-0004-0000-0000-000056010000}"/>
-    <hyperlink ref="B346" r:id="rId344" xr:uid="{00000000-0004-0000-0000-000057010000}"/>
-    <hyperlink ref="B347" r:id="rId345" xr:uid="{00000000-0004-0000-0000-000058010000}"/>
-    <hyperlink ref="B348" r:id="rId346" xr:uid="{00000000-0004-0000-0000-000059010000}"/>
-    <hyperlink ref="B349" r:id="rId347" xr:uid="{00000000-0004-0000-0000-00005A010000}"/>
-    <hyperlink ref="B350" r:id="rId348" xr:uid="{00000000-0004-0000-0000-00005B010000}"/>
-    <hyperlink ref="B351" r:id="rId349" xr:uid="{00000000-0004-0000-0000-00005C010000}"/>
-    <hyperlink ref="B352" r:id="rId350" xr:uid="{00000000-0004-0000-0000-00005D010000}"/>
-    <hyperlink ref="B353" r:id="rId351" xr:uid="{00000000-0004-0000-0000-00005E010000}"/>
-    <hyperlink ref="B354" r:id="rId352" xr:uid="{00000000-0004-0000-0000-00005F010000}"/>
-    <hyperlink ref="B355" r:id="rId353" xr:uid="{00000000-0004-0000-0000-000060010000}"/>
-    <hyperlink ref="B356" r:id="rId354" xr:uid="{00000000-0004-0000-0000-000061010000}"/>
-    <hyperlink ref="B357" r:id="rId355" xr:uid="{00000000-0004-0000-0000-000062010000}"/>
-    <hyperlink ref="B358" r:id="rId356" xr:uid="{00000000-0004-0000-0000-000063010000}"/>
-    <hyperlink ref="B359" r:id="rId357" xr:uid="{00000000-0004-0000-0000-000064010000}"/>
-    <hyperlink ref="B360" r:id="rId358" xr:uid="{00000000-0004-0000-0000-000065010000}"/>
-    <hyperlink ref="B361" r:id="rId359" xr:uid="{00000000-0004-0000-0000-000066010000}"/>
-    <hyperlink ref="B362" r:id="rId360" xr:uid="{00000000-0004-0000-0000-000067010000}"/>
-    <hyperlink ref="B363" r:id="rId361" xr:uid="{00000000-0004-0000-0000-000068010000}"/>
-    <hyperlink ref="B364" r:id="rId362" xr:uid="{00000000-0004-0000-0000-000069010000}"/>
-    <hyperlink ref="B365" r:id="rId363" xr:uid="{00000000-0004-0000-0000-00006A010000}"/>
-    <hyperlink ref="B366" r:id="rId364" xr:uid="{00000000-0004-0000-0000-00006B010000}"/>
-    <hyperlink ref="B367" r:id="rId365" xr:uid="{00000000-0004-0000-0000-00006C010000}"/>
-    <hyperlink ref="B368" r:id="rId366" xr:uid="{00000000-0004-0000-0000-00006D010000}"/>
-    <hyperlink ref="B369" r:id="rId367" xr:uid="{00000000-0004-0000-0000-00006E010000}"/>
-    <hyperlink ref="B370" r:id="rId368" xr:uid="{00000000-0004-0000-0000-00006F010000}"/>
-    <hyperlink ref="B371" r:id="rId369" xr:uid="{00000000-0004-0000-0000-000070010000}"/>
-    <hyperlink ref="B372" r:id="rId370" xr:uid="{00000000-0004-0000-0000-000071010000}"/>
-    <hyperlink ref="B373" r:id="rId371" xr:uid="{00000000-0004-0000-0000-000072010000}"/>
-    <hyperlink ref="B374" r:id="rId372" xr:uid="{00000000-0004-0000-0000-000073010000}"/>
-    <hyperlink ref="B375" r:id="rId373" xr:uid="{00000000-0004-0000-0000-000074010000}"/>
-    <hyperlink ref="B376" r:id="rId374" xr:uid="{00000000-0004-0000-0000-000075010000}"/>
-    <hyperlink ref="B377" r:id="rId375" xr:uid="{00000000-0004-0000-0000-000076010000}"/>
-    <hyperlink ref="B378" r:id="rId376" xr:uid="{00000000-0004-0000-0000-000077010000}"/>
-    <hyperlink ref="B379" r:id="rId377" xr:uid="{00000000-0004-0000-0000-000078010000}"/>
-    <hyperlink ref="B380" r:id="rId378" xr:uid="{00000000-0004-0000-0000-000079010000}"/>
-    <hyperlink ref="B381" r:id="rId379" xr:uid="{00000000-0004-0000-0000-00007A010000}"/>
-    <hyperlink ref="B382" r:id="rId380" xr:uid="{00000000-0004-0000-0000-00007B010000}"/>
-    <hyperlink ref="B383" r:id="rId381" xr:uid="{00000000-0004-0000-0000-00007C010000}"/>
-    <hyperlink ref="B384" r:id="rId382" xr:uid="{00000000-0004-0000-0000-00007D010000}"/>
-    <hyperlink ref="B385" r:id="rId383" xr:uid="{00000000-0004-0000-0000-00007E010000}"/>
-    <hyperlink ref="B386" r:id="rId384" xr:uid="{00000000-0004-0000-0000-00007F010000}"/>
-    <hyperlink ref="B387" r:id="rId385" xr:uid="{00000000-0004-0000-0000-000080010000}"/>
-    <hyperlink ref="B388" r:id="rId386" xr:uid="{00000000-0004-0000-0000-000081010000}"/>
-    <hyperlink ref="B389" r:id="rId387" xr:uid="{00000000-0004-0000-0000-000082010000}"/>
-    <hyperlink ref="B390" r:id="rId388" xr:uid="{00000000-0004-0000-0000-000083010000}"/>
-    <hyperlink ref="B391" r:id="rId389" xr:uid="{00000000-0004-0000-0000-000084010000}"/>
-    <hyperlink ref="B392" r:id="rId390" xr:uid="{00000000-0004-0000-0000-000085010000}"/>
-    <hyperlink ref="B393" r:id="rId391" xr:uid="{00000000-0004-0000-0000-000086010000}"/>
-    <hyperlink ref="B394" r:id="rId392" xr:uid="{00000000-0004-0000-0000-000087010000}"/>
-    <hyperlink ref="B395" r:id="rId393" xr:uid="{00000000-0004-0000-0000-000088010000}"/>
-    <hyperlink ref="B396" r:id="rId394" xr:uid="{00000000-0004-0000-0000-000089010000}"/>
-    <hyperlink ref="B397" r:id="rId395" xr:uid="{00000000-0004-0000-0000-00008A010000}"/>
-    <hyperlink ref="B398" r:id="rId396" xr:uid="{00000000-0004-0000-0000-00008B010000}"/>
-    <hyperlink ref="B399" r:id="rId397" xr:uid="{00000000-0004-0000-0000-00008C010000}"/>
-    <hyperlink ref="B400" r:id="rId398" xr:uid="{00000000-0004-0000-0000-00008D010000}"/>
-    <hyperlink ref="B401" r:id="rId399" xr:uid="{00000000-0004-0000-0000-00008E010000}"/>
-    <hyperlink ref="B402" r:id="rId400" xr:uid="{00000000-0004-0000-0000-00008F010000}"/>
-    <hyperlink ref="B403" r:id="rId401" xr:uid="{00000000-0004-0000-0000-000090010000}"/>
-    <hyperlink ref="B404" r:id="rId402" xr:uid="{00000000-0004-0000-0000-000091010000}"/>
-    <hyperlink ref="B405" r:id="rId403" xr:uid="{00000000-0004-0000-0000-000092010000}"/>
-    <hyperlink ref="B406" r:id="rId404" xr:uid="{00000000-0004-0000-0000-000093010000}"/>
-    <hyperlink ref="B407" r:id="rId405" xr:uid="{00000000-0004-0000-0000-000094010000}"/>
-    <hyperlink ref="B408" r:id="rId406" xr:uid="{00000000-0004-0000-0000-000095010000}"/>
-    <hyperlink ref="B409" r:id="rId407" xr:uid="{00000000-0004-0000-0000-000096010000}"/>
-    <hyperlink ref="B410" r:id="rId408" xr:uid="{00000000-0004-0000-0000-000097010000}"/>
-    <hyperlink ref="B411" r:id="rId409" xr:uid="{00000000-0004-0000-0000-000098010000}"/>
-    <hyperlink ref="B412" r:id="rId410" xr:uid="{00000000-0004-0000-0000-000099010000}"/>
-    <hyperlink ref="B413" r:id="rId411" xr:uid="{00000000-0004-0000-0000-00009A010000}"/>
-    <hyperlink ref="B414" r:id="rId412" xr:uid="{00000000-0004-0000-0000-00009B010000}"/>
-    <hyperlink ref="B415" r:id="rId413" xr:uid="{00000000-0004-0000-0000-00009C010000}"/>
-    <hyperlink ref="B416" r:id="rId414" xr:uid="{00000000-0004-0000-0000-00009D010000}"/>
-    <hyperlink ref="B417" r:id="rId415" xr:uid="{00000000-0004-0000-0000-00009E010000}"/>
-    <hyperlink ref="B418" r:id="rId416" xr:uid="{00000000-0004-0000-0000-00009F010000}"/>
-    <hyperlink ref="B419" r:id="rId417" xr:uid="{00000000-0004-0000-0000-0000A0010000}"/>
-    <hyperlink ref="B420" r:id="rId418" xr:uid="{00000000-0004-0000-0000-0000A1010000}"/>
-    <hyperlink ref="B421" r:id="rId419" xr:uid="{00000000-0004-0000-0000-0000A2010000}"/>
-    <hyperlink ref="B422" r:id="rId420" xr:uid="{00000000-0004-0000-0000-0000A3010000}"/>
-    <hyperlink ref="B423" r:id="rId421" xr:uid="{00000000-0004-0000-0000-0000A4010000}"/>
-    <hyperlink ref="B424" r:id="rId422" xr:uid="{00000000-0004-0000-0000-0000A5010000}"/>
-    <hyperlink ref="B425" r:id="rId423" xr:uid="{00000000-0004-0000-0000-0000A6010000}"/>
-    <hyperlink ref="B426" r:id="rId424" xr:uid="{00000000-0004-0000-0000-0000A7010000}"/>
-    <hyperlink ref="B427" r:id="rId425" xr:uid="{00000000-0004-0000-0000-0000A8010000}"/>
-    <hyperlink ref="B428" r:id="rId426" xr:uid="{00000000-0004-0000-0000-0000A9010000}"/>
-    <hyperlink ref="B429" r:id="rId427" xr:uid="{00000000-0004-0000-0000-0000AA010000}"/>
-    <hyperlink ref="B430" r:id="rId428" xr:uid="{00000000-0004-0000-0000-0000AB010000}"/>
-    <hyperlink ref="B431" r:id="rId429" xr:uid="{00000000-0004-0000-0000-0000AC010000}"/>
-    <hyperlink ref="B432" r:id="rId430" xr:uid="{00000000-0004-0000-0000-0000AD010000}"/>
-    <hyperlink ref="B433" r:id="rId431" xr:uid="{00000000-0004-0000-0000-0000AE010000}"/>
-    <hyperlink ref="B434" r:id="rId432" xr:uid="{00000000-0004-0000-0000-0000AF010000}"/>
-    <hyperlink ref="B435" r:id="rId433" xr:uid="{00000000-0004-0000-0000-0000B0010000}"/>
-    <hyperlink ref="B436" r:id="rId434" xr:uid="{00000000-0004-0000-0000-0000B1010000}"/>
-    <hyperlink ref="B437" r:id="rId435" xr:uid="{00000000-0004-0000-0000-0000B2010000}"/>
-    <hyperlink ref="B438" r:id="rId436" xr:uid="{00000000-0004-0000-0000-0000B3010000}"/>
-    <hyperlink ref="B439" r:id="rId437" xr:uid="{00000000-0004-0000-0000-0000B4010000}"/>
-    <hyperlink ref="B440" r:id="rId438" xr:uid="{00000000-0004-0000-0000-0000B5010000}"/>
-    <hyperlink ref="B441" r:id="rId439" xr:uid="{00000000-0004-0000-0000-0000B6010000}"/>
-    <hyperlink ref="B442" r:id="rId440" xr:uid="{00000000-0004-0000-0000-0000B7010000}"/>
-    <hyperlink ref="B443" r:id="rId441" xr:uid="{00000000-0004-0000-0000-0000B8010000}"/>
-    <hyperlink ref="B444" r:id="rId442" xr:uid="{00000000-0004-0000-0000-0000B9010000}"/>
-    <hyperlink ref="B445" r:id="rId443" xr:uid="{00000000-0004-0000-0000-0000BA010000}"/>
-    <hyperlink ref="B446" r:id="rId444" xr:uid="{00000000-0004-0000-0000-0000BB010000}"/>
-    <hyperlink ref="B447" r:id="rId445" xr:uid="{00000000-0004-0000-0000-0000BC010000}"/>
-    <hyperlink ref="B448" r:id="rId446" xr:uid="{00000000-0004-0000-0000-0000BD010000}"/>
-    <hyperlink ref="B449" r:id="rId447" xr:uid="{00000000-0004-0000-0000-0000BE010000}"/>
-    <hyperlink ref="B450" r:id="rId448" xr:uid="{00000000-0004-0000-0000-0000BF010000}"/>
-    <hyperlink ref="B451" r:id="rId449" xr:uid="{00000000-0004-0000-0000-0000C0010000}"/>
-    <hyperlink ref="B452" r:id="rId450" xr:uid="{00000000-0004-0000-0000-0000C1010000}"/>
-    <hyperlink ref="B453" r:id="rId451" xr:uid="{00000000-0004-0000-0000-0000C2010000}"/>
-    <hyperlink ref="B454" r:id="rId452" xr:uid="{00000000-0004-0000-0000-0000C3010000}"/>
-    <hyperlink ref="B455" r:id="rId453" xr:uid="{00000000-0004-0000-0000-0000C4010000}"/>
-    <hyperlink ref="B456" r:id="rId454" xr:uid="{00000000-0004-0000-0000-0000C5010000}"/>
-    <hyperlink ref="B457" r:id="rId455" xr:uid="{00000000-0004-0000-0000-0000C6010000}"/>
-    <hyperlink ref="B458" r:id="rId456" xr:uid="{00000000-0004-0000-0000-0000C7010000}"/>
-    <hyperlink ref="B459" r:id="rId457" xr:uid="{00000000-0004-0000-0000-0000C8010000}"/>
-    <hyperlink ref="B460" r:id="rId458" xr:uid="{00000000-0004-0000-0000-0000C9010000}"/>
-    <hyperlink ref="B461" r:id="rId459" xr:uid="{00000000-0004-0000-0000-0000CA010000}"/>
-    <hyperlink ref="B462" r:id="rId460" xr:uid="{00000000-0004-0000-0000-0000CB010000}"/>
-    <hyperlink ref="B463" r:id="rId461" xr:uid="{00000000-0004-0000-0000-0000CC010000}"/>
-    <hyperlink ref="B464" r:id="rId462" xr:uid="{00000000-0004-0000-0000-0000CD010000}"/>
-    <hyperlink ref="B465" r:id="rId463" xr:uid="{00000000-0004-0000-0000-0000CE010000}"/>
-    <hyperlink ref="B466" r:id="rId464" xr:uid="{00000000-0004-0000-0000-0000CF010000}"/>
-    <hyperlink ref="B467" r:id="rId465" xr:uid="{00000000-0004-0000-0000-0000D0010000}"/>
-    <hyperlink ref="B468" r:id="rId466" xr:uid="{00000000-0004-0000-0000-0000D1010000}"/>
-    <hyperlink ref="B469" r:id="rId467" xr:uid="{00000000-0004-0000-0000-0000D2010000}"/>
-    <hyperlink ref="B470" r:id="rId468" xr:uid="{00000000-0004-0000-0000-0000D3010000}"/>
-    <hyperlink ref="B471" r:id="rId469" xr:uid="{00000000-0004-0000-0000-0000D4010000}"/>
-    <hyperlink ref="B472" r:id="rId470" xr:uid="{00000000-0004-0000-0000-0000D5010000}"/>
-    <hyperlink ref="B473" r:id="rId471" xr:uid="{00000000-0004-0000-0000-0000D6010000}"/>
-    <hyperlink ref="B474" r:id="rId472" xr:uid="{00000000-0004-0000-0000-0000D7010000}"/>
-    <hyperlink ref="B475" r:id="rId473" xr:uid="{00000000-0004-0000-0000-0000D8010000}"/>
-    <hyperlink ref="B476" r:id="rId474" xr:uid="{00000000-0004-0000-0000-0000D9010000}"/>
-    <hyperlink ref="B477" r:id="rId475" xr:uid="{00000000-0004-0000-0000-0000DA010000}"/>
-    <hyperlink ref="B478" r:id="rId476" xr:uid="{00000000-0004-0000-0000-0000DB010000}"/>
-    <hyperlink ref="B479" r:id="rId477" xr:uid="{00000000-0004-0000-0000-0000DC010000}"/>
-    <hyperlink ref="B480" r:id="rId478" xr:uid="{00000000-0004-0000-0000-0000DD010000}"/>
-    <hyperlink ref="B481" r:id="rId479" xr:uid="{00000000-0004-0000-0000-0000DE010000}"/>
-    <hyperlink ref="B482" r:id="rId480" xr:uid="{00000000-0004-0000-0000-0000DF010000}"/>
-    <hyperlink ref="B483" r:id="rId481" xr:uid="{00000000-0004-0000-0000-0000E0010000}"/>
-    <hyperlink ref="B484" r:id="rId482" xr:uid="{00000000-0004-0000-0000-0000E1010000}"/>
-    <hyperlink ref="B485" r:id="rId483" xr:uid="{00000000-0004-0000-0000-0000E2010000}"/>
-    <hyperlink ref="B486" r:id="rId484" xr:uid="{00000000-0004-0000-0000-0000E3010000}"/>
-    <hyperlink ref="B487" r:id="rId485" xr:uid="{00000000-0004-0000-0000-0000E4010000}"/>
-    <hyperlink ref="B488" r:id="rId486" xr:uid="{00000000-0004-0000-0000-0000E5010000}"/>
-    <hyperlink ref="B489" r:id="rId487" xr:uid="{00000000-0004-0000-0000-0000E6010000}"/>
-    <hyperlink ref="B490" r:id="rId488" xr:uid="{00000000-0004-0000-0000-0000E7010000}"/>
-    <hyperlink ref="B491" r:id="rId489" xr:uid="{00000000-0004-0000-0000-0000E8010000}"/>
-    <hyperlink ref="B492" r:id="rId490" xr:uid="{00000000-0004-0000-0000-0000E9010000}"/>
-    <hyperlink ref="B493" r:id="rId491" xr:uid="{00000000-0004-0000-0000-0000EA010000}"/>
-    <hyperlink ref="B494" r:id="rId492" xr:uid="{00000000-0004-0000-0000-0000EB010000}"/>
-    <hyperlink ref="B495" r:id="rId493" xr:uid="{00000000-0004-0000-0000-0000EC010000}"/>
-    <hyperlink ref="B496" r:id="rId494" xr:uid="{00000000-0004-0000-0000-0000ED010000}"/>
-    <hyperlink ref="B497" r:id="rId495" xr:uid="{00000000-0004-0000-0000-0000EE010000}"/>
-    <hyperlink ref="B498" r:id="rId496" xr:uid="{00000000-0004-0000-0000-0000EF010000}"/>
-    <hyperlink ref="B499" r:id="rId497" xr:uid="{00000000-0004-0000-0000-0000F0010000}"/>
-    <hyperlink ref="B500" r:id="rId498" xr:uid="{00000000-0004-0000-0000-0000F1010000}"/>
-    <hyperlink ref="B501" r:id="rId499" xr:uid="{00000000-0004-0000-0000-0000F2010000}"/>
-    <hyperlink ref="B502" r:id="rId500" xr:uid="{00000000-0004-0000-0000-0000F3010000}"/>
-    <hyperlink ref="B503" r:id="rId501" xr:uid="{00000000-0004-0000-0000-0000F4010000}"/>
-    <hyperlink ref="B504" r:id="rId502" xr:uid="{00000000-0004-0000-0000-0000F5010000}"/>
-    <hyperlink ref="B505" r:id="rId503" xr:uid="{00000000-0004-0000-0000-0000F6010000}"/>
-    <hyperlink ref="B506" r:id="rId504" xr:uid="{00000000-0004-0000-0000-0000F7010000}"/>
-    <hyperlink ref="B507" r:id="rId505" xr:uid="{00000000-0004-0000-0000-0000F8010000}"/>
-    <hyperlink ref="B508" r:id="rId506" xr:uid="{00000000-0004-0000-0000-0000F9010000}"/>
-    <hyperlink ref="B509" r:id="rId507" xr:uid="{00000000-0004-0000-0000-0000FA010000}"/>
-    <hyperlink ref="B510" r:id="rId508" xr:uid="{00000000-0004-0000-0000-0000FB010000}"/>
-    <hyperlink ref="B511" r:id="rId509" xr:uid="{00000000-0004-0000-0000-0000FC010000}"/>
-    <hyperlink ref="B512" r:id="rId510" xr:uid="{00000000-0004-0000-0000-0000FD010000}"/>
-    <hyperlink ref="B513" r:id="rId511" xr:uid="{00000000-0004-0000-0000-0000FE010000}"/>
-    <hyperlink ref="B514" r:id="rId512" xr:uid="{00000000-0004-0000-0000-0000FF010000}"/>
-    <hyperlink ref="B515" r:id="rId513" xr:uid="{00000000-0004-0000-0000-000000020000}"/>
-    <hyperlink ref="B516" r:id="rId514" xr:uid="{00000000-0004-0000-0000-000001020000}"/>
-    <hyperlink ref="B517" r:id="rId515" xr:uid="{00000000-0004-0000-0000-000002020000}"/>
-    <hyperlink ref="B518" r:id="rId516" xr:uid="{00000000-0004-0000-0000-000003020000}"/>
-    <hyperlink ref="B519" r:id="rId517" xr:uid="{00000000-0004-0000-0000-000004020000}"/>
-    <hyperlink ref="B520" r:id="rId518" xr:uid="{00000000-0004-0000-0000-000005020000}"/>
-    <hyperlink ref="B521" r:id="rId519" xr:uid="{00000000-0004-0000-0000-000006020000}"/>
-    <hyperlink ref="B522" r:id="rId520" xr:uid="{00000000-0004-0000-0000-000007020000}"/>
-    <hyperlink ref="B523" r:id="rId521" xr:uid="{00000000-0004-0000-0000-000008020000}"/>
-    <hyperlink ref="B524" r:id="rId522" xr:uid="{00000000-0004-0000-0000-000009020000}"/>
-    <hyperlink ref="B525" r:id="rId523" xr:uid="{00000000-0004-0000-0000-00000A020000}"/>
-    <hyperlink ref="B526" r:id="rId524" xr:uid="{00000000-0004-0000-0000-00000B020000}"/>
-    <hyperlink ref="B527" r:id="rId525" xr:uid="{00000000-0004-0000-0000-00000C020000}"/>
-    <hyperlink ref="B528" r:id="rId526" xr:uid="{00000000-0004-0000-0000-00000D020000}"/>
-    <hyperlink ref="B529" r:id="rId527" xr:uid="{00000000-0004-0000-0000-00000E020000}"/>
-    <hyperlink ref="B530" r:id="rId528" xr:uid="{00000000-0004-0000-0000-00000F020000}"/>
-    <hyperlink ref="B531" r:id="rId529" xr:uid="{00000000-0004-0000-0000-000010020000}"/>
-    <hyperlink ref="B532" r:id="rId530" xr:uid="{00000000-0004-0000-0000-000011020000}"/>
-    <hyperlink ref="B533" r:id="rId531" xr:uid="{00000000-0004-0000-0000-000012020000}"/>
-    <hyperlink ref="B534" r:id="rId532" xr:uid="{00000000-0004-0000-0000-000013020000}"/>
-    <hyperlink ref="B535" r:id="rId533" xr:uid="{00000000-0004-0000-0000-000014020000}"/>
-    <hyperlink ref="B536" r:id="rId534" xr:uid="{00000000-0004-0000-0000-000015020000}"/>
-    <hyperlink ref="B537" r:id="rId535" xr:uid="{00000000-0004-0000-0000-000016020000}"/>
-    <hyperlink ref="B538" r:id="rId536" xr:uid="{00000000-0004-0000-0000-000017020000}"/>
-    <hyperlink ref="B539" r:id="rId537" xr:uid="{00000000-0004-0000-0000-000018020000}"/>
-    <hyperlink ref="B540" r:id="rId538" xr:uid="{00000000-0004-0000-0000-000019020000}"/>
-    <hyperlink ref="B541" r:id="rId539" xr:uid="{00000000-0004-0000-0000-00001A020000}"/>
-    <hyperlink ref="B542" r:id="rId540" xr:uid="{00000000-0004-0000-0000-00001B020000}"/>
-    <hyperlink ref="B543" r:id="rId541" xr:uid="{00000000-0004-0000-0000-00001C020000}"/>
-    <hyperlink ref="B544" r:id="rId542" xr:uid="{00000000-0004-0000-0000-00001D020000}"/>
-    <hyperlink ref="B545" r:id="rId543" xr:uid="{00000000-0004-0000-0000-00001E020000}"/>
-    <hyperlink ref="B546" r:id="rId544" xr:uid="{00000000-0004-0000-0000-00001F020000}"/>
-    <hyperlink ref="B547" r:id="rId545" xr:uid="{00000000-0004-0000-0000-000020020000}"/>
-    <hyperlink ref="B548" r:id="rId546" xr:uid="{00000000-0004-0000-0000-000021020000}"/>
-    <hyperlink ref="B549" r:id="rId547" xr:uid="{00000000-0004-0000-0000-000022020000}"/>
-    <hyperlink ref="B550" r:id="rId548" xr:uid="{00000000-0004-0000-0000-000023020000}"/>
-    <hyperlink ref="B551" r:id="rId549" xr:uid="{00000000-0004-0000-0000-000024020000}"/>
-    <hyperlink ref="B552" r:id="rId550" xr:uid="{00000000-0004-0000-0000-000025020000}"/>
-    <hyperlink ref="B553" r:id="rId551" xr:uid="{00000000-0004-0000-0000-000026020000}"/>
-    <hyperlink ref="B554" r:id="rId552" xr:uid="{00000000-0004-0000-0000-000027020000}"/>
-    <hyperlink ref="B555" r:id="rId553" xr:uid="{00000000-0004-0000-0000-000028020000}"/>
-    <hyperlink ref="B556" r:id="rId554" xr:uid="{00000000-0004-0000-0000-000029020000}"/>
-    <hyperlink ref="B557" r:id="rId555" xr:uid="{00000000-0004-0000-0000-00002A020000}"/>
-    <hyperlink ref="B558" r:id="rId556" xr:uid="{00000000-0004-0000-0000-00002B020000}"/>
-    <hyperlink ref="B559" r:id="rId557" xr:uid="{00000000-0004-0000-0000-00002C020000}"/>
-    <hyperlink ref="B560" r:id="rId558" xr:uid="{00000000-0004-0000-0000-00002D020000}"/>
-    <hyperlink ref="B561" r:id="rId559" xr:uid="{00000000-0004-0000-0000-00002E020000}"/>
-    <hyperlink ref="B562" r:id="rId560" xr:uid="{00000000-0004-0000-0000-00002F020000}"/>
-    <hyperlink ref="B563" r:id="rId561" xr:uid="{00000000-0004-0000-0000-000030020000}"/>
-    <hyperlink ref="B564" r:id="rId562" xr:uid="{00000000-0004-0000-0000-000031020000}"/>
-    <hyperlink ref="B565" r:id="rId563" xr:uid="{00000000-0004-0000-0000-000032020000}"/>
-    <hyperlink ref="B566" r:id="rId564" xr:uid="{00000000-0004-0000-0000-000033020000}"/>
-    <hyperlink ref="B567" r:id="rId565" xr:uid="{00000000-0004-0000-0000-000034020000}"/>
-    <hyperlink ref="B568" r:id="rId566" xr:uid="{00000000-0004-0000-0000-000035020000}"/>
-    <hyperlink ref="B569" r:id="rId567" xr:uid="{00000000-0004-0000-0000-000036020000}"/>
-    <hyperlink ref="B570" r:id="rId568" xr:uid="{00000000-0004-0000-0000-000037020000}"/>
-    <hyperlink ref="B571" r:id="rId569" xr:uid="{00000000-0004-0000-0000-000038020000}"/>
-    <hyperlink ref="B572" r:id="rId570" xr:uid="{00000000-0004-0000-0000-000039020000}"/>
-    <hyperlink ref="B573" r:id="rId571" xr:uid="{00000000-0004-0000-0000-00003A020000}"/>
-    <hyperlink ref="B574" r:id="rId572" xr:uid="{00000000-0004-0000-0000-00003B020000}"/>
-    <hyperlink ref="B575" r:id="rId573" xr:uid="{00000000-0004-0000-0000-00003C020000}"/>
-    <hyperlink ref="B576" r:id="rId574" xr:uid="{00000000-0004-0000-0000-00003D020000}"/>
-    <hyperlink ref="B577" r:id="rId575" xr:uid="{00000000-0004-0000-0000-00003E020000}"/>
-    <hyperlink ref="B578" r:id="rId576" xr:uid="{00000000-0004-0000-0000-00003F020000}"/>
-    <hyperlink ref="B579" r:id="rId577" xr:uid="{00000000-0004-0000-0000-000040020000}"/>
-    <hyperlink ref="B580" r:id="rId578" xr:uid="{00000000-0004-0000-0000-000041020000}"/>
-    <hyperlink ref="B581" r:id="rId579" xr:uid="{00000000-0004-0000-0000-000042020000}"/>
-    <hyperlink ref="B582" r:id="rId580" xr:uid="{00000000-0004-0000-0000-000043020000}"/>
-    <hyperlink ref="B583" r:id="rId581" xr:uid="{00000000-0004-0000-0000-000044020000}"/>
-    <hyperlink ref="B584" r:id="rId582" xr:uid="{00000000-0004-0000-0000-000045020000}"/>
-    <hyperlink ref="B585" r:id="rId583" xr:uid="{00000000-0004-0000-0000-000046020000}"/>
-    <hyperlink ref="B586" r:id="rId584" xr:uid="{00000000-0004-0000-0000-000047020000}"/>
-    <hyperlink ref="B587" r:id="rId585" xr:uid="{00000000-0004-0000-0000-000048020000}"/>
-    <hyperlink ref="B588" r:id="rId586" xr:uid="{00000000-0004-0000-0000-000049020000}"/>
-    <hyperlink ref="B589" r:id="rId587" xr:uid="{00000000-0004-0000-0000-00004A020000}"/>
-    <hyperlink ref="B590" r:id="rId588" xr:uid="{00000000-0004-0000-0000-00004B020000}"/>
-    <hyperlink ref="B591" r:id="rId589" xr:uid="{00000000-0004-0000-0000-00004C020000}"/>
-    <hyperlink ref="B592" r:id="rId590" xr:uid="{00000000-0004-0000-0000-00004D020000}"/>
-    <hyperlink ref="B593" r:id="rId591" xr:uid="{00000000-0004-0000-0000-00004E020000}"/>
-    <hyperlink ref="B594" r:id="rId592" xr:uid="{00000000-0004-0000-0000-00004F020000}"/>
-    <hyperlink ref="B595" r:id="rId593" xr:uid="{00000000-0004-0000-0000-000050020000}"/>
-    <hyperlink ref="B596" r:id="rId594" xr:uid="{00000000-0004-0000-0000-000051020000}"/>
-    <hyperlink ref="B597" r:id="rId595" xr:uid="{00000000-0004-0000-0000-000052020000}"/>
-    <hyperlink ref="B598" r:id="rId596" xr:uid="{00000000-0004-0000-0000-000053020000}"/>
-    <hyperlink ref="B599" r:id="rId597" xr:uid="{00000000-0004-0000-0000-000054020000}"/>
-    <hyperlink ref="B600" r:id="rId598" xr:uid="{00000000-0004-0000-0000-000055020000}"/>
-    <hyperlink ref="B601" r:id="rId599" xr:uid="{00000000-0004-0000-0000-000056020000}"/>
-    <hyperlink ref="B602" r:id="rId600" xr:uid="{00000000-0004-0000-0000-000057020000}"/>
-    <hyperlink ref="B603" r:id="rId601" xr:uid="{00000000-0004-0000-0000-000058020000}"/>
-    <hyperlink ref="B604" r:id="rId602" xr:uid="{00000000-0004-0000-0000-000059020000}"/>
-    <hyperlink ref="B605" r:id="rId603" xr:uid="{00000000-0004-0000-0000-00005A020000}"/>
-    <hyperlink ref="B606" r:id="rId604" xr:uid="{00000000-0004-0000-0000-00005B020000}"/>
-    <hyperlink ref="B607" r:id="rId605" xr:uid="{00000000-0004-0000-0000-00005C020000}"/>
-    <hyperlink ref="B608" r:id="rId606" xr:uid="{00000000-0004-0000-0000-00005D020000}"/>
-    <hyperlink ref="B609" r:id="rId607" xr:uid="{00000000-0004-0000-0000-00005E020000}"/>
-    <hyperlink ref="B610" r:id="rId608" xr:uid="{00000000-0004-0000-0000-00005F020000}"/>
-    <hyperlink ref="B611" r:id="rId609" xr:uid="{00000000-0004-0000-0000-000060020000}"/>
-    <hyperlink ref="B612" r:id="rId610" xr:uid="{00000000-0004-0000-0000-000061020000}"/>
-    <hyperlink ref="B613" r:id="rId611" xr:uid="{00000000-0004-0000-0000-000062020000}"/>
-    <hyperlink ref="B614" r:id="rId612" xr:uid="{00000000-0004-0000-0000-000063020000}"/>
-    <hyperlink ref="B615" r:id="rId613" xr:uid="{00000000-0004-0000-0000-000064020000}"/>
-    <hyperlink ref="B616" r:id="rId614" xr:uid="{00000000-0004-0000-0000-000065020000}"/>
-    <hyperlink ref="B617" r:id="rId615" xr:uid="{00000000-0004-0000-0000-000066020000}"/>
-    <hyperlink ref="B618" r:id="rId616" xr:uid="{00000000-0004-0000-0000-000067020000}"/>
-    <hyperlink ref="B619" r:id="rId617" xr:uid="{00000000-0004-0000-0000-000068020000}"/>
-    <hyperlink ref="B620" r:id="rId618" xr:uid="{00000000-0004-0000-0000-000069020000}"/>
-    <hyperlink ref="B621" r:id="rId619" xr:uid="{00000000-0004-0000-0000-00006A020000}"/>
-    <hyperlink ref="B622" r:id="rId620" xr:uid="{00000000-0004-0000-0000-00006B020000}"/>
-    <hyperlink ref="B623" r:id="rId621" xr:uid="{00000000-0004-0000-0000-00006C020000}"/>
-    <hyperlink ref="B624" r:id="rId622" xr:uid="{00000000-0004-0000-0000-00006D020000}"/>
-    <hyperlink ref="B625" r:id="rId623" xr:uid="{00000000-0004-0000-0000-00006E020000}"/>
-    <hyperlink ref="B626" r:id="rId624" xr:uid="{00000000-0004-0000-0000-00006F020000}"/>
-    <hyperlink ref="B627" r:id="rId625" xr:uid="{00000000-0004-0000-0000-000070020000}"/>
-    <hyperlink ref="B628" r:id="rId626" xr:uid="{00000000-0004-0000-0000-000071020000}"/>
-    <hyperlink ref="B629" r:id="rId627" xr:uid="{00000000-0004-0000-0000-000072020000}"/>
-    <hyperlink ref="B630" r:id="rId628" xr:uid="{00000000-0004-0000-0000-000073020000}"/>
-    <hyperlink ref="B631" r:id="rId629" xr:uid="{00000000-0004-0000-0000-000074020000}"/>
-    <hyperlink ref="B632" r:id="rId630" xr:uid="{00000000-0004-0000-0000-000075020000}"/>
-    <hyperlink ref="B633" r:id="rId631" xr:uid="{00000000-0004-0000-0000-000076020000}"/>
-    <hyperlink ref="B634" r:id="rId632" xr:uid="{00000000-0004-0000-0000-000077020000}"/>
-    <hyperlink ref="B635" r:id="rId633" xr:uid="{00000000-0004-0000-0000-000078020000}"/>
-    <hyperlink ref="B636" r:id="rId634" xr:uid="{00000000-0004-0000-0000-000079020000}"/>
-    <hyperlink ref="B637" r:id="rId635" xr:uid="{00000000-0004-0000-0000-00007A020000}"/>
-    <hyperlink ref="B638" r:id="rId636" xr:uid="{00000000-0004-0000-0000-00007B020000}"/>
-    <hyperlink ref="B639" r:id="rId637" xr:uid="{00000000-0004-0000-0000-00007C020000}"/>
-    <hyperlink ref="B640" r:id="rId638" xr:uid="{00000000-0004-0000-0000-00007D020000}"/>
-    <hyperlink ref="B641" r:id="rId639" xr:uid="{00000000-0004-0000-0000-00007E020000}"/>
-    <hyperlink ref="B642" r:id="rId640" xr:uid="{00000000-0004-0000-0000-00007F020000}"/>
-    <hyperlink ref="B643" r:id="rId641" xr:uid="{00000000-0004-0000-0000-000080020000}"/>
-    <hyperlink ref="B644" r:id="rId642" xr:uid="{00000000-0004-0000-0000-000081020000}"/>
-    <hyperlink ref="B645" r:id="rId643" xr:uid="{00000000-0004-0000-0000-000082020000}"/>
-    <hyperlink ref="B646" r:id="rId644" xr:uid="{00000000-0004-0000-0000-000083020000}"/>
-    <hyperlink ref="B647" r:id="rId645" xr:uid="{00000000-0004-0000-0000-000084020000}"/>
-    <hyperlink ref="B648" r:id="rId646" xr:uid="{00000000-0004-0000-0000-000085020000}"/>
-    <hyperlink ref="B649" r:id="rId647" xr:uid="{00000000-0004-0000-0000-000086020000}"/>
-    <hyperlink ref="B650" r:id="rId648" xr:uid="{00000000-0004-0000-0000-000087020000}"/>
-    <hyperlink ref="B651" r:id="rId649" xr:uid="{00000000-0004-0000-0000-000088020000}"/>
-    <hyperlink ref="B652" r:id="rId650" xr:uid="{00000000-0004-0000-0000-000089020000}"/>
-    <hyperlink ref="B653" r:id="rId651" xr:uid="{00000000-0004-0000-0000-00008A020000}"/>
-    <hyperlink ref="B654" r:id="rId652" xr:uid="{00000000-0004-0000-0000-00008B020000}"/>
-    <hyperlink ref="B655" r:id="rId653" xr:uid="{00000000-0004-0000-0000-00008C020000}"/>
-    <hyperlink ref="B656" r:id="rId654" xr:uid="{00000000-0004-0000-0000-00008D020000}"/>
-    <hyperlink ref="B657" r:id="rId655" xr:uid="{00000000-0004-0000-0000-00008E020000}"/>
-    <hyperlink ref="B658" r:id="rId656" xr:uid="{00000000-0004-0000-0000-00008F020000}"/>
-    <hyperlink ref="B659" r:id="rId657" xr:uid="{00000000-0004-0000-0000-000090020000}"/>
-    <hyperlink ref="B660" r:id="rId658" xr:uid="{00000000-0004-0000-0000-000091020000}"/>
-    <hyperlink ref="B661" r:id="rId659" xr:uid="{00000000-0004-0000-0000-000092020000}"/>
-    <hyperlink ref="B662" r:id="rId660" xr:uid="{00000000-0004-0000-0000-000093020000}"/>
-    <hyperlink ref="B663" r:id="rId661" xr:uid="{00000000-0004-0000-0000-000094020000}"/>
-    <hyperlink ref="B664" r:id="rId662" xr:uid="{00000000-0004-0000-0000-000095020000}"/>
-    <hyperlink ref="B665" r:id="rId663" xr:uid="{00000000-0004-0000-0000-000096020000}"/>
-    <hyperlink ref="B666" r:id="rId664" xr:uid="{00000000-0004-0000-0000-000097020000}"/>
-    <hyperlink ref="B667" r:id="rId665" xr:uid="{00000000-0004-0000-0000-000098020000}"/>
-    <hyperlink ref="B668" r:id="rId666" xr:uid="{00000000-0004-0000-0000-000099020000}"/>
-    <hyperlink ref="B669" r:id="rId667" xr:uid="{00000000-0004-0000-0000-00009A020000}"/>
-    <hyperlink ref="B670" r:id="rId668" xr:uid="{00000000-0004-0000-0000-00009B020000}"/>
-    <hyperlink ref="B671" r:id="rId669" xr:uid="{00000000-0004-0000-0000-00009C020000}"/>
-    <hyperlink ref="B672" r:id="rId670" xr:uid="{00000000-0004-0000-0000-00009D020000}"/>
-    <hyperlink ref="B673" r:id="rId671" xr:uid="{00000000-0004-0000-0000-00009E020000}"/>
-    <hyperlink ref="B674" r:id="rId672" xr:uid="{00000000-0004-0000-0000-00009F020000}"/>
-    <hyperlink ref="B675" r:id="rId673" xr:uid="{00000000-0004-0000-0000-0000A0020000}"/>
-    <hyperlink ref="B676" r:id="rId674" xr:uid="{00000000-0004-0000-0000-0000A1020000}"/>
-    <hyperlink ref="B677" r:id="rId675" xr:uid="{00000000-0004-0000-0000-0000A2020000}"/>
-    <hyperlink ref="B678" r:id="rId676" xr:uid="{00000000-0004-0000-0000-0000A3020000}"/>
-    <hyperlink ref="B679" r:id="rId677" xr:uid="{00000000-0004-0000-0000-0000A4020000}"/>
-    <hyperlink ref="B680" r:id="rId678" xr:uid="{00000000-0004-0000-0000-0000A5020000}"/>
-    <hyperlink ref="B681" r:id="rId679" xr:uid="{00000000-0004-0000-0000-0000A6020000}"/>
-    <hyperlink ref="B682" r:id="rId680" xr:uid="{00000000-0004-0000-0000-0000A7020000}"/>
-    <hyperlink ref="B683" r:id="rId681" xr:uid="{00000000-0004-0000-0000-0000A8020000}"/>
-    <hyperlink ref="B684" r:id="rId682" xr:uid="{00000000-0004-0000-0000-0000A9020000}"/>
-    <hyperlink ref="B685" r:id="rId683" xr:uid="{00000000-0004-0000-0000-0000AA020000}"/>
-    <hyperlink ref="B686" r:id="rId684" xr:uid="{00000000-0004-0000-0000-0000AB020000}"/>
-    <hyperlink ref="B687" r:id="rId685" xr:uid="{00000000-0004-0000-0000-0000AC020000}"/>
-    <hyperlink ref="B688" r:id="rId686" xr:uid="{00000000-0004-0000-0000-0000AD020000}"/>
-    <hyperlink ref="B689" r:id="rId687" xr:uid="{00000000-0004-0000-0000-0000AE020000}"/>
-    <hyperlink ref="B690" r:id="rId688" xr:uid="{00000000-0004-0000-0000-0000AF020000}"/>
-    <hyperlink ref="B691" r:id="rId689" xr:uid="{00000000-0004-0000-0000-0000B0020000}"/>
-    <hyperlink ref="B692" r:id="rId690" xr:uid="{00000000-0004-0000-0000-0000B1020000}"/>
-    <hyperlink ref="B693" r:id="rId691" xr:uid="{00000000-0004-0000-0000-0000B2020000}"/>
-    <hyperlink ref="B694" r:id="rId692" xr:uid="{00000000-0004-0000-0000-0000B3020000}"/>
-    <hyperlink ref="B695" r:id="rId693" xr:uid="{00000000-0004-0000-0000-0000B4020000}"/>
-    <hyperlink ref="B696" r:id="rId694" xr:uid="{00000000-0004-0000-0000-0000B5020000}"/>
-    <hyperlink ref="B697" r:id="rId695" xr:uid="{00000000-0004-0000-0000-0000B6020000}"/>
-    <hyperlink ref="B698" r:id="rId696" xr:uid="{00000000-0004-0000-0000-0000B7020000}"/>
-    <hyperlink ref="B699" r:id="rId697" xr:uid="{00000000-0004-0000-0000-0000B8020000}"/>
-    <hyperlink ref="B700" r:id="rId698" xr:uid="{00000000-0004-0000-0000-0000B9020000}"/>
-    <hyperlink ref="B701" r:id="rId699" xr:uid="{00000000-0004-0000-0000-0000BA020000}"/>
-    <hyperlink ref="B702" r:id="rId700" xr:uid="{00000000-0004-0000-0000-0000BB020000}"/>
-    <hyperlink ref="B703" r:id="rId701" xr:uid="{00000000-0004-0000-0000-0000BC020000}"/>
-    <hyperlink ref="B704" r:id="rId702" xr:uid="{00000000-0004-0000-0000-0000BD020000}"/>
-    <hyperlink ref="B705" r:id="rId703" xr:uid="{00000000-0004-0000-0000-0000BE020000}"/>
-    <hyperlink ref="B706" r:id="rId704" xr:uid="{00000000-0004-0000-0000-0000BF020000}"/>
-    <hyperlink ref="B707" r:id="rId705" xr:uid="{00000000-0004-0000-0000-0000C0020000}"/>
-    <hyperlink ref="B708" r:id="rId706" xr:uid="{00000000-0004-0000-0000-0000C1020000}"/>
-    <hyperlink ref="B709" r:id="rId707" xr:uid="{00000000-0004-0000-0000-0000C2020000}"/>
-    <hyperlink ref="B710" r:id="rId708" xr:uid="{00000000-0004-0000-0000-0000C3020000}"/>
-    <hyperlink ref="B711" r:id="rId709" xr:uid="{00000000-0004-0000-0000-0000C4020000}"/>
-    <hyperlink ref="B712" r:id="rId710" xr:uid="{00000000-0004-0000-0000-0000C5020000}"/>
-    <hyperlink ref="B713" r:id="rId711" xr:uid="{00000000-0004-0000-0000-0000C6020000}"/>
-    <hyperlink ref="B714" r:id="rId712" xr:uid="{00000000-0004-0000-0000-0000C7020000}"/>
-    <hyperlink ref="B715" r:id="rId713" xr:uid="{00000000-0004-0000-0000-0000C8020000}"/>
-    <hyperlink ref="B716" r:id="rId714" xr:uid="{00000000-0004-0000-0000-0000C9020000}"/>
-    <hyperlink ref="B717" r:id="rId715" xr:uid="{00000000-0004-0000-0000-0000CA020000}"/>
-    <hyperlink ref="B718" r:id="rId716" xr:uid="{00000000-0004-0000-0000-0000CB020000}"/>
-    <hyperlink ref="B719" r:id="rId717" xr:uid="{00000000-0004-0000-0000-0000CC020000}"/>
-    <hyperlink ref="B720" r:id="rId718" xr:uid="{00000000-0004-0000-0000-0000CD020000}"/>
-    <hyperlink ref="B721" r:id="rId719" xr:uid="{00000000-0004-0000-0000-0000CE020000}"/>
-    <hyperlink ref="B722" r:id="rId720" xr:uid="{00000000-0004-0000-0000-0000CF020000}"/>
-    <hyperlink ref="B723" r:id="rId721" xr:uid="{00000000-0004-0000-0000-0000D0020000}"/>
-    <hyperlink ref="B724" r:id="rId722" xr:uid="{00000000-0004-0000-0000-0000D1020000}"/>
-    <hyperlink ref="B725" r:id="rId723" xr:uid="{00000000-0004-0000-0000-0000D2020000}"/>
-    <hyperlink ref="B726" r:id="rId724" xr:uid="{00000000-0004-0000-0000-0000D3020000}"/>
-    <hyperlink ref="B727" r:id="rId725" xr:uid="{00000000-0004-0000-0000-0000D4020000}"/>
-    <hyperlink ref="B728" r:id="rId726" xr:uid="{00000000-0004-0000-0000-0000D5020000}"/>
-    <hyperlink ref="B729" r:id="rId727" xr:uid="{00000000-0004-0000-0000-0000D6020000}"/>
-    <hyperlink ref="B730" r:id="rId728" xr:uid="{00000000-0004-0000-0000-0000D7020000}"/>
-    <hyperlink ref="B731" r:id="rId729" xr:uid="{00000000-0004-0000-0000-0000D8020000}"/>
-    <hyperlink ref="B732" r:id="rId730" xr:uid="{00000000-0004-0000-0000-0000D9020000}"/>
-    <hyperlink ref="B733" r:id="rId731" xr:uid="{00000000-0004-0000-0000-0000DA020000}"/>
-    <hyperlink ref="B734" r:id="rId732" xr:uid="{00000000-0004-0000-0000-0000DB020000}"/>
-    <hyperlink ref="B735" r:id="rId733" xr:uid="{00000000-0004-0000-0000-0000DC020000}"/>
-    <hyperlink ref="B736" r:id="rId734" xr:uid="{00000000-0004-0000-0000-0000DD020000}"/>
-    <hyperlink ref="B737" r:id="rId735" xr:uid="{00000000-0004-0000-0000-0000DE020000}"/>
-    <hyperlink ref="B738" r:id="rId736" xr:uid="{00000000-0004-0000-0000-0000DF020000}"/>
-    <hyperlink ref="B739" r:id="rId737" xr:uid="{00000000-0004-0000-0000-0000E0020000}"/>
-    <hyperlink ref="B740" r:id="rId738" xr:uid="{00000000-0004-0000-0000-0000E1020000}"/>
-    <hyperlink ref="B741" r:id="rId739" xr:uid="{00000000-0004-0000-0000-0000E2020000}"/>
-    <hyperlink ref="B742" r:id="rId740" xr:uid="{00000000-0004-0000-0000-0000E3020000}"/>
-    <hyperlink ref="B743" r:id="rId741" xr:uid="{00000000-0004-0000-0000-0000E4020000}"/>
-    <hyperlink ref="B744" r:id="rId742" xr:uid="{00000000-0004-0000-0000-0000E5020000}"/>
-    <hyperlink ref="B745" r:id="rId743" xr:uid="{00000000-0004-0000-0000-0000E6020000}"/>
-    <hyperlink ref="B746" r:id="rId744" xr:uid="{00000000-0004-0000-0000-0000E7020000}"/>
-    <hyperlink ref="B747" r:id="rId745" xr:uid="{00000000-0004-0000-0000-0000E8020000}"/>
-    <hyperlink ref="B748" r:id="rId746" xr:uid="{00000000-0004-0000-0000-0000E9020000}"/>
-    <hyperlink ref="B749" r:id="rId747" xr:uid="{00000000-0004-0000-0000-0000EA020000}"/>
-    <hyperlink ref="B750" r:id="rId748" xr:uid="{00000000-0004-0000-0000-0000EB020000}"/>
-    <hyperlink ref="B751" r:id="rId749" xr:uid="{00000000-0004-0000-0000-0000EC020000}"/>
-    <hyperlink ref="B752" r:id="rId750" xr:uid="{00000000-0004-0000-0000-0000ED020000}"/>
-    <hyperlink ref="B753" r:id="rId751" xr:uid="{00000000-0004-0000-0000-0000EE020000}"/>
-    <hyperlink ref="B754" r:id="rId752" xr:uid="{00000000-0004-0000-0000-0000EF020000}"/>
-    <hyperlink ref="B755" r:id="rId753" xr:uid="{00000000-0004-0000-0000-0000F0020000}"/>
-    <hyperlink ref="B756" r:id="rId754" xr:uid="{00000000-0004-0000-0000-0000F1020000}"/>
-    <hyperlink ref="B757" r:id="rId755" xr:uid="{00000000-0004-0000-0000-0000F2020000}"/>
-    <hyperlink ref="B758" r:id="rId756" xr:uid="{00000000-0004-0000-0000-0000F3020000}"/>
-    <hyperlink ref="B759" r:id="rId757" xr:uid="{00000000-0004-0000-0000-0000F4020000}"/>
-    <hyperlink ref="B760" r:id="rId758" xr:uid="{00000000-0004-0000-0000-0000F5020000}"/>
-    <hyperlink ref="B761" r:id="rId759" xr:uid="{00000000-0004-0000-0000-0000F6020000}"/>
-    <hyperlink ref="B762" r:id="rId760" xr:uid="{00000000-0004-0000-0000-0000F7020000}"/>
-    <hyperlink ref="B763" r:id="rId761" xr:uid="{00000000-0004-0000-0000-0000F8020000}"/>
-    <hyperlink ref="B764" r:id="rId762" xr:uid="{00000000-0004-0000-0000-0000F9020000}"/>
-    <hyperlink ref="B765" r:id="rId763" xr:uid="{00000000-0004-0000-0000-0000FA020000}"/>
-    <hyperlink ref="B766" r:id="rId764" xr:uid="{00000000-0004-0000-0000-0000FB020000}"/>
-    <hyperlink ref="B767" r:id="rId765" xr:uid="{00000000-0004-0000-0000-0000FC020000}"/>
-    <hyperlink ref="B768" r:id="rId766" xr:uid="{00000000-0004-0000-0000-0000FD020000}"/>
-    <hyperlink ref="B769" r:id="rId767" xr:uid="{00000000-0004-0000-0000-0000FE020000}"/>
-    <hyperlink ref="B770" r:id="rId768" xr:uid="{00000000-0004-0000-0000-0000FF020000}"/>
-    <hyperlink ref="B771" r:id="rId769" xr:uid="{00000000-0004-0000-0000-000000030000}"/>
-    <hyperlink ref="B772" r:id="rId770" xr:uid="{00000000-0004-0000-0000-000001030000}"/>
-    <hyperlink ref="B773" r:id="rId771" xr:uid="{00000000-0004-0000-0000-000002030000}"/>
-    <hyperlink ref="B774" r:id="rId772" xr:uid="{00000000-0004-0000-0000-000003030000}"/>
-    <hyperlink ref="B775" r:id="rId773" xr:uid="{00000000-0004-0000-0000-000004030000}"/>
-    <hyperlink ref="B776" r:id="rId774" xr:uid="{00000000-0004-0000-0000-000005030000}"/>
-    <hyperlink ref="B777" r:id="rId775" xr:uid="{00000000-0004-0000-0000-000006030000}"/>
-    <hyperlink ref="B778" r:id="rId776" xr:uid="{00000000-0004-0000-0000-000007030000}"/>
-    <hyperlink ref="B779" r:id="rId777" xr:uid="{00000000-0004-0000-0000-000008030000}"/>
-    <hyperlink ref="B780" r:id="rId778" xr:uid="{00000000-0004-0000-0000-000009030000}"/>
-    <hyperlink ref="B781" r:id="rId779" xr:uid="{00000000-0004-0000-0000-00000A030000}"/>
-    <hyperlink ref="B782" r:id="rId780" xr:uid="{00000000-0004-0000-0000-00000B030000}"/>
-    <hyperlink ref="B783" r:id="rId781" xr:uid="{00000000-0004-0000-0000-00000C030000}"/>
-    <hyperlink ref="B784" r:id="rId782" xr:uid="{00000000-0004-0000-0000-00000D030000}"/>
-    <hyperlink ref="B785" r:id="rId783" xr:uid="{00000000-0004-0000-0000-00000E030000}"/>
-    <hyperlink ref="B786" r:id="rId784" xr:uid="{00000000-0004-0000-0000-00000F030000}"/>
-    <hyperlink ref="B787" r:id="rId785" xr:uid="{00000000-0004-0000-0000-000010030000}"/>
-    <hyperlink ref="B788" r:id="rId786" xr:uid="{00000000-0004-0000-0000-000011030000}"/>
-    <hyperlink ref="B789" r:id="rId787" xr:uid="{00000000-0004-0000-0000-000012030000}"/>
-    <hyperlink ref="B790" r:id="rId788" xr:uid="{00000000-0004-0000-0000-000013030000}"/>
-    <hyperlink ref="B791" r:id="rId789" xr:uid="{00000000-0004-0000-0000-000014030000}"/>
-    <hyperlink ref="B792" r:id="rId790" xr:uid="{00000000-0004-0000-0000-000015030000}"/>
-    <hyperlink ref="B793" r:id="rId791" xr:uid="{00000000-0004-0000-0000-000016030000}"/>
-    <hyperlink ref="B794" r:id="rId792" xr:uid="{00000000-0004-0000-0000-000017030000}"/>
-    <hyperlink ref="B795" r:id="rId793" xr:uid="{00000000-0004-0000-0000-000018030000}"/>
-    <hyperlink ref="B796" r:id="rId794" xr:uid="{00000000-0004-0000-0000-000019030000}"/>
-    <hyperlink ref="B797" r:id="rId795" xr:uid="{00000000-0004-0000-0000-00001A030000}"/>
-    <hyperlink ref="B798" r:id="rId796" xr:uid="{00000000-0004-0000-0000-00001B030000}"/>
-    <hyperlink ref="B799" r:id="rId797" xr:uid="{00000000-0004-0000-0000-00001C030000}"/>
-    <hyperlink ref="B800" r:id="rId798" xr:uid="{00000000-0004-0000-0000-00001D030000}"/>
-    <hyperlink ref="B801" r:id="rId799" xr:uid="{00000000-0004-0000-0000-00001E030000}"/>
-    <hyperlink ref="B802" r:id="rId800" xr:uid="{00000000-0004-0000-0000-00001F030000}"/>
-    <hyperlink ref="B803" r:id="rId801" xr:uid="{00000000-0004-0000-0000-000020030000}"/>
-    <hyperlink ref="B804" r:id="rId802" xr:uid="{00000000-0004-0000-0000-000021030000}"/>
-    <hyperlink ref="B805" r:id="rId803" xr:uid="{00000000-0004-0000-0000-000022030000}"/>
-    <hyperlink ref="B806" r:id="rId804" xr:uid="{00000000-0004-0000-0000-000023030000}"/>
-    <hyperlink ref="B807" r:id="rId805" xr:uid="{00000000-0004-0000-0000-000024030000}"/>
-    <hyperlink ref="B808" r:id="rId806" xr:uid="{00000000-0004-0000-0000-000025030000}"/>
-    <hyperlink ref="B809" r:id="rId807" xr:uid="{00000000-0004-0000-0000-000026030000}"/>
-    <hyperlink ref="B810" r:id="rId808" xr:uid="{00000000-0004-0000-0000-000027030000}"/>
-    <hyperlink ref="B811" r:id="rId809" xr:uid="{00000000-0004-0000-0000-000028030000}"/>
-    <hyperlink ref="B812" r:id="rId810" xr:uid="{00000000-0004-0000-0000-000029030000}"/>
-    <hyperlink ref="B813" r:id="rId811" xr:uid="{00000000-0004-0000-0000-00002A030000}"/>
-    <hyperlink ref="B814" r:id="rId812" xr:uid="{00000000-0004-0000-0000-00002B030000}"/>
-    <hyperlink ref="B815" r:id="rId813" xr:uid="{00000000-0004-0000-0000-00002C030000}"/>
-    <hyperlink ref="B816" r:id="rId814" xr:uid="{00000000-0004-0000-0000-00002D030000}"/>
-    <hyperlink ref="B817" r:id="rId815" xr:uid="{00000000-0004-0000-0000-00002E030000}"/>
-    <hyperlink ref="B818" r:id="rId816" xr:uid="{00000000-0004-0000-0000-00002F030000}"/>
-    <hyperlink ref="B819" r:id="rId817" xr:uid="{00000000-0004-0000-0000-000030030000}"/>
-    <hyperlink ref="B820" r:id="rId818" xr:uid="{00000000-0004-0000-0000-000031030000}"/>
-    <hyperlink ref="B821" r:id="rId819" xr:uid="{00000000-0004-0000-0000-000032030000}"/>
-    <hyperlink ref="B822" r:id="rId820" xr:uid="{00000000-0004-0000-0000-000033030000}"/>
-    <hyperlink ref="B823" r:id="rId821" xr:uid="{00000000-0004-0000-0000-000034030000}"/>
-    <hyperlink ref="B824" r:id="rId822" xr:uid="{00000000-0004-0000-0000-000035030000}"/>
-    <hyperlink ref="B825" r:id="rId823" xr:uid="{00000000-0004-0000-0000-000036030000}"/>
-    <hyperlink ref="B826" r:id="rId824" xr:uid="{00000000-0004-0000-0000-000037030000}"/>
-    <hyperlink ref="B827" r:id="rId825" xr:uid="{00000000-0004-0000-0000-000038030000}"/>
-    <hyperlink ref="B828" r:id="rId826" xr:uid="{00000000-0004-0000-0000-000039030000}"/>
-    <hyperlink ref="B829" r:id="rId827" xr:uid="{00000000-0004-0000-0000-00003A030000}"/>
-    <hyperlink ref="B830" r:id="rId828" xr:uid="{00000000-0004-0000-0000-00003B030000}"/>
-    <hyperlink ref="B831" r:id="rId829" xr:uid="{00000000-0004-0000-0000-00003C030000}"/>
-    <hyperlink ref="B832" r:id="rId830" xr:uid="{00000000-0004-0000-0000-00003D030000}"/>
-    <hyperlink ref="B833" r:id="rId831" xr:uid="{00000000-0004-0000-0000-00003E030000}"/>
-    <hyperlink ref="B834" r:id="rId832" xr:uid="{00000000-0004-0000-0000-00003F030000}"/>
-    <hyperlink ref="B835" r:id="rId833" xr:uid="{00000000-0004-0000-0000-000040030000}"/>
-    <hyperlink ref="B836" r:id="rId834" xr:uid="{00000000-0004-0000-0000-000041030000}"/>
-    <hyperlink ref="B837" r:id="rId835" xr:uid="{00000000-0004-0000-0000-000042030000}"/>
-    <hyperlink ref="B838" r:id="rId836" xr:uid="{00000000-0004-0000-0000-000043030000}"/>
-    <hyperlink ref="B839" r:id="rId837" xr:uid="{00000000-0004-0000-0000-000044030000}"/>
-    <hyperlink ref="B840" r:id="rId838" xr:uid="{00000000-0004-0000-0000-000045030000}"/>
-    <hyperlink ref="B841" r:id="rId839" xr:uid="{00000000-0004-0000-0000-000046030000}"/>
-    <hyperlink ref="B842" r:id="rId840" xr:uid="{00000000-0004-0000-0000-000047030000}"/>
-    <hyperlink ref="B843" r:id="rId841" xr:uid="{00000000-0004-0000-0000-000048030000}"/>
-    <hyperlink ref="B844" r:id="rId842" xr:uid="{00000000-0004-0000-0000-000049030000}"/>
-    <hyperlink ref="B845" r:id="rId843" xr:uid="{00000000-0004-0000-0000-00004A030000}"/>
-    <hyperlink ref="B846" r:id="rId844" xr:uid="{00000000-0004-0000-0000-00004B030000}"/>
-    <hyperlink ref="B847" r:id="rId845" xr:uid="{00000000-0004-0000-0000-00004C030000}"/>
-    <hyperlink ref="B848" r:id="rId846" xr:uid="{00000000-0004-0000-0000-00004D030000}"/>
-    <hyperlink ref="B849" r:id="rId847" xr:uid="{00000000-0004-0000-0000-00004E030000}"/>
-    <hyperlink ref="B850" r:id="rId848" xr:uid="{00000000-0004-0000-0000-00004F030000}"/>
-    <hyperlink ref="B851" r:id="rId849" xr:uid="{00000000-0004-0000-0000-000050030000}"/>
-    <hyperlink ref="B852" r:id="rId850" xr:uid="{00000000-0004-0000-0000-000051030000}"/>
-    <hyperlink ref="B853" r:id="rId851" xr:uid="{00000000-0004-0000-0000-000052030000}"/>
-    <hyperlink ref="B854" r:id="rId852" xr:uid="{00000000-0004-0000-0000-000053030000}"/>
-    <hyperlink ref="B855" r:id="rId853" xr:uid="{00000000-0004-0000-0000-000054030000}"/>
-    <hyperlink ref="B856" r:id="rId854" xr:uid="{00000000-0004-0000-0000-000055030000}"/>
-    <hyperlink ref="B857" r:id="rId855" xr:uid="{00000000-0004-0000-0000-000056030000}"/>
-    <hyperlink ref="B858" r:id="rId856" xr:uid="{00000000-0004-0000-0000-000057030000}"/>
-    <hyperlink ref="B859" r:id="rId857" xr:uid="{00000000-0004-0000-0000-000058030000}"/>
-    <hyperlink ref="B860" r:id="rId858" xr:uid="{00000000-0004-0000-0000-000059030000}"/>
-    <hyperlink ref="B861" r:id="rId859" xr:uid="{00000000-0004-0000-0000-00005A030000}"/>
-    <hyperlink ref="B862" r:id="rId860" xr:uid="{00000000-0004-0000-0000-00005B030000}"/>
-    <hyperlink ref="B863" r:id="rId861" xr:uid="{00000000-0004-0000-0000-00005C030000}"/>
-    <hyperlink ref="B864" r:id="rId862" xr:uid="{00000000-0004-0000-0000-00005D030000}"/>
-    <hyperlink ref="B865" r:id="rId863" xr:uid="{00000000-0004-0000-0000-00005E030000}"/>
-    <hyperlink ref="B866" r:id="rId864" xr:uid="{00000000-0004-0000-0000-00005F030000}"/>
-    <hyperlink ref="B867" r:id="rId865" xr:uid="{00000000-0004-0000-0000-000060030000}"/>
-    <hyperlink ref="B868" r:id="rId866" xr:uid="{00000000-0004-0000-0000-000061030000}"/>
-    <hyperlink ref="B869" r:id="rId867" xr:uid="{00000000-0004-0000-0000-000062030000}"/>
-    <hyperlink ref="B870" r:id="rId868" xr:uid="{00000000-0004-0000-0000-000063030000}"/>
-    <hyperlink ref="B871" r:id="rId869" xr:uid="{00000000-0004-0000-0000-000064030000}"/>
-    <hyperlink ref="B872" r:id="rId870" xr:uid="{00000000-0004-0000-0000-000065030000}"/>
-    <hyperlink ref="B873" r:id="rId871" xr:uid="{00000000-0004-0000-0000-000066030000}"/>
-    <hyperlink ref="B874" r:id="rId872" xr:uid="{00000000-0004-0000-0000-000067030000}"/>
-    <hyperlink ref="B875" r:id="rId873" xr:uid="{00000000-0004-0000-0000-000068030000}"/>
-    <hyperlink ref="B876" r:id="rId874" xr:uid="{00000000-0004-0000-0000-000069030000}"/>
-    <hyperlink ref="B877" r:id="rId875" xr:uid="{00000000-0004-0000-0000-00006A030000}"/>
-    <hyperlink ref="B878" r:id="rId876" xr:uid="{00000000-0004-0000-0000-00006B030000}"/>
-    <hyperlink ref="B879" r:id="rId877" xr:uid="{00000000-0004-0000-0000-00006C030000}"/>
-    <hyperlink ref="B880" r:id="rId878" xr:uid="{00000000-0004-0000-0000-00006D030000}"/>
-    <hyperlink ref="B881" r:id="rId879" xr:uid="{00000000-0004-0000-0000-00006E030000}"/>
-    <hyperlink ref="B882" r:id="rId880" xr:uid="{00000000-0004-0000-0000-00006F030000}"/>
-    <hyperlink ref="B883" r:id="rId881" xr:uid="{00000000-0004-0000-0000-000070030000}"/>
-    <hyperlink ref="B884" r:id="rId882" xr:uid="{00000000-0004-0000-0000-000071030000}"/>
-    <hyperlink ref="B885" r:id="rId883" xr:uid="{00000000-0004-0000-0000-000072030000}"/>
-    <hyperlink ref="B886" r:id="rId884" xr:uid="{00000000-0004-0000-0000-000073030000}"/>
-    <hyperlink ref="B887" r:id="rId885" xr:uid="{00000000-0004-0000-0000-000074030000}"/>
-    <hyperlink ref="B888" r:id="rId886" xr:uid="{00000000-0004-0000-0000-000075030000}"/>
-    <hyperlink ref="B889" r:id="rId887" xr:uid="{00000000-0004-0000-0000-000076030000}"/>
-    <hyperlink ref="B890" r:id="rId888" xr:uid="{00000000-0004-0000-0000-000077030000}"/>
-    <hyperlink ref="B891" r:id="rId889" xr:uid="{00000000-0004-0000-0000-000078030000}"/>
-    <hyperlink ref="B892" r:id="rId890" xr:uid="{00000000-0004-0000-0000-000079030000}"/>
-    <hyperlink ref="B893" r:id="rId891" xr:uid="{00000000-0004-0000-0000-00007A030000}"/>
-    <hyperlink ref="B894" r:id="rId892" xr:uid="{00000000-0004-0000-0000-00007B030000}"/>
-    <hyperlink ref="B895" r:id="rId893" xr:uid="{00000000-0004-0000-0000-00007C030000}"/>
-    <hyperlink ref="B896" r:id="rId894" xr:uid="{00000000-0004-0000-0000-00007D030000}"/>
-    <hyperlink ref="B897" r:id="rId895" xr:uid="{00000000-0004-0000-0000-00007E030000}"/>
-    <hyperlink ref="B898" r:id="rId896" xr:uid="{00000000-0004-0000-0000-00007F030000}"/>
-    <hyperlink ref="B899" r:id="rId897" xr:uid="{00000000-0004-0000-0000-000080030000}"/>
-    <hyperlink ref="B900" r:id="rId898" xr:uid="{00000000-0004-0000-0000-000081030000}"/>
-    <hyperlink ref="B901" r:id="rId899" xr:uid="{00000000-0004-0000-0000-000082030000}"/>
-    <hyperlink ref="B902" r:id="rId900" xr:uid="{00000000-0004-0000-0000-000083030000}"/>
-    <hyperlink ref="B903" r:id="rId901" xr:uid="{00000000-0004-0000-0000-000084030000}"/>
-    <hyperlink ref="B904" r:id="rId902" xr:uid="{00000000-0004-0000-0000-000085030000}"/>
-    <hyperlink ref="B905" r:id="rId903" xr:uid="{00000000-0004-0000-0000-000086030000}"/>
-    <hyperlink ref="B906" r:id="rId904" xr:uid="{00000000-0004-0000-0000-000087030000}"/>
-    <hyperlink ref="B907" r:id="rId905" xr:uid="{00000000-0004-0000-0000-000088030000}"/>
-    <hyperlink ref="B908" r:id="rId906" xr:uid="{00000000-0004-0000-0000-000089030000}"/>
-    <hyperlink ref="B909" r:id="rId907" xr:uid="{00000000-0004-0000-0000-00008A030000}"/>
-    <hyperlink ref="B910" r:id="rId908" xr:uid="{00000000-0004-0000-0000-00008B030000}"/>
-    <hyperlink ref="B911" r:id="rId909" xr:uid="{00000000-0004-0000-0000-00008C030000}"/>
-    <hyperlink ref="B912" r:id="rId910" xr:uid="{00000000-0004-0000-0000-00008D030000}"/>
-    <hyperlink ref="B913" r:id="rId911" xr:uid="{00000000-0004-0000-0000-00008E030000}"/>
-    <hyperlink ref="B914" r:id="rId912" xr:uid="{00000000-0004-0000-0000-00008F030000}"/>
-    <hyperlink ref="B915" r:id="rId913" xr:uid="{00000000-0004-0000-0000-000090030000}"/>
-    <hyperlink ref="B916" r:id="rId914" xr:uid="{00000000-0004-0000-0000-000091030000}"/>
-    <hyperlink ref="B917" r:id="rId915" xr:uid="{00000000-0004-0000-0000-000092030000}"/>
-    <hyperlink ref="B918" r:id="rId916" xr:uid="{00000000-0004-0000-0000-000093030000}"/>
-    <hyperlink ref="B919" r:id="rId917" xr:uid="{00000000-0004-0000-0000-000094030000}"/>
-    <hyperlink ref="B920" r:id="rId918" xr:uid="{00000000-0004-0000-0000-000095030000}"/>
-    <hyperlink ref="B921" r:id="rId919" xr:uid="{00000000-0004-0000-0000-000096030000}"/>
-    <hyperlink ref="B922" r:id="rId920" xr:uid="{00000000-0004-0000-0000-000097030000}"/>
-    <hyperlink ref="B923" r:id="rId921" xr:uid="{00000000-0004-0000-0000-000098030000}"/>
-    <hyperlink ref="B924" r:id="rId922" xr:uid="{00000000-0004-0000-0000-000099030000}"/>
-    <hyperlink ref="B925" r:id="rId923" xr:uid="{00000000-0004-0000-0000-00009A030000}"/>
-    <hyperlink ref="B926" r:id="rId924" xr:uid="{00000000-0004-0000-0000-00009B030000}"/>
-    <hyperlink ref="B927" r:id="rId925" xr:uid="{00000000-0004-0000-0000-00009C030000}"/>
-    <hyperlink ref="B928" r:id="rId926" xr:uid="{00000000-0004-0000-0000-00009D030000}"/>
-    <hyperlink ref="B929" r:id="rId927" xr:uid="{00000000-0004-0000-0000-00009E030000}"/>
-    <hyperlink ref="B930" r:id="rId928" xr:uid="{00000000-0004-0000-0000-00009F030000}"/>
-    <hyperlink ref="B931" r:id="rId929" xr:uid="{00000000-0004-0000-0000-0000A0030000}"/>
-    <hyperlink ref="B932" r:id="rId930" xr:uid="{00000000-0004-0000-0000-0000A1030000}"/>
-    <hyperlink ref="B933" r:id="rId931" xr:uid="{00000000-0004-0000-0000-0000A2030000}"/>
-    <hyperlink ref="B934" r:id="rId932" xr:uid="{00000000-0004-0000-0000-0000A3030000}"/>
-    <hyperlink ref="B935" r:id="rId933" xr:uid="{00000000-0004-0000-0000-0000A4030000}"/>
-    <hyperlink ref="B936" r:id="rId934" xr:uid="{00000000-0004-0000-0000-0000A5030000}"/>
-    <hyperlink ref="B937" r:id="rId935" xr:uid="{00000000-0004-0000-0000-0000A6030000}"/>
-    <hyperlink ref="B938" r:id="rId936" xr:uid="{00000000-0004-0000-0000-0000A7030000}"/>
-    <hyperlink ref="B939" r:id="rId937" xr:uid="{00000000-0004-0000-0000-0000A8030000}"/>
-    <hyperlink ref="B940" r:id="rId938" xr:uid="{00000000-0004-0000-0000-0000A9030000}"/>
-    <hyperlink ref="B941" r:id="rId939" xr:uid="{00000000-0004-0000-0000-0000AA030000}"/>
-    <hyperlink ref="B942" r:id="rId940" xr:uid="{00000000-0004-0000-0000-0000AB030000}"/>
-    <hyperlink ref="B943" r:id="rId941" xr:uid="{00000000-0004-0000-0000-0000AC030000}"/>
-    <hyperlink ref="B944" r:id="rId942" xr:uid="{00000000-0004-0000-0000-0000AD030000}"/>
-    <hyperlink ref="B945" r:id="rId943" xr:uid="{00000000-0004-0000-0000-0000AE030000}"/>
-    <hyperlink ref="B946" r:id="rId944" xr:uid="{00000000-0004-0000-0000-0000AF030000}"/>
-    <hyperlink ref="B947" r:id="rId945" xr:uid="{00000000-0004-0000-0000-0000B0030000}"/>
-    <hyperlink ref="B948" r:id="rId946" xr:uid="{00000000-0004-0000-0000-0000B1030000}"/>
-    <hyperlink ref="B949" r:id="rId947" xr:uid="{00000000-0004-0000-0000-0000B2030000}"/>
-    <hyperlink ref="B950" r:id="rId948" xr:uid="{00000000-0004-0000-0000-0000B3030000}"/>
-    <hyperlink ref="B951" r:id="rId949" xr:uid="{00000000-0004-0000-0000-0000B4030000}"/>
-    <hyperlink ref="B952" r:id="rId950" xr:uid="{00000000-0004-0000-0000-0000B5030000}"/>
-    <hyperlink ref="B953" r:id="rId951" xr:uid="{00000000-0004-0000-0000-0000B6030000}"/>
-    <hyperlink ref="B954" r:id="rId952" xr:uid="{00000000-0004-0000-0000-0000B7030000}"/>
-    <hyperlink ref="B955" r:id="rId953" xr:uid="{00000000-0004-0000-0000-0000B8030000}"/>
-    <hyperlink ref="B956" r:id="rId954" xr:uid="{00000000-0004-0000-0000-0000B9030000}"/>
-    <hyperlink ref="B957" r:id="rId955" xr:uid="{00000000-0004-0000-0000-0000BA030000}"/>
-    <hyperlink ref="B958" r:id="rId956" xr:uid="{00000000-0004-0000-0000-0000BB030000}"/>
-    <hyperlink ref="B959" r:id="rId957" xr:uid="{00000000-0004-0000-0000-0000BC030000}"/>
-    <hyperlink ref="B960" r:id="rId958" xr:uid="{00000000-0004-0000-0000-0000BD030000}"/>
-    <hyperlink ref="B961" r:id="rId959" xr:uid="{00000000-0004-0000-0000-0000BE030000}"/>
-    <hyperlink ref="B962" r:id="rId960" xr:uid="{00000000-0004-0000-0000-0000BF030000}"/>
-    <hyperlink ref="B963" r:id="rId961" xr:uid="{00000000-0004-0000-0000-0000C0030000}"/>
-    <hyperlink ref="B964" r:id="rId962" xr:uid="{00000000-0004-0000-0000-0000C1030000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Entenmann's en:doughnuts category
</commit_message>
<xml_diff>
--- a/comprehensive_grocery_certifications_COMPLETE.xlsx
+++ b/comprehensive_grocery_certifications_COMPLETE.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1185" uniqueCount="1185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1187" uniqueCount="1187">
   <si>
     <t>Product_Brand</t>
   </si>
@@ -3575,6 +3575,12 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>en:doughnuts</t>
+  </si>
+  <si>
+    <t>Donuts, Pastries</t>
   </si>
 </sst>
 </file>
@@ -3931,7 +3937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K965"/>
+  <dimension ref="A1:K966"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="33.1481857299805" customWidth="1"/>
@@ -31998,971 +32004,1004 @@
         <v>18</v>
       </c>
     </row>
+    <row r="966">
+      <c r="A966" s="0" t="s">
+        <v>290</v>
+      </c>
+      <c r="B966" s="1" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C966" s="0" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D966" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="E966" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="F966" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="G966" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="H966" s="0" t="s">
+        <v>1186</v>
+      </c>
+      <c r="I966" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="K966" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1"/>
-    <hyperlink ref="B4" r:id="rId2"/>
-    <hyperlink ref="B5" r:id="rId3"/>
-    <hyperlink ref="B6" r:id="rId4"/>
-    <hyperlink ref="B7" r:id="rId5"/>
-    <hyperlink ref="B8" r:id="rId6"/>
-    <hyperlink ref="B9" r:id="rId7"/>
-    <hyperlink ref="B10" r:id="rId8"/>
-    <hyperlink ref="B11" r:id="rId9"/>
-    <hyperlink ref="B12" r:id="rId10"/>
-    <hyperlink ref="B13" r:id="rId11"/>
-    <hyperlink ref="B14" r:id="rId12"/>
-    <hyperlink ref="B15" r:id="rId13"/>
-    <hyperlink ref="B16" r:id="rId14"/>
-    <hyperlink ref="B17" r:id="rId15"/>
-    <hyperlink ref="B18" r:id="rId16"/>
-    <hyperlink ref="B19" r:id="rId17"/>
-    <hyperlink ref="B20" r:id="rId18"/>
-    <hyperlink ref="B21" r:id="rId19"/>
-    <hyperlink ref="B22" r:id="rId20"/>
-    <hyperlink ref="B23" r:id="rId21"/>
-    <hyperlink ref="B24" r:id="rId22"/>
-    <hyperlink ref="B25" r:id="rId23"/>
-    <hyperlink ref="B26" r:id="rId24"/>
-    <hyperlink ref="B27" r:id="rId25"/>
-    <hyperlink ref="B28" r:id="rId26"/>
-    <hyperlink ref="B29" r:id="rId27"/>
-    <hyperlink ref="B30" r:id="rId28"/>
-    <hyperlink ref="B31" r:id="rId29"/>
-    <hyperlink ref="B32" r:id="rId30"/>
-    <hyperlink ref="B33" r:id="rId31"/>
-    <hyperlink ref="B34" r:id="rId32"/>
-    <hyperlink ref="B35" r:id="rId33"/>
-    <hyperlink ref="B36" r:id="rId34"/>
-    <hyperlink ref="B37" r:id="rId35"/>
-    <hyperlink ref="B38" r:id="rId36"/>
-    <hyperlink ref="B39" r:id="rId37"/>
-    <hyperlink ref="B40" r:id="rId38"/>
-    <hyperlink ref="B41" r:id="rId39"/>
-    <hyperlink ref="B42" r:id="rId40"/>
-    <hyperlink ref="B43" r:id="rId41"/>
-    <hyperlink ref="B44" r:id="rId42"/>
-    <hyperlink ref="B45" r:id="rId43"/>
-    <hyperlink ref="B46" r:id="rId44"/>
-    <hyperlink ref="B47" r:id="rId45"/>
-    <hyperlink ref="B48" r:id="rId46"/>
-    <hyperlink ref="B49" r:id="rId47"/>
-    <hyperlink ref="B50" r:id="rId48"/>
-    <hyperlink ref="B51" r:id="rId49"/>
-    <hyperlink ref="B52" r:id="rId50"/>
-    <hyperlink ref="B53" r:id="rId51"/>
-    <hyperlink ref="B54" r:id="rId52"/>
-    <hyperlink ref="B55" r:id="rId53"/>
-    <hyperlink ref="B56" r:id="rId54"/>
-    <hyperlink ref="B57" r:id="rId55"/>
-    <hyperlink ref="B58" r:id="rId56"/>
-    <hyperlink ref="B59" r:id="rId57"/>
-    <hyperlink ref="B60" r:id="rId58"/>
-    <hyperlink ref="B61" r:id="rId59"/>
-    <hyperlink ref="B62" r:id="rId60"/>
-    <hyperlink ref="B63" r:id="rId61"/>
-    <hyperlink ref="B64" r:id="rId62"/>
-    <hyperlink ref="B65" r:id="rId63"/>
-    <hyperlink ref="B66" r:id="rId64"/>
-    <hyperlink ref="B67" r:id="rId65"/>
-    <hyperlink ref="B68" r:id="rId66"/>
-    <hyperlink ref="B69" r:id="rId67"/>
-    <hyperlink ref="B70" r:id="rId68"/>
-    <hyperlink ref="B71" r:id="rId69"/>
-    <hyperlink ref="B72" r:id="rId70"/>
-    <hyperlink ref="B73" r:id="rId71"/>
-    <hyperlink ref="B74" r:id="rId72"/>
-    <hyperlink ref="B75" r:id="rId73"/>
-    <hyperlink ref="B76" r:id="rId74"/>
-    <hyperlink ref="B77" r:id="rId75"/>
-    <hyperlink ref="B78" r:id="rId76"/>
-    <hyperlink ref="B79" r:id="rId77"/>
-    <hyperlink ref="B80" r:id="rId78"/>
-    <hyperlink ref="B81" r:id="rId79"/>
-    <hyperlink ref="B82" r:id="rId80"/>
-    <hyperlink ref="B83" r:id="rId81"/>
-    <hyperlink ref="B84" r:id="rId82"/>
-    <hyperlink ref="B85" r:id="rId83"/>
-    <hyperlink ref="B86" r:id="rId84"/>
-    <hyperlink ref="B87" r:id="rId85"/>
-    <hyperlink ref="B88" r:id="rId86"/>
-    <hyperlink ref="B89" r:id="rId87"/>
-    <hyperlink ref="B90" r:id="rId88"/>
-    <hyperlink ref="B91" r:id="rId89"/>
-    <hyperlink ref="B92" r:id="rId90"/>
-    <hyperlink ref="B93" r:id="rId91"/>
-    <hyperlink ref="B94" r:id="rId92"/>
-    <hyperlink ref="B95" r:id="rId93"/>
-    <hyperlink ref="B96" r:id="rId94"/>
-    <hyperlink ref="B97" r:id="rId95"/>
-    <hyperlink ref="B98" r:id="rId96"/>
-    <hyperlink ref="B99" r:id="rId97"/>
-    <hyperlink ref="B100" r:id="rId98"/>
-    <hyperlink ref="B101" r:id="rId99"/>
-    <hyperlink ref="B102" r:id="rId100"/>
-    <hyperlink ref="B103" r:id="rId101"/>
-    <hyperlink ref="B104" r:id="rId102"/>
-    <hyperlink ref="B105" r:id="rId103"/>
-    <hyperlink ref="B106" r:id="rId104"/>
-    <hyperlink ref="B107" r:id="rId105"/>
-    <hyperlink ref="B108" r:id="rId106"/>
-    <hyperlink ref="B109" r:id="rId107"/>
-    <hyperlink ref="B110" r:id="rId108"/>
-    <hyperlink ref="B111" r:id="rId109"/>
-    <hyperlink ref="B112" r:id="rId110"/>
-    <hyperlink ref="B113" r:id="rId111"/>
-    <hyperlink ref="B114" r:id="rId112"/>
-    <hyperlink ref="B115" r:id="rId113"/>
-    <hyperlink ref="B116" r:id="rId114"/>
-    <hyperlink ref="B117" r:id="rId115"/>
-    <hyperlink ref="B118" r:id="rId116"/>
-    <hyperlink ref="B119" r:id="rId117"/>
-    <hyperlink ref="B120" r:id="rId118"/>
-    <hyperlink ref="B121" r:id="rId119"/>
-    <hyperlink ref="B122" r:id="rId120"/>
-    <hyperlink ref="B123" r:id="rId121"/>
-    <hyperlink ref="B124" r:id="rId122"/>
-    <hyperlink ref="B125" r:id="rId123"/>
-    <hyperlink ref="B126" r:id="rId124"/>
-    <hyperlink ref="B127" r:id="rId125"/>
-    <hyperlink ref="B128" r:id="rId126"/>
-    <hyperlink ref="B129" r:id="rId127"/>
-    <hyperlink ref="B130" r:id="rId128"/>
-    <hyperlink ref="B131" r:id="rId129"/>
-    <hyperlink ref="B132" r:id="rId130"/>
-    <hyperlink ref="B133" r:id="rId131"/>
-    <hyperlink ref="B134" r:id="rId132"/>
-    <hyperlink ref="B135" r:id="rId133"/>
-    <hyperlink ref="B136" r:id="rId134"/>
-    <hyperlink ref="B137" r:id="rId135"/>
-    <hyperlink ref="B138" r:id="rId136"/>
-    <hyperlink ref="B139" r:id="rId137"/>
-    <hyperlink ref="B140" r:id="rId138"/>
-    <hyperlink ref="B141" r:id="rId139"/>
-    <hyperlink ref="B142" r:id="rId140"/>
-    <hyperlink ref="B143" r:id="rId141"/>
-    <hyperlink ref="B144" r:id="rId142"/>
-    <hyperlink ref="B145" r:id="rId143"/>
-    <hyperlink ref="B146" r:id="rId144"/>
-    <hyperlink ref="B147" r:id="rId145"/>
-    <hyperlink ref="B148" r:id="rId146"/>
-    <hyperlink ref="B149" r:id="rId147"/>
-    <hyperlink ref="B150" r:id="rId148"/>
-    <hyperlink ref="B151" r:id="rId149"/>
-    <hyperlink ref="B152" r:id="rId150"/>
-    <hyperlink ref="B153" r:id="rId151"/>
-    <hyperlink ref="B154" r:id="rId152"/>
-    <hyperlink ref="B155" r:id="rId153"/>
-    <hyperlink ref="B156" r:id="rId154"/>
-    <hyperlink ref="B157" r:id="rId155"/>
-    <hyperlink ref="B158" r:id="rId156"/>
-    <hyperlink ref="B159" r:id="rId157"/>
-    <hyperlink ref="B160" r:id="rId158"/>
-    <hyperlink ref="B161" r:id="rId159"/>
-    <hyperlink ref="B162" r:id="rId160"/>
-    <hyperlink ref="B163" r:id="rId161"/>
-    <hyperlink ref="B164" r:id="rId162"/>
-    <hyperlink ref="B165" r:id="rId163"/>
-    <hyperlink ref="B166" r:id="rId164"/>
-    <hyperlink ref="B167" r:id="rId165"/>
-    <hyperlink ref="B168" r:id="rId166"/>
-    <hyperlink ref="B169" r:id="rId167"/>
-    <hyperlink ref="B170" r:id="rId168"/>
-    <hyperlink ref="B171" r:id="rId169"/>
-    <hyperlink ref="B172" r:id="rId170"/>
-    <hyperlink ref="B173" r:id="rId171"/>
-    <hyperlink ref="B174" r:id="rId172"/>
-    <hyperlink ref="B175" r:id="rId173"/>
-    <hyperlink ref="B176" r:id="rId174"/>
-    <hyperlink ref="B177" r:id="rId175"/>
-    <hyperlink ref="B178" r:id="rId176"/>
-    <hyperlink ref="B179" r:id="rId177"/>
-    <hyperlink ref="B180" r:id="rId178"/>
-    <hyperlink ref="B181" r:id="rId179"/>
-    <hyperlink ref="B182" r:id="rId180"/>
-    <hyperlink ref="B183" r:id="rId181"/>
-    <hyperlink ref="B184" r:id="rId182"/>
-    <hyperlink ref="B185" r:id="rId183"/>
-    <hyperlink ref="B186" r:id="rId184"/>
-    <hyperlink ref="B187" r:id="rId185"/>
-    <hyperlink ref="B188" r:id="rId186"/>
-    <hyperlink ref="B189" r:id="rId187"/>
-    <hyperlink ref="B190" r:id="rId188"/>
-    <hyperlink ref="B191" r:id="rId189"/>
-    <hyperlink ref="B192" r:id="rId190"/>
-    <hyperlink ref="B193" r:id="rId191"/>
-    <hyperlink ref="B194" r:id="rId192"/>
-    <hyperlink ref="B195" r:id="rId193"/>
-    <hyperlink ref="B196" r:id="rId194"/>
-    <hyperlink ref="B197" r:id="rId195"/>
-    <hyperlink ref="B198" r:id="rId196"/>
-    <hyperlink ref="B199" r:id="rId197"/>
-    <hyperlink ref="B200" r:id="rId198"/>
-    <hyperlink ref="B201" r:id="rId199"/>
-    <hyperlink ref="B202" r:id="rId200"/>
-    <hyperlink ref="B203" r:id="rId201"/>
-    <hyperlink ref="B204" r:id="rId202"/>
-    <hyperlink ref="B205" r:id="rId203"/>
-    <hyperlink ref="B206" r:id="rId204"/>
-    <hyperlink ref="B207" r:id="rId205"/>
-    <hyperlink ref="B208" r:id="rId206"/>
-    <hyperlink ref="B209" r:id="rId207"/>
-    <hyperlink ref="B210" r:id="rId208"/>
-    <hyperlink ref="B211" r:id="rId209"/>
-    <hyperlink ref="B212" r:id="rId210"/>
-    <hyperlink ref="B213" r:id="rId211"/>
-    <hyperlink ref="B214" r:id="rId212"/>
-    <hyperlink ref="B215" r:id="rId213"/>
-    <hyperlink ref="B216" r:id="rId214"/>
-    <hyperlink ref="B217" r:id="rId215"/>
-    <hyperlink ref="B218" r:id="rId216"/>
-    <hyperlink ref="B219" r:id="rId217"/>
-    <hyperlink ref="B220" r:id="rId218"/>
-    <hyperlink ref="B221" r:id="rId219"/>
-    <hyperlink ref="B222" r:id="rId220"/>
-    <hyperlink ref="B223" r:id="rId221"/>
-    <hyperlink ref="B224" r:id="rId222"/>
-    <hyperlink ref="B225" r:id="rId223"/>
-    <hyperlink ref="B226" r:id="rId224"/>
-    <hyperlink ref="B227" r:id="rId225"/>
-    <hyperlink ref="B228" r:id="rId226"/>
-    <hyperlink ref="B229" r:id="rId227"/>
-    <hyperlink ref="B230" r:id="rId228"/>
-    <hyperlink ref="B231" r:id="rId229"/>
-    <hyperlink ref="B232" r:id="rId230"/>
-    <hyperlink ref="B233" r:id="rId231"/>
-    <hyperlink ref="B234" r:id="rId232"/>
-    <hyperlink ref="B235" r:id="rId233"/>
-    <hyperlink ref="B236" r:id="rId234"/>
-    <hyperlink ref="B237" r:id="rId235"/>
-    <hyperlink ref="B238" r:id="rId236"/>
-    <hyperlink ref="B239" r:id="rId237"/>
-    <hyperlink ref="B240" r:id="rId238"/>
-    <hyperlink ref="B241" r:id="rId239"/>
-    <hyperlink ref="B242" r:id="rId240"/>
-    <hyperlink ref="B243" r:id="rId241"/>
-    <hyperlink ref="B244" r:id="rId242"/>
-    <hyperlink ref="B245" r:id="rId243"/>
-    <hyperlink ref="B246" r:id="rId244"/>
-    <hyperlink ref="B247" r:id="rId245"/>
-    <hyperlink ref="B248" r:id="rId246"/>
-    <hyperlink ref="B249" r:id="rId247"/>
-    <hyperlink ref="B250" r:id="rId248"/>
-    <hyperlink ref="B251" r:id="rId249"/>
-    <hyperlink ref="B252" r:id="rId250"/>
-    <hyperlink ref="B253" r:id="rId251"/>
-    <hyperlink ref="B254" r:id="rId252"/>
-    <hyperlink ref="B255" r:id="rId253"/>
-    <hyperlink ref="B256" r:id="rId254"/>
-    <hyperlink ref="B257" r:id="rId255"/>
-    <hyperlink ref="B258" r:id="rId256"/>
-    <hyperlink ref="B259" r:id="rId257"/>
-    <hyperlink ref="B260" r:id="rId258"/>
-    <hyperlink ref="B261" r:id="rId259"/>
-    <hyperlink ref="B262" r:id="rId260"/>
-    <hyperlink ref="B263" r:id="rId261"/>
-    <hyperlink ref="B264" r:id="rId262"/>
-    <hyperlink ref="B265" r:id="rId263"/>
-    <hyperlink ref="B266" r:id="rId264"/>
-    <hyperlink ref="B267" r:id="rId265"/>
-    <hyperlink ref="B268" r:id="rId266"/>
-    <hyperlink ref="B269" r:id="rId267"/>
-    <hyperlink ref="B270" r:id="rId268"/>
-    <hyperlink ref="B271" r:id="rId269"/>
-    <hyperlink ref="B272" r:id="rId270"/>
-    <hyperlink ref="B273" r:id="rId271"/>
-    <hyperlink ref="B274" r:id="rId272"/>
-    <hyperlink ref="B275" r:id="rId273"/>
-    <hyperlink ref="B276" r:id="rId274"/>
-    <hyperlink ref="B277" r:id="rId275"/>
-    <hyperlink ref="B278" r:id="rId276"/>
-    <hyperlink ref="B279" r:id="rId277"/>
-    <hyperlink ref="B280" r:id="rId278"/>
-    <hyperlink ref="B281" r:id="rId279"/>
-    <hyperlink ref="B282" r:id="rId280"/>
-    <hyperlink ref="B283" r:id="rId281"/>
-    <hyperlink ref="B284" r:id="rId282"/>
-    <hyperlink ref="B285" r:id="rId283"/>
-    <hyperlink ref="B286" r:id="rId284"/>
-    <hyperlink ref="B287" r:id="rId285"/>
-    <hyperlink ref="B288" r:id="rId286"/>
-    <hyperlink ref="B289" r:id="rId287"/>
-    <hyperlink ref="B290" r:id="rId288"/>
-    <hyperlink ref="B291" r:id="rId289"/>
-    <hyperlink ref="B292" r:id="rId290"/>
-    <hyperlink ref="B293" r:id="rId291"/>
-    <hyperlink ref="B294" r:id="rId292"/>
-    <hyperlink ref="B295" r:id="rId293"/>
-    <hyperlink ref="B296" r:id="rId294"/>
-    <hyperlink ref="B297" r:id="rId295"/>
-    <hyperlink ref="B298" r:id="rId296"/>
-    <hyperlink ref="B299" r:id="rId297"/>
-    <hyperlink ref="B300" r:id="rId298"/>
-    <hyperlink ref="B301" r:id="rId299"/>
-    <hyperlink ref="B302" r:id="rId300"/>
-    <hyperlink ref="B303" r:id="rId301"/>
-    <hyperlink ref="B304" r:id="rId302"/>
-    <hyperlink ref="B305" r:id="rId303"/>
-    <hyperlink ref="B306" r:id="rId304"/>
-    <hyperlink ref="B307" r:id="rId305"/>
-    <hyperlink ref="B308" r:id="rId306"/>
-    <hyperlink ref="B309" r:id="rId307"/>
-    <hyperlink ref="B310" r:id="rId308"/>
-    <hyperlink ref="B311" r:id="rId309"/>
-    <hyperlink ref="B312" r:id="rId310"/>
-    <hyperlink ref="B313" r:id="rId311"/>
-    <hyperlink ref="B314" r:id="rId312"/>
-    <hyperlink ref="B315" r:id="rId313"/>
-    <hyperlink ref="B316" r:id="rId314"/>
-    <hyperlink ref="B317" r:id="rId315"/>
-    <hyperlink ref="B318" r:id="rId316"/>
-    <hyperlink ref="B319" r:id="rId317"/>
-    <hyperlink ref="B320" r:id="rId318"/>
-    <hyperlink ref="B321" r:id="rId319"/>
-    <hyperlink ref="B322" r:id="rId320"/>
-    <hyperlink ref="B323" r:id="rId321"/>
-    <hyperlink ref="B324" r:id="rId322"/>
-    <hyperlink ref="B325" r:id="rId323"/>
-    <hyperlink ref="B326" r:id="rId324"/>
-    <hyperlink ref="B327" r:id="rId325"/>
-    <hyperlink ref="B328" r:id="rId326"/>
-    <hyperlink ref="B329" r:id="rId327"/>
-    <hyperlink ref="B330" r:id="rId328"/>
-    <hyperlink ref="B331" r:id="rId329"/>
-    <hyperlink ref="B332" r:id="rId330"/>
-    <hyperlink ref="B333" r:id="rId331"/>
-    <hyperlink ref="B334" r:id="rId332"/>
-    <hyperlink ref="B335" r:id="rId333"/>
-    <hyperlink ref="B336" r:id="rId334"/>
-    <hyperlink ref="B337" r:id="rId335"/>
-    <hyperlink ref="B338" r:id="rId336"/>
-    <hyperlink ref="B339" r:id="rId337"/>
-    <hyperlink ref="B340" r:id="rId338"/>
-    <hyperlink ref="B341" r:id="rId339"/>
-    <hyperlink ref="B342" r:id="rId340"/>
-    <hyperlink ref="B343" r:id="rId341"/>
-    <hyperlink ref="B344" r:id="rId342"/>
-    <hyperlink ref="B345" r:id="rId343"/>
-    <hyperlink ref="B346" r:id="rId344"/>
-    <hyperlink ref="B347" r:id="rId345"/>
-    <hyperlink ref="B348" r:id="rId346"/>
-    <hyperlink ref="B349" r:id="rId347"/>
-    <hyperlink ref="B350" r:id="rId348"/>
-    <hyperlink ref="B351" r:id="rId349"/>
-    <hyperlink ref="B352" r:id="rId350"/>
-    <hyperlink ref="B353" r:id="rId351"/>
-    <hyperlink ref="B354" r:id="rId352"/>
-    <hyperlink ref="B355" r:id="rId353"/>
-    <hyperlink ref="B356" r:id="rId354"/>
-    <hyperlink ref="B357" r:id="rId355"/>
-    <hyperlink ref="B358" r:id="rId356"/>
-    <hyperlink ref="B359" r:id="rId357"/>
-    <hyperlink ref="B360" r:id="rId358"/>
-    <hyperlink ref="B361" r:id="rId359"/>
-    <hyperlink ref="B362" r:id="rId360"/>
-    <hyperlink ref="B363" r:id="rId361"/>
-    <hyperlink ref="B364" r:id="rId362"/>
-    <hyperlink ref="B365" r:id="rId363"/>
-    <hyperlink ref="B366" r:id="rId364"/>
-    <hyperlink ref="B367" r:id="rId365"/>
-    <hyperlink ref="B368" r:id="rId366"/>
-    <hyperlink ref="B369" r:id="rId367"/>
-    <hyperlink ref="B370" r:id="rId368"/>
-    <hyperlink ref="B371" r:id="rId369"/>
-    <hyperlink ref="B372" r:id="rId370"/>
-    <hyperlink ref="B373" r:id="rId371"/>
-    <hyperlink ref="B374" r:id="rId372"/>
-    <hyperlink ref="B375" r:id="rId373"/>
-    <hyperlink ref="B376" r:id="rId374"/>
-    <hyperlink ref="B377" r:id="rId375"/>
-    <hyperlink ref="B378" r:id="rId376"/>
-    <hyperlink ref="B379" r:id="rId377"/>
-    <hyperlink ref="B380" r:id="rId378"/>
-    <hyperlink ref="B381" r:id="rId379"/>
-    <hyperlink ref="B382" r:id="rId380"/>
-    <hyperlink ref="B383" r:id="rId381"/>
-    <hyperlink ref="B384" r:id="rId382"/>
-    <hyperlink ref="B385" r:id="rId383"/>
-    <hyperlink ref="B386" r:id="rId384"/>
-    <hyperlink ref="B387" r:id="rId385"/>
-    <hyperlink ref="B388" r:id="rId386"/>
-    <hyperlink ref="B389" r:id="rId387"/>
-    <hyperlink ref="B390" r:id="rId388"/>
-    <hyperlink ref="B391" r:id="rId389"/>
-    <hyperlink ref="B392" r:id="rId390"/>
-    <hyperlink ref="B393" r:id="rId391"/>
-    <hyperlink ref="B394" r:id="rId392"/>
-    <hyperlink ref="B395" r:id="rId393"/>
-    <hyperlink ref="B396" r:id="rId394"/>
-    <hyperlink ref="B397" r:id="rId395"/>
-    <hyperlink ref="B398" r:id="rId396"/>
-    <hyperlink ref="B399" r:id="rId397"/>
-    <hyperlink ref="B400" r:id="rId398"/>
-    <hyperlink ref="B401" r:id="rId399"/>
-    <hyperlink ref="B402" r:id="rId400"/>
-    <hyperlink ref="B403" r:id="rId401"/>
-    <hyperlink ref="B404" r:id="rId402"/>
-    <hyperlink ref="B405" r:id="rId403"/>
-    <hyperlink ref="B406" r:id="rId404"/>
-    <hyperlink ref="B407" r:id="rId405"/>
-    <hyperlink ref="B408" r:id="rId406"/>
-    <hyperlink ref="B409" r:id="rId407"/>
-    <hyperlink ref="B410" r:id="rId408"/>
-    <hyperlink ref="B411" r:id="rId409"/>
-    <hyperlink ref="B412" r:id="rId410"/>
-    <hyperlink ref="B413" r:id="rId411"/>
-    <hyperlink ref="B414" r:id="rId412"/>
-    <hyperlink ref="B415" r:id="rId413"/>
-    <hyperlink ref="B416" r:id="rId414"/>
-    <hyperlink ref="B417" r:id="rId415"/>
-    <hyperlink ref="B418" r:id="rId416"/>
-    <hyperlink ref="B419" r:id="rId417"/>
-    <hyperlink ref="B420" r:id="rId418"/>
-    <hyperlink ref="B421" r:id="rId419"/>
-    <hyperlink ref="B422" r:id="rId420"/>
-    <hyperlink ref="B423" r:id="rId421"/>
-    <hyperlink ref="B424" r:id="rId422"/>
-    <hyperlink ref="B425" r:id="rId423"/>
-    <hyperlink ref="B426" r:id="rId424"/>
-    <hyperlink ref="B427" r:id="rId425"/>
-    <hyperlink ref="B428" r:id="rId426"/>
-    <hyperlink ref="B429" r:id="rId427"/>
-    <hyperlink ref="B430" r:id="rId428"/>
-    <hyperlink ref="B431" r:id="rId429"/>
-    <hyperlink ref="B432" r:id="rId430"/>
-    <hyperlink ref="B433" r:id="rId431"/>
-    <hyperlink ref="B434" r:id="rId432"/>
-    <hyperlink ref="B435" r:id="rId433"/>
-    <hyperlink ref="B436" r:id="rId434"/>
-    <hyperlink ref="B437" r:id="rId435"/>
-    <hyperlink ref="B438" r:id="rId436"/>
-    <hyperlink ref="B439" r:id="rId437"/>
-    <hyperlink ref="B440" r:id="rId438"/>
-    <hyperlink ref="B441" r:id="rId439"/>
-    <hyperlink ref="B442" r:id="rId440"/>
-    <hyperlink ref="B443" r:id="rId441"/>
-    <hyperlink ref="B444" r:id="rId442"/>
-    <hyperlink ref="B445" r:id="rId443"/>
-    <hyperlink ref="B446" r:id="rId444"/>
-    <hyperlink ref="B447" r:id="rId445"/>
-    <hyperlink ref="B448" r:id="rId446"/>
-    <hyperlink ref="B449" r:id="rId447"/>
-    <hyperlink ref="B450" r:id="rId448"/>
-    <hyperlink ref="B451" r:id="rId449"/>
-    <hyperlink ref="B452" r:id="rId450"/>
-    <hyperlink ref="B453" r:id="rId451"/>
-    <hyperlink ref="B454" r:id="rId452"/>
-    <hyperlink ref="B455" r:id="rId453"/>
-    <hyperlink ref="B456" r:id="rId454"/>
-    <hyperlink ref="B457" r:id="rId455"/>
-    <hyperlink ref="B458" r:id="rId456"/>
-    <hyperlink ref="B459" r:id="rId457"/>
-    <hyperlink ref="B460" r:id="rId458"/>
-    <hyperlink ref="B461" r:id="rId459"/>
-    <hyperlink ref="B462" r:id="rId460"/>
-    <hyperlink ref="B463" r:id="rId461"/>
-    <hyperlink ref="B464" r:id="rId462"/>
-    <hyperlink ref="B465" r:id="rId463"/>
-    <hyperlink ref="B466" r:id="rId464"/>
-    <hyperlink ref="B467" r:id="rId465"/>
-    <hyperlink ref="B468" r:id="rId466"/>
-    <hyperlink ref="B469" r:id="rId467"/>
-    <hyperlink ref="B470" r:id="rId468"/>
-    <hyperlink ref="B471" r:id="rId469"/>
-    <hyperlink ref="B472" r:id="rId470"/>
-    <hyperlink ref="B473" r:id="rId471"/>
-    <hyperlink ref="B474" r:id="rId472"/>
-    <hyperlink ref="B475" r:id="rId473"/>
-    <hyperlink ref="B476" r:id="rId474"/>
-    <hyperlink ref="B477" r:id="rId475"/>
-    <hyperlink ref="B478" r:id="rId476"/>
-    <hyperlink ref="B479" r:id="rId477"/>
-    <hyperlink ref="B480" r:id="rId478"/>
-    <hyperlink ref="B481" r:id="rId479"/>
-    <hyperlink ref="B482" r:id="rId480"/>
-    <hyperlink ref="B483" r:id="rId481"/>
-    <hyperlink ref="B484" r:id="rId482"/>
-    <hyperlink ref="B485" r:id="rId483"/>
-    <hyperlink ref="B486" r:id="rId484"/>
-    <hyperlink ref="B487" r:id="rId485"/>
-    <hyperlink ref="B488" r:id="rId486"/>
-    <hyperlink ref="B489" r:id="rId487"/>
-    <hyperlink ref="B490" r:id="rId488"/>
-    <hyperlink ref="B491" r:id="rId489"/>
-    <hyperlink ref="B492" r:id="rId490"/>
-    <hyperlink ref="B493" r:id="rId491"/>
-    <hyperlink ref="B494" r:id="rId492"/>
-    <hyperlink ref="B495" r:id="rId493"/>
-    <hyperlink ref="B496" r:id="rId494"/>
-    <hyperlink ref="B497" r:id="rId495"/>
-    <hyperlink ref="B498" r:id="rId496"/>
-    <hyperlink ref="B499" r:id="rId497"/>
-    <hyperlink ref="B500" r:id="rId498"/>
-    <hyperlink ref="B501" r:id="rId499"/>
-    <hyperlink ref="B502" r:id="rId500"/>
-    <hyperlink ref="B503" r:id="rId501"/>
-    <hyperlink ref="B504" r:id="rId502"/>
-    <hyperlink ref="B505" r:id="rId503"/>
-    <hyperlink ref="B506" r:id="rId504"/>
-    <hyperlink ref="B507" r:id="rId505"/>
-    <hyperlink ref="B508" r:id="rId506"/>
-    <hyperlink ref="B509" r:id="rId507"/>
-    <hyperlink ref="B510" r:id="rId508"/>
-    <hyperlink ref="B511" r:id="rId509"/>
-    <hyperlink ref="B512" r:id="rId510"/>
-    <hyperlink ref="B513" r:id="rId511"/>
-    <hyperlink ref="B514" r:id="rId512"/>
-    <hyperlink ref="B515" r:id="rId513"/>
-    <hyperlink ref="B516" r:id="rId514"/>
-    <hyperlink ref="B517" r:id="rId515"/>
-    <hyperlink ref="B518" r:id="rId516"/>
-    <hyperlink ref="B519" r:id="rId517"/>
-    <hyperlink ref="B520" r:id="rId518"/>
-    <hyperlink ref="B521" r:id="rId519"/>
-    <hyperlink ref="B522" r:id="rId520"/>
-    <hyperlink ref="B523" r:id="rId521"/>
-    <hyperlink ref="B524" r:id="rId522"/>
-    <hyperlink ref="B525" r:id="rId523"/>
-    <hyperlink ref="B526" r:id="rId524"/>
-    <hyperlink ref="B527" r:id="rId525"/>
-    <hyperlink ref="B528" r:id="rId526"/>
-    <hyperlink ref="B529" r:id="rId527"/>
-    <hyperlink ref="B530" r:id="rId528"/>
-    <hyperlink ref="B531" r:id="rId529"/>
-    <hyperlink ref="B532" r:id="rId530"/>
-    <hyperlink ref="B533" r:id="rId531"/>
-    <hyperlink ref="B534" r:id="rId532"/>
-    <hyperlink ref="B535" r:id="rId533"/>
-    <hyperlink ref="B536" r:id="rId534"/>
-    <hyperlink ref="B537" r:id="rId535"/>
-    <hyperlink ref="B538" r:id="rId536"/>
-    <hyperlink ref="B539" r:id="rId537"/>
-    <hyperlink ref="B540" r:id="rId538"/>
-    <hyperlink ref="B541" r:id="rId539"/>
-    <hyperlink ref="B542" r:id="rId540"/>
-    <hyperlink ref="B543" r:id="rId541"/>
-    <hyperlink ref="B544" r:id="rId542"/>
-    <hyperlink ref="B545" r:id="rId543"/>
-    <hyperlink ref="B546" r:id="rId544"/>
-    <hyperlink ref="B547" r:id="rId545"/>
-    <hyperlink ref="B548" r:id="rId546"/>
-    <hyperlink ref="B549" r:id="rId547"/>
-    <hyperlink ref="B550" r:id="rId548"/>
-    <hyperlink ref="B551" r:id="rId549"/>
-    <hyperlink ref="B552" r:id="rId550"/>
-    <hyperlink ref="B553" r:id="rId551"/>
-    <hyperlink ref="B554" r:id="rId552"/>
-    <hyperlink ref="B555" r:id="rId553"/>
-    <hyperlink ref="B556" r:id="rId554"/>
-    <hyperlink ref="B557" r:id="rId555"/>
-    <hyperlink ref="B558" r:id="rId556"/>
-    <hyperlink ref="B559" r:id="rId557"/>
-    <hyperlink ref="B560" r:id="rId558"/>
-    <hyperlink ref="B561" r:id="rId559"/>
-    <hyperlink ref="B562" r:id="rId560"/>
-    <hyperlink ref="B563" r:id="rId561"/>
-    <hyperlink ref="B564" r:id="rId562"/>
-    <hyperlink ref="B565" r:id="rId563"/>
-    <hyperlink ref="B566" r:id="rId564"/>
-    <hyperlink ref="B567" r:id="rId565"/>
-    <hyperlink ref="B568" r:id="rId566"/>
-    <hyperlink ref="B569" r:id="rId567"/>
-    <hyperlink ref="B570" r:id="rId568"/>
-    <hyperlink ref="B571" r:id="rId569"/>
-    <hyperlink ref="B572" r:id="rId570"/>
-    <hyperlink ref="B573" r:id="rId571"/>
-    <hyperlink ref="B574" r:id="rId572"/>
-    <hyperlink ref="B575" r:id="rId573"/>
-    <hyperlink ref="B576" r:id="rId574"/>
-    <hyperlink ref="B577" r:id="rId575"/>
-    <hyperlink ref="B578" r:id="rId576"/>
-    <hyperlink ref="B579" r:id="rId577"/>
-    <hyperlink ref="B580" r:id="rId578"/>
-    <hyperlink ref="B581" r:id="rId579"/>
-    <hyperlink ref="B582" r:id="rId580"/>
-    <hyperlink ref="B583" r:id="rId581"/>
-    <hyperlink ref="B584" r:id="rId582"/>
-    <hyperlink ref="B585" r:id="rId583"/>
-    <hyperlink ref="B586" r:id="rId584"/>
-    <hyperlink ref="B587" r:id="rId585"/>
-    <hyperlink ref="B588" r:id="rId586"/>
-    <hyperlink ref="B589" r:id="rId587"/>
-    <hyperlink ref="B590" r:id="rId588"/>
-    <hyperlink ref="B591" r:id="rId589"/>
-    <hyperlink ref="B592" r:id="rId590"/>
-    <hyperlink ref="B593" r:id="rId591"/>
-    <hyperlink ref="B594" r:id="rId592"/>
-    <hyperlink ref="B595" r:id="rId593"/>
-    <hyperlink ref="B596" r:id="rId594"/>
-    <hyperlink ref="B597" r:id="rId595"/>
-    <hyperlink ref="B598" r:id="rId596"/>
-    <hyperlink ref="B599" r:id="rId597"/>
-    <hyperlink ref="B600" r:id="rId598"/>
-    <hyperlink ref="B601" r:id="rId599"/>
-    <hyperlink ref="B602" r:id="rId600"/>
-    <hyperlink ref="B603" r:id="rId601"/>
-    <hyperlink ref="B604" r:id="rId602"/>
-    <hyperlink ref="B605" r:id="rId603"/>
-    <hyperlink ref="B606" r:id="rId604"/>
-    <hyperlink ref="B607" r:id="rId605"/>
-    <hyperlink ref="B608" r:id="rId606"/>
-    <hyperlink ref="B609" r:id="rId607"/>
-    <hyperlink ref="B610" r:id="rId608"/>
-    <hyperlink ref="B611" r:id="rId609"/>
-    <hyperlink ref="B612" r:id="rId610"/>
-    <hyperlink ref="B613" r:id="rId611"/>
-    <hyperlink ref="B614" r:id="rId612"/>
-    <hyperlink ref="B615" r:id="rId613"/>
-    <hyperlink ref="B616" r:id="rId614"/>
-    <hyperlink ref="B617" r:id="rId615"/>
-    <hyperlink ref="B618" r:id="rId616"/>
-    <hyperlink ref="B619" r:id="rId617"/>
-    <hyperlink ref="B620" r:id="rId618"/>
-    <hyperlink ref="B621" r:id="rId619"/>
-    <hyperlink ref="B622" r:id="rId620"/>
-    <hyperlink ref="B623" r:id="rId621"/>
-    <hyperlink ref="B624" r:id="rId622"/>
-    <hyperlink ref="B625" r:id="rId623"/>
-    <hyperlink ref="B626" r:id="rId624"/>
-    <hyperlink ref="B627" r:id="rId625"/>
-    <hyperlink ref="B628" r:id="rId626"/>
-    <hyperlink ref="B629" r:id="rId627"/>
-    <hyperlink ref="B630" r:id="rId628"/>
-    <hyperlink ref="B631" r:id="rId629"/>
-    <hyperlink ref="B632" r:id="rId630"/>
-    <hyperlink ref="B633" r:id="rId631"/>
-    <hyperlink ref="B634" r:id="rId632"/>
-    <hyperlink ref="B635" r:id="rId633"/>
-    <hyperlink ref="B636" r:id="rId634"/>
-    <hyperlink ref="B637" r:id="rId635"/>
-    <hyperlink ref="B638" r:id="rId636"/>
-    <hyperlink ref="B639" r:id="rId637"/>
-    <hyperlink ref="B640" r:id="rId638"/>
-    <hyperlink ref="B641" r:id="rId639"/>
-    <hyperlink ref="B642" r:id="rId640"/>
-    <hyperlink ref="B643" r:id="rId641"/>
-    <hyperlink ref="B644" r:id="rId642"/>
-    <hyperlink ref="B645" r:id="rId643"/>
-    <hyperlink ref="B646" r:id="rId644"/>
-    <hyperlink ref="B647" r:id="rId645"/>
-    <hyperlink ref="B648" r:id="rId646"/>
-    <hyperlink ref="B649" r:id="rId647"/>
-    <hyperlink ref="B650" r:id="rId648"/>
-    <hyperlink ref="B651" r:id="rId649"/>
-    <hyperlink ref="B652" r:id="rId650"/>
-    <hyperlink ref="B653" r:id="rId651"/>
-    <hyperlink ref="B654" r:id="rId652"/>
-    <hyperlink ref="B655" r:id="rId653"/>
-    <hyperlink ref="B656" r:id="rId654"/>
-    <hyperlink ref="B657" r:id="rId655"/>
-    <hyperlink ref="B658" r:id="rId656"/>
-    <hyperlink ref="B659" r:id="rId657"/>
-    <hyperlink ref="B660" r:id="rId658"/>
-    <hyperlink ref="B661" r:id="rId659"/>
-    <hyperlink ref="B662" r:id="rId660"/>
-    <hyperlink ref="B663" r:id="rId661"/>
-    <hyperlink ref="B664" r:id="rId662"/>
-    <hyperlink ref="B665" r:id="rId663"/>
-    <hyperlink ref="B666" r:id="rId664"/>
-    <hyperlink ref="B667" r:id="rId665"/>
-    <hyperlink ref="B668" r:id="rId666"/>
-    <hyperlink ref="B669" r:id="rId667"/>
-    <hyperlink ref="B670" r:id="rId668"/>
-    <hyperlink ref="B671" r:id="rId669"/>
-    <hyperlink ref="B672" r:id="rId670"/>
-    <hyperlink ref="B673" r:id="rId671"/>
-    <hyperlink ref="B674" r:id="rId672"/>
-    <hyperlink ref="B675" r:id="rId673"/>
-    <hyperlink ref="B676" r:id="rId674"/>
-    <hyperlink ref="B677" r:id="rId675"/>
-    <hyperlink ref="B678" r:id="rId676"/>
-    <hyperlink ref="B679" r:id="rId677"/>
-    <hyperlink ref="B680" r:id="rId678"/>
-    <hyperlink ref="B681" r:id="rId679"/>
-    <hyperlink ref="B682" r:id="rId680"/>
-    <hyperlink ref="B683" r:id="rId681"/>
-    <hyperlink ref="B684" r:id="rId682"/>
-    <hyperlink ref="B685" r:id="rId683"/>
-    <hyperlink ref="B686" r:id="rId684"/>
-    <hyperlink ref="B687" r:id="rId685"/>
-    <hyperlink ref="B688" r:id="rId686"/>
-    <hyperlink ref="B689" r:id="rId687"/>
-    <hyperlink ref="B690" r:id="rId688"/>
-    <hyperlink ref="B691" r:id="rId689"/>
-    <hyperlink ref="B692" r:id="rId690"/>
-    <hyperlink ref="B693" r:id="rId691"/>
-    <hyperlink ref="B694" r:id="rId692"/>
-    <hyperlink ref="B695" r:id="rId693"/>
-    <hyperlink ref="B696" r:id="rId694"/>
-    <hyperlink ref="B697" r:id="rId695"/>
-    <hyperlink ref="B698" r:id="rId696"/>
-    <hyperlink ref="B699" r:id="rId697"/>
-    <hyperlink ref="B700" r:id="rId698"/>
-    <hyperlink ref="B701" r:id="rId699"/>
-    <hyperlink ref="B702" r:id="rId700"/>
-    <hyperlink ref="B703" r:id="rId701"/>
-    <hyperlink ref="B704" r:id="rId702"/>
-    <hyperlink ref="B705" r:id="rId703"/>
-    <hyperlink ref="B706" r:id="rId704"/>
-    <hyperlink ref="B707" r:id="rId705"/>
-    <hyperlink ref="B708" r:id="rId706"/>
-    <hyperlink ref="B709" r:id="rId707"/>
-    <hyperlink ref="B710" r:id="rId708"/>
-    <hyperlink ref="B711" r:id="rId709"/>
-    <hyperlink ref="B712" r:id="rId710"/>
-    <hyperlink ref="B713" r:id="rId711"/>
-    <hyperlink ref="B714" r:id="rId712"/>
-    <hyperlink ref="B715" r:id="rId713"/>
-    <hyperlink ref="B716" r:id="rId714"/>
-    <hyperlink ref="B717" r:id="rId715"/>
-    <hyperlink ref="B718" r:id="rId716"/>
-    <hyperlink ref="B719" r:id="rId717"/>
-    <hyperlink ref="B720" r:id="rId718"/>
-    <hyperlink ref="B721" r:id="rId719"/>
-    <hyperlink ref="B722" r:id="rId720"/>
-    <hyperlink ref="B723" r:id="rId721"/>
-    <hyperlink ref="B724" r:id="rId722"/>
-    <hyperlink ref="B725" r:id="rId723"/>
-    <hyperlink ref="B726" r:id="rId724"/>
-    <hyperlink ref="B727" r:id="rId725"/>
-    <hyperlink ref="B728" r:id="rId726"/>
-    <hyperlink ref="B729" r:id="rId727"/>
-    <hyperlink ref="B730" r:id="rId728"/>
-    <hyperlink ref="B731" r:id="rId729"/>
-    <hyperlink ref="B732" r:id="rId730"/>
-    <hyperlink ref="B733" r:id="rId731"/>
-    <hyperlink ref="B734" r:id="rId732"/>
-    <hyperlink ref="B735" r:id="rId733"/>
-    <hyperlink ref="B736" r:id="rId734"/>
-    <hyperlink ref="B737" r:id="rId735"/>
-    <hyperlink ref="B738" r:id="rId736"/>
-    <hyperlink ref="B739" r:id="rId737"/>
-    <hyperlink ref="B740" r:id="rId738"/>
-    <hyperlink ref="B741" r:id="rId739"/>
-    <hyperlink ref="B742" r:id="rId740"/>
-    <hyperlink ref="B743" r:id="rId741"/>
-    <hyperlink ref="B744" r:id="rId742"/>
-    <hyperlink ref="B745" r:id="rId743"/>
-    <hyperlink ref="B746" r:id="rId744"/>
-    <hyperlink ref="B747" r:id="rId745"/>
-    <hyperlink ref="B748" r:id="rId746"/>
-    <hyperlink ref="B749" r:id="rId747"/>
-    <hyperlink ref="B750" r:id="rId748"/>
-    <hyperlink ref="B751" r:id="rId749"/>
-    <hyperlink ref="B752" r:id="rId750"/>
-    <hyperlink ref="B753" r:id="rId751"/>
-    <hyperlink ref="B754" r:id="rId752"/>
-    <hyperlink ref="B755" r:id="rId753"/>
-    <hyperlink ref="B756" r:id="rId754"/>
-    <hyperlink ref="B757" r:id="rId755"/>
-    <hyperlink ref="B758" r:id="rId756"/>
-    <hyperlink ref="B759" r:id="rId757"/>
-    <hyperlink ref="B760" r:id="rId758"/>
-    <hyperlink ref="B761" r:id="rId759"/>
-    <hyperlink ref="B762" r:id="rId760"/>
-    <hyperlink ref="B763" r:id="rId761"/>
-    <hyperlink ref="B764" r:id="rId762"/>
-    <hyperlink ref="B765" r:id="rId763"/>
-    <hyperlink ref="B766" r:id="rId764"/>
-    <hyperlink ref="B767" r:id="rId765"/>
-    <hyperlink ref="B768" r:id="rId766"/>
-    <hyperlink ref="B769" r:id="rId767"/>
-    <hyperlink ref="B770" r:id="rId768"/>
-    <hyperlink ref="B771" r:id="rId769"/>
-    <hyperlink ref="B772" r:id="rId770"/>
-    <hyperlink ref="B773" r:id="rId771"/>
-    <hyperlink ref="B774" r:id="rId772"/>
-    <hyperlink ref="B775" r:id="rId773"/>
-    <hyperlink ref="B776" r:id="rId774"/>
-    <hyperlink ref="B777" r:id="rId775"/>
-    <hyperlink ref="B778" r:id="rId776"/>
-    <hyperlink ref="B779" r:id="rId777"/>
-    <hyperlink ref="B780" r:id="rId778"/>
-    <hyperlink ref="B781" r:id="rId779"/>
-    <hyperlink ref="B782" r:id="rId780"/>
-    <hyperlink ref="B783" r:id="rId781"/>
-    <hyperlink ref="B784" r:id="rId782"/>
-    <hyperlink ref="B785" r:id="rId783"/>
-    <hyperlink ref="B786" r:id="rId784"/>
-    <hyperlink ref="B787" r:id="rId785"/>
-    <hyperlink ref="B788" r:id="rId786"/>
-    <hyperlink ref="B789" r:id="rId787"/>
-    <hyperlink ref="B790" r:id="rId788"/>
-    <hyperlink ref="B791" r:id="rId789"/>
-    <hyperlink ref="B792" r:id="rId790"/>
-    <hyperlink ref="B793" r:id="rId791"/>
-    <hyperlink ref="B794" r:id="rId792"/>
-    <hyperlink ref="B795" r:id="rId793"/>
-    <hyperlink ref="B796" r:id="rId794"/>
-    <hyperlink ref="B797" r:id="rId795"/>
-    <hyperlink ref="B798" r:id="rId796"/>
-    <hyperlink ref="B799" r:id="rId797"/>
-    <hyperlink ref="B800" r:id="rId798"/>
-    <hyperlink ref="B801" r:id="rId799"/>
-    <hyperlink ref="B802" r:id="rId800"/>
-    <hyperlink ref="B803" r:id="rId801"/>
-    <hyperlink ref="B804" r:id="rId802"/>
-    <hyperlink ref="B805" r:id="rId803"/>
-    <hyperlink ref="B806" r:id="rId804"/>
-    <hyperlink ref="B807" r:id="rId805"/>
-    <hyperlink ref="B808" r:id="rId806"/>
-    <hyperlink ref="B809" r:id="rId807"/>
-    <hyperlink ref="B810" r:id="rId808"/>
-    <hyperlink ref="B811" r:id="rId809"/>
-    <hyperlink ref="B812" r:id="rId810"/>
-    <hyperlink ref="B813" r:id="rId811"/>
-    <hyperlink ref="B814" r:id="rId812"/>
-    <hyperlink ref="B815" r:id="rId813"/>
-    <hyperlink ref="B816" r:id="rId814"/>
-    <hyperlink ref="B817" r:id="rId815"/>
-    <hyperlink ref="B818" r:id="rId816"/>
-    <hyperlink ref="B819" r:id="rId817"/>
-    <hyperlink ref="B820" r:id="rId818"/>
-    <hyperlink ref="B821" r:id="rId819"/>
-    <hyperlink ref="B822" r:id="rId820"/>
-    <hyperlink ref="B823" r:id="rId821"/>
-    <hyperlink ref="B824" r:id="rId822"/>
-    <hyperlink ref="B825" r:id="rId823"/>
-    <hyperlink ref="B826" r:id="rId824"/>
-    <hyperlink ref="B827" r:id="rId825"/>
-    <hyperlink ref="B828" r:id="rId826"/>
-    <hyperlink ref="B829" r:id="rId827"/>
-    <hyperlink ref="B830" r:id="rId828"/>
-    <hyperlink ref="B831" r:id="rId829"/>
-    <hyperlink ref="B832" r:id="rId830"/>
-    <hyperlink ref="B833" r:id="rId831"/>
-    <hyperlink ref="B834" r:id="rId832"/>
-    <hyperlink ref="B835" r:id="rId833"/>
-    <hyperlink ref="B836" r:id="rId834"/>
-    <hyperlink ref="B837" r:id="rId835"/>
-    <hyperlink ref="B838" r:id="rId836"/>
-    <hyperlink ref="B839" r:id="rId837"/>
-    <hyperlink ref="B840" r:id="rId838"/>
-    <hyperlink ref="B841" r:id="rId839"/>
-    <hyperlink ref="B842" r:id="rId840"/>
-    <hyperlink ref="B843" r:id="rId841"/>
-    <hyperlink ref="B844" r:id="rId842"/>
-    <hyperlink ref="B845" r:id="rId843"/>
-    <hyperlink ref="B846" r:id="rId844"/>
-    <hyperlink ref="B847" r:id="rId845"/>
-    <hyperlink ref="B848" r:id="rId846"/>
-    <hyperlink ref="B849" r:id="rId847"/>
-    <hyperlink ref="B850" r:id="rId848"/>
-    <hyperlink ref="B851" r:id="rId849"/>
-    <hyperlink ref="B852" r:id="rId850"/>
-    <hyperlink ref="B853" r:id="rId851"/>
-    <hyperlink ref="B854" r:id="rId852"/>
-    <hyperlink ref="B855" r:id="rId853"/>
-    <hyperlink ref="B856" r:id="rId854"/>
-    <hyperlink ref="B857" r:id="rId855"/>
-    <hyperlink ref="B858" r:id="rId856"/>
-    <hyperlink ref="B859" r:id="rId857"/>
-    <hyperlink ref="B860" r:id="rId858"/>
-    <hyperlink ref="B861" r:id="rId859"/>
-    <hyperlink ref="B862" r:id="rId860"/>
-    <hyperlink ref="B863" r:id="rId861"/>
-    <hyperlink ref="B864" r:id="rId862"/>
-    <hyperlink ref="B865" r:id="rId863"/>
-    <hyperlink ref="B866" r:id="rId864"/>
-    <hyperlink ref="B867" r:id="rId865"/>
-    <hyperlink ref="B868" r:id="rId866"/>
-    <hyperlink ref="B869" r:id="rId867"/>
-    <hyperlink ref="B870" r:id="rId868"/>
-    <hyperlink ref="B871" r:id="rId869"/>
-    <hyperlink ref="B872" r:id="rId870"/>
-    <hyperlink ref="B873" r:id="rId871"/>
-    <hyperlink ref="B874" r:id="rId872"/>
-    <hyperlink ref="B875" r:id="rId873"/>
-    <hyperlink ref="B876" r:id="rId874"/>
-    <hyperlink ref="B877" r:id="rId875"/>
-    <hyperlink ref="B878" r:id="rId876"/>
-    <hyperlink ref="B879" r:id="rId877"/>
-    <hyperlink ref="B880" r:id="rId878"/>
-    <hyperlink ref="B881" r:id="rId879"/>
-    <hyperlink ref="B882" r:id="rId880"/>
-    <hyperlink ref="B883" r:id="rId881"/>
-    <hyperlink ref="B884" r:id="rId882"/>
-    <hyperlink ref="B885" r:id="rId883"/>
-    <hyperlink ref="B886" r:id="rId884"/>
-    <hyperlink ref="B887" r:id="rId885"/>
-    <hyperlink ref="B888" r:id="rId886"/>
-    <hyperlink ref="B889" r:id="rId887"/>
-    <hyperlink ref="B890" r:id="rId888"/>
-    <hyperlink ref="B891" r:id="rId889"/>
-    <hyperlink ref="B892" r:id="rId890"/>
-    <hyperlink ref="B893" r:id="rId891"/>
-    <hyperlink ref="B894" r:id="rId892"/>
-    <hyperlink ref="B895" r:id="rId893"/>
-    <hyperlink ref="B896" r:id="rId894"/>
-    <hyperlink ref="B897" r:id="rId895"/>
-    <hyperlink ref="B898" r:id="rId896"/>
-    <hyperlink ref="B899" r:id="rId897"/>
-    <hyperlink ref="B900" r:id="rId898"/>
-    <hyperlink ref="B901" r:id="rId899"/>
-    <hyperlink ref="B902" r:id="rId900"/>
-    <hyperlink ref="B903" r:id="rId901"/>
-    <hyperlink ref="B904" r:id="rId902"/>
-    <hyperlink ref="B905" r:id="rId903"/>
-    <hyperlink ref="B906" r:id="rId904"/>
-    <hyperlink ref="B907" r:id="rId905"/>
-    <hyperlink ref="B908" r:id="rId906"/>
-    <hyperlink ref="B909" r:id="rId907"/>
-    <hyperlink ref="B910" r:id="rId908"/>
-    <hyperlink ref="B911" r:id="rId909"/>
-    <hyperlink ref="B912" r:id="rId910"/>
-    <hyperlink ref="B913" r:id="rId911"/>
-    <hyperlink ref="B914" r:id="rId912"/>
-    <hyperlink ref="B915" r:id="rId913"/>
-    <hyperlink ref="B916" r:id="rId914"/>
-    <hyperlink ref="B917" r:id="rId915"/>
-    <hyperlink ref="B918" r:id="rId916"/>
-    <hyperlink ref="B919" r:id="rId917"/>
-    <hyperlink ref="B920" r:id="rId918"/>
-    <hyperlink ref="B921" r:id="rId919"/>
-    <hyperlink ref="B922" r:id="rId920"/>
-    <hyperlink ref="B923" r:id="rId921"/>
-    <hyperlink ref="B924" r:id="rId922"/>
-    <hyperlink ref="B925" r:id="rId923"/>
-    <hyperlink ref="B926" r:id="rId924"/>
-    <hyperlink ref="B927" r:id="rId925"/>
-    <hyperlink ref="B928" r:id="rId926"/>
-    <hyperlink ref="B929" r:id="rId927"/>
-    <hyperlink ref="B930" r:id="rId928"/>
-    <hyperlink ref="B931" r:id="rId929"/>
-    <hyperlink ref="B932" r:id="rId930"/>
-    <hyperlink ref="B933" r:id="rId931"/>
-    <hyperlink ref="B934" r:id="rId932"/>
-    <hyperlink ref="B935" r:id="rId933"/>
-    <hyperlink ref="B936" r:id="rId934"/>
-    <hyperlink ref="B937" r:id="rId935"/>
-    <hyperlink ref="B938" r:id="rId936"/>
-    <hyperlink ref="B939" r:id="rId937"/>
-    <hyperlink ref="B940" r:id="rId938"/>
-    <hyperlink ref="B941" r:id="rId939"/>
-    <hyperlink ref="B942" r:id="rId940"/>
-    <hyperlink ref="B943" r:id="rId941"/>
-    <hyperlink ref="B944" r:id="rId942"/>
-    <hyperlink ref="B945" r:id="rId943"/>
-    <hyperlink ref="B946" r:id="rId944"/>
-    <hyperlink ref="B947" r:id="rId945"/>
-    <hyperlink ref="B948" r:id="rId946"/>
-    <hyperlink ref="B949" r:id="rId947"/>
-    <hyperlink ref="B950" r:id="rId948"/>
-    <hyperlink ref="B951" r:id="rId949"/>
-    <hyperlink ref="B952" r:id="rId950"/>
-    <hyperlink ref="B953" r:id="rId951"/>
-    <hyperlink ref="B954" r:id="rId952"/>
-    <hyperlink ref="B955" r:id="rId953"/>
-    <hyperlink ref="B956" r:id="rId954"/>
-    <hyperlink ref="B957" r:id="rId955"/>
-    <hyperlink ref="B958" r:id="rId956"/>
-    <hyperlink ref="B959" r:id="rId957"/>
-    <hyperlink ref="B960" r:id="rId958"/>
-    <hyperlink ref="B961" r:id="rId959"/>
-    <hyperlink ref="B962" r:id="rId960"/>
-    <hyperlink ref="B963" r:id="rId961"/>
-    <hyperlink ref="B964" r:id="rId962"/>
-    <hyperlink ref="B965" r:id="rId963"/>
+    <hyperlink ref="B3" r:id="rId963"/>
+    <hyperlink ref="B4" r:id="rId964"/>
+    <hyperlink ref="B5" r:id="rId965"/>
+    <hyperlink ref="B6" r:id="rId966"/>
+    <hyperlink ref="B7" r:id="rId967"/>
+    <hyperlink ref="B8" r:id="rId968"/>
+    <hyperlink ref="B9" r:id="rId969"/>
+    <hyperlink ref="B10" r:id="rId970"/>
+    <hyperlink ref="B11" r:id="rId971"/>
+    <hyperlink ref="B12" r:id="rId972"/>
+    <hyperlink ref="B13" r:id="rId973"/>
+    <hyperlink ref="B14" r:id="rId974"/>
+    <hyperlink ref="B15" r:id="rId975"/>
+    <hyperlink ref="B16" r:id="rId976"/>
+    <hyperlink ref="B17" r:id="rId977"/>
+    <hyperlink ref="B18" r:id="rId978"/>
+    <hyperlink ref="B19" r:id="rId979"/>
+    <hyperlink ref="B20" r:id="rId980"/>
+    <hyperlink ref="B21" r:id="rId981"/>
+    <hyperlink ref="B22" r:id="rId982"/>
+    <hyperlink ref="B23" r:id="rId983"/>
+    <hyperlink ref="B24" r:id="rId984"/>
+    <hyperlink ref="B25" r:id="rId985"/>
+    <hyperlink ref="B26" r:id="rId986"/>
+    <hyperlink ref="B27" r:id="rId987"/>
+    <hyperlink ref="B28" r:id="rId988"/>
+    <hyperlink ref="B29" r:id="rId989"/>
+    <hyperlink ref="B30" r:id="rId990"/>
+    <hyperlink ref="B31" r:id="rId991"/>
+    <hyperlink ref="B32" r:id="rId992"/>
+    <hyperlink ref="B33" r:id="rId993"/>
+    <hyperlink ref="B34" r:id="rId994"/>
+    <hyperlink ref="B35" r:id="rId995"/>
+    <hyperlink ref="B36" r:id="rId996"/>
+    <hyperlink ref="B37" r:id="rId997"/>
+    <hyperlink ref="B38" r:id="rId998"/>
+    <hyperlink ref="B39" r:id="rId999"/>
+    <hyperlink ref="B40" r:id="rId1000"/>
+    <hyperlink ref="B41" r:id="rId1001"/>
+    <hyperlink ref="B42" r:id="rId1002"/>
+    <hyperlink ref="B43" r:id="rId1003"/>
+    <hyperlink ref="B44" r:id="rId1004"/>
+    <hyperlink ref="B45" r:id="rId1005"/>
+    <hyperlink ref="B46" r:id="rId1006"/>
+    <hyperlink ref="B47" r:id="rId1007"/>
+    <hyperlink ref="B48" r:id="rId1008"/>
+    <hyperlink ref="B49" r:id="rId1009"/>
+    <hyperlink ref="B50" r:id="rId1010"/>
+    <hyperlink ref="B51" r:id="rId1011"/>
+    <hyperlink ref="B52" r:id="rId1012"/>
+    <hyperlink ref="B53" r:id="rId1013"/>
+    <hyperlink ref="B54" r:id="rId1014"/>
+    <hyperlink ref="B55" r:id="rId1015"/>
+    <hyperlink ref="B56" r:id="rId1016"/>
+    <hyperlink ref="B57" r:id="rId1017"/>
+    <hyperlink ref="B58" r:id="rId1018"/>
+    <hyperlink ref="B59" r:id="rId1019"/>
+    <hyperlink ref="B60" r:id="rId1020"/>
+    <hyperlink ref="B61" r:id="rId1021"/>
+    <hyperlink ref="B62" r:id="rId1022"/>
+    <hyperlink ref="B63" r:id="rId1023"/>
+    <hyperlink ref="B64" r:id="rId1024"/>
+    <hyperlink ref="B65" r:id="rId1025"/>
+    <hyperlink ref="B66" r:id="rId1026"/>
+    <hyperlink ref="B67" r:id="rId1027"/>
+    <hyperlink ref="B68" r:id="rId1028"/>
+    <hyperlink ref="B69" r:id="rId1029"/>
+    <hyperlink ref="B70" r:id="rId1030"/>
+    <hyperlink ref="B71" r:id="rId1031"/>
+    <hyperlink ref="B72" r:id="rId1032"/>
+    <hyperlink ref="B73" r:id="rId1033"/>
+    <hyperlink ref="B74" r:id="rId1034"/>
+    <hyperlink ref="B75" r:id="rId1035"/>
+    <hyperlink ref="B76" r:id="rId1036"/>
+    <hyperlink ref="B77" r:id="rId1037"/>
+    <hyperlink ref="B78" r:id="rId1038"/>
+    <hyperlink ref="B79" r:id="rId1039"/>
+    <hyperlink ref="B80" r:id="rId1040"/>
+    <hyperlink ref="B81" r:id="rId1041"/>
+    <hyperlink ref="B82" r:id="rId1042"/>
+    <hyperlink ref="B83" r:id="rId1043"/>
+    <hyperlink ref="B84" r:id="rId1044"/>
+    <hyperlink ref="B85" r:id="rId1045"/>
+    <hyperlink ref="B86" r:id="rId1046"/>
+    <hyperlink ref="B87" r:id="rId1047"/>
+    <hyperlink ref="B88" r:id="rId1048"/>
+    <hyperlink ref="B89" r:id="rId1049"/>
+    <hyperlink ref="B90" r:id="rId1050"/>
+    <hyperlink ref="B91" r:id="rId1051"/>
+    <hyperlink ref="B92" r:id="rId1052"/>
+    <hyperlink ref="B93" r:id="rId1053"/>
+    <hyperlink ref="B94" r:id="rId1054"/>
+    <hyperlink ref="B95" r:id="rId1055"/>
+    <hyperlink ref="B96" r:id="rId1056"/>
+    <hyperlink ref="B97" r:id="rId1057"/>
+    <hyperlink ref="B98" r:id="rId1058"/>
+    <hyperlink ref="B99" r:id="rId1059"/>
+    <hyperlink ref="B100" r:id="rId1060"/>
+    <hyperlink ref="B101" r:id="rId1061"/>
+    <hyperlink ref="B102" r:id="rId1062"/>
+    <hyperlink ref="B103" r:id="rId1063"/>
+    <hyperlink ref="B104" r:id="rId1064"/>
+    <hyperlink ref="B105" r:id="rId1065"/>
+    <hyperlink ref="B106" r:id="rId1066"/>
+    <hyperlink ref="B107" r:id="rId1067"/>
+    <hyperlink ref="B108" r:id="rId1068"/>
+    <hyperlink ref="B109" r:id="rId1069"/>
+    <hyperlink ref="B110" r:id="rId1070"/>
+    <hyperlink ref="B111" r:id="rId1071"/>
+    <hyperlink ref="B112" r:id="rId1072"/>
+    <hyperlink ref="B113" r:id="rId1073"/>
+    <hyperlink ref="B114" r:id="rId1074"/>
+    <hyperlink ref="B115" r:id="rId1075"/>
+    <hyperlink ref="B116" r:id="rId1076"/>
+    <hyperlink ref="B117" r:id="rId1077"/>
+    <hyperlink ref="B118" r:id="rId1078"/>
+    <hyperlink ref="B119" r:id="rId1079"/>
+    <hyperlink ref="B120" r:id="rId1080"/>
+    <hyperlink ref="B121" r:id="rId1081"/>
+    <hyperlink ref="B122" r:id="rId1082"/>
+    <hyperlink ref="B123" r:id="rId1083"/>
+    <hyperlink ref="B124" r:id="rId1084"/>
+    <hyperlink ref="B125" r:id="rId1085"/>
+    <hyperlink ref="B126" r:id="rId1086"/>
+    <hyperlink ref="B127" r:id="rId1087"/>
+    <hyperlink ref="B128" r:id="rId1088"/>
+    <hyperlink ref="B129" r:id="rId1089"/>
+    <hyperlink ref="B130" r:id="rId1090"/>
+    <hyperlink ref="B131" r:id="rId1091"/>
+    <hyperlink ref="B132" r:id="rId1092"/>
+    <hyperlink ref="B133" r:id="rId1093"/>
+    <hyperlink ref="B134" r:id="rId1094"/>
+    <hyperlink ref="B135" r:id="rId1095"/>
+    <hyperlink ref="B136" r:id="rId1096"/>
+    <hyperlink ref="B137" r:id="rId1097"/>
+    <hyperlink ref="B138" r:id="rId1098"/>
+    <hyperlink ref="B139" r:id="rId1099"/>
+    <hyperlink ref="B140" r:id="rId1100"/>
+    <hyperlink ref="B141" r:id="rId1101"/>
+    <hyperlink ref="B142" r:id="rId1102"/>
+    <hyperlink ref="B143" r:id="rId1103"/>
+    <hyperlink ref="B144" r:id="rId1104"/>
+    <hyperlink ref="B145" r:id="rId1105"/>
+    <hyperlink ref="B146" r:id="rId1106"/>
+    <hyperlink ref="B147" r:id="rId1107"/>
+    <hyperlink ref="B148" r:id="rId1108"/>
+    <hyperlink ref="B149" r:id="rId1109"/>
+    <hyperlink ref="B150" r:id="rId1110"/>
+    <hyperlink ref="B151" r:id="rId1111"/>
+    <hyperlink ref="B152" r:id="rId1112"/>
+    <hyperlink ref="B153" r:id="rId1113"/>
+    <hyperlink ref="B154" r:id="rId1114"/>
+    <hyperlink ref="B155" r:id="rId1115"/>
+    <hyperlink ref="B156" r:id="rId1116"/>
+    <hyperlink ref="B157" r:id="rId1117"/>
+    <hyperlink ref="B158" r:id="rId1118"/>
+    <hyperlink ref="B159" r:id="rId1119"/>
+    <hyperlink ref="B160" r:id="rId1120"/>
+    <hyperlink ref="B161" r:id="rId1121"/>
+    <hyperlink ref="B162" r:id="rId1122"/>
+    <hyperlink ref="B163" r:id="rId1123"/>
+    <hyperlink ref="B164" r:id="rId1124"/>
+    <hyperlink ref="B165" r:id="rId1125"/>
+    <hyperlink ref="B166" r:id="rId1126"/>
+    <hyperlink ref="B167" r:id="rId1127"/>
+    <hyperlink ref="B168" r:id="rId1128"/>
+    <hyperlink ref="B169" r:id="rId1129"/>
+    <hyperlink ref="B170" r:id="rId1130"/>
+    <hyperlink ref="B171" r:id="rId1131"/>
+    <hyperlink ref="B172" r:id="rId1132"/>
+    <hyperlink ref="B173" r:id="rId1133"/>
+    <hyperlink ref="B174" r:id="rId1134"/>
+    <hyperlink ref="B175" r:id="rId1135"/>
+    <hyperlink ref="B176" r:id="rId1136"/>
+    <hyperlink ref="B177" r:id="rId1137"/>
+    <hyperlink ref="B178" r:id="rId1138"/>
+    <hyperlink ref="B179" r:id="rId1139"/>
+    <hyperlink ref="B180" r:id="rId1140"/>
+    <hyperlink ref="B181" r:id="rId1141"/>
+    <hyperlink ref="B182" r:id="rId1142"/>
+    <hyperlink ref="B183" r:id="rId1143"/>
+    <hyperlink ref="B184" r:id="rId1144"/>
+    <hyperlink ref="B185" r:id="rId1145"/>
+    <hyperlink ref="B186" r:id="rId1146"/>
+    <hyperlink ref="B187" r:id="rId1147"/>
+    <hyperlink ref="B188" r:id="rId1148"/>
+    <hyperlink ref="B189" r:id="rId1149"/>
+    <hyperlink ref="B190" r:id="rId1150"/>
+    <hyperlink ref="B191" r:id="rId1151"/>
+    <hyperlink ref="B192" r:id="rId1152"/>
+    <hyperlink ref="B193" r:id="rId1153"/>
+    <hyperlink ref="B194" r:id="rId1154"/>
+    <hyperlink ref="B195" r:id="rId1155"/>
+    <hyperlink ref="B196" r:id="rId1156"/>
+    <hyperlink ref="B197" r:id="rId1157"/>
+    <hyperlink ref="B198" r:id="rId1158"/>
+    <hyperlink ref="B199" r:id="rId1159"/>
+    <hyperlink ref="B200" r:id="rId1160"/>
+    <hyperlink ref="B201" r:id="rId1161"/>
+    <hyperlink ref="B202" r:id="rId1162"/>
+    <hyperlink ref="B203" r:id="rId1163"/>
+    <hyperlink ref="B204" r:id="rId1164"/>
+    <hyperlink ref="B205" r:id="rId1165"/>
+    <hyperlink ref="B206" r:id="rId1166"/>
+    <hyperlink ref="B207" r:id="rId1167"/>
+    <hyperlink ref="B208" r:id="rId1168"/>
+    <hyperlink ref="B209" r:id="rId1169"/>
+    <hyperlink ref="B210" r:id="rId1170"/>
+    <hyperlink ref="B211" r:id="rId1171"/>
+    <hyperlink ref="B212" r:id="rId1172"/>
+    <hyperlink ref="B213" r:id="rId1173"/>
+    <hyperlink ref="B214" r:id="rId1174"/>
+    <hyperlink ref="B215" r:id="rId1175"/>
+    <hyperlink ref="B216" r:id="rId1176"/>
+    <hyperlink ref="B217" r:id="rId1177"/>
+    <hyperlink ref="B218" r:id="rId1178"/>
+    <hyperlink ref="B219" r:id="rId1179"/>
+    <hyperlink ref="B220" r:id="rId1180"/>
+    <hyperlink ref="B221" r:id="rId1181"/>
+    <hyperlink ref="B222" r:id="rId1182"/>
+    <hyperlink ref="B223" r:id="rId1183"/>
+    <hyperlink ref="B224" r:id="rId1184"/>
+    <hyperlink ref="B225" r:id="rId1185"/>
+    <hyperlink ref="B226" r:id="rId1186"/>
+    <hyperlink ref="B227" r:id="rId1187"/>
+    <hyperlink ref="B228" r:id="rId1188"/>
+    <hyperlink ref="B229" r:id="rId1189"/>
+    <hyperlink ref="B230" r:id="rId1190"/>
+    <hyperlink ref="B231" r:id="rId1191"/>
+    <hyperlink ref="B232" r:id="rId1192"/>
+    <hyperlink ref="B233" r:id="rId1193"/>
+    <hyperlink ref="B234" r:id="rId1194"/>
+    <hyperlink ref="B235" r:id="rId1195"/>
+    <hyperlink ref="B236" r:id="rId1196"/>
+    <hyperlink ref="B237" r:id="rId1197"/>
+    <hyperlink ref="B238" r:id="rId1198"/>
+    <hyperlink ref="B239" r:id="rId1199"/>
+    <hyperlink ref="B240" r:id="rId1200"/>
+    <hyperlink ref="B241" r:id="rId1201"/>
+    <hyperlink ref="B242" r:id="rId1202"/>
+    <hyperlink ref="B243" r:id="rId1203"/>
+    <hyperlink ref="B244" r:id="rId1204"/>
+    <hyperlink ref="B245" r:id="rId1205"/>
+    <hyperlink ref="B246" r:id="rId1206"/>
+    <hyperlink ref="B247" r:id="rId1207"/>
+    <hyperlink ref="B248" r:id="rId1208"/>
+    <hyperlink ref="B249" r:id="rId1209"/>
+    <hyperlink ref="B250" r:id="rId1210"/>
+    <hyperlink ref="B251" r:id="rId1211"/>
+    <hyperlink ref="B252" r:id="rId1212"/>
+    <hyperlink ref="B253" r:id="rId1213"/>
+    <hyperlink ref="B254" r:id="rId1214"/>
+    <hyperlink ref="B255" r:id="rId1215"/>
+    <hyperlink ref="B256" r:id="rId1216"/>
+    <hyperlink ref="B257" r:id="rId1217"/>
+    <hyperlink ref="B258" r:id="rId1218"/>
+    <hyperlink ref="B259" r:id="rId1219"/>
+    <hyperlink ref="B260" r:id="rId1220"/>
+    <hyperlink ref="B261" r:id="rId1221"/>
+    <hyperlink ref="B262" r:id="rId1222"/>
+    <hyperlink ref="B263" r:id="rId1223"/>
+    <hyperlink ref="B264" r:id="rId1224"/>
+    <hyperlink ref="B265" r:id="rId1225"/>
+    <hyperlink ref="B266" r:id="rId1226"/>
+    <hyperlink ref="B267" r:id="rId1227"/>
+    <hyperlink ref="B268" r:id="rId1228"/>
+    <hyperlink ref="B269" r:id="rId1229"/>
+    <hyperlink ref="B270" r:id="rId1230"/>
+    <hyperlink ref="B271" r:id="rId1231"/>
+    <hyperlink ref="B272" r:id="rId1232"/>
+    <hyperlink ref="B273" r:id="rId1233"/>
+    <hyperlink ref="B274" r:id="rId1234"/>
+    <hyperlink ref="B275" r:id="rId1235"/>
+    <hyperlink ref="B276" r:id="rId1236"/>
+    <hyperlink ref="B277" r:id="rId1237"/>
+    <hyperlink ref="B278" r:id="rId1238"/>
+    <hyperlink ref="B279" r:id="rId1239"/>
+    <hyperlink ref="B280" r:id="rId1240"/>
+    <hyperlink ref="B281" r:id="rId1241"/>
+    <hyperlink ref="B282" r:id="rId1242"/>
+    <hyperlink ref="B283" r:id="rId1243"/>
+    <hyperlink ref="B284" r:id="rId1244"/>
+    <hyperlink ref="B285" r:id="rId1245"/>
+    <hyperlink ref="B286" r:id="rId1246"/>
+    <hyperlink ref="B287" r:id="rId1247"/>
+    <hyperlink ref="B288" r:id="rId1248"/>
+    <hyperlink ref="B289" r:id="rId1249"/>
+    <hyperlink ref="B290" r:id="rId1250"/>
+    <hyperlink ref="B291" r:id="rId1251"/>
+    <hyperlink ref="B292" r:id="rId1252"/>
+    <hyperlink ref="B293" r:id="rId1253"/>
+    <hyperlink ref="B294" r:id="rId1254"/>
+    <hyperlink ref="B295" r:id="rId1255"/>
+    <hyperlink ref="B296" r:id="rId1256"/>
+    <hyperlink ref="B297" r:id="rId1257"/>
+    <hyperlink ref="B298" r:id="rId1258"/>
+    <hyperlink ref="B299" r:id="rId1259"/>
+    <hyperlink ref="B300" r:id="rId1260"/>
+    <hyperlink ref="B301" r:id="rId1261"/>
+    <hyperlink ref="B302" r:id="rId1262"/>
+    <hyperlink ref="B303" r:id="rId1263"/>
+    <hyperlink ref="B304" r:id="rId1264"/>
+    <hyperlink ref="B305" r:id="rId1265"/>
+    <hyperlink ref="B306" r:id="rId1266"/>
+    <hyperlink ref="B307" r:id="rId1267"/>
+    <hyperlink ref="B308" r:id="rId1268"/>
+    <hyperlink ref="B309" r:id="rId1269"/>
+    <hyperlink ref="B310" r:id="rId1270"/>
+    <hyperlink ref="B311" r:id="rId1271"/>
+    <hyperlink ref="B312" r:id="rId1272"/>
+    <hyperlink ref="B313" r:id="rId1273"/>
+    <hyperlink ref="B314" r:id="rId1274"/>
+    <hyperlink ref="B315" r:id="rId1275"/>
+    <hyperlink ref="B316" r:id="rId1276"/>
+    <hyperlink ref="B317" r:id="rId1277"/>
+    <hyperlink ref="B318" r:id="rId1278"/>
+    <hyperlink ref="B319" r:id="rId1279"/>
+    <hyperlink ref="B320" r:id="rId1280"/>
+    <hyperlink ref="B321" r:id="rId1281"/>
+    <hyperlink ref="B322" r:id="rId1282"/>
+    <hyperlink ref="B323" r:id="rId1283"/>
+    <hyperlink ref="B324" r:id="rId1284"/>
+    <hyperlink ref="B325" r:id="rId1285"/>
+    <hyperlink ref="B326" r:id="rId1286"/>
+    <hyperlink ref="B327" r:id="rId1287"/>
+    <hyperlink ref="B328" r:id="rId1288"/>
+    <hyperlink ref="B329" r:id="rId1289"/>
+    <hyperlink ref="B330" r:id="rId1290"/>
+    <hyperlink ref="B331" r:id="rId1291"/>
+    <hyperlink ref="B332" r:id="rId1292"/>
+    <hyperlink ref="B333" r:id="rId1293"/>
+    <hyperlink ref="B334" r:id="rId1294"/>
+    <hyperlink ref="B335" r:id="rId1295"/>
+    <hyperlink ref="B336" r:id="rId1296"/>
+    <hyperlink ref="B337" r:id="rId1297"/>
+    <hyperlink ref="B338" r:id="rId1298"/>
+    <hyperlink ref="B339" r:id="rId1299"/>
+    <hyperlink ref="B340" r:id="rId1300"/>
+    <hyperlink ref="B341" r:id="rId1301"/>
+    <hyperlink ref="B342" r:id="rId1302"/>
+    <hyperlink ref="B343" r:id="rId1303"/>
+    <hyperlink ref="B344" r:id="rId1304"/>
+    <hyperlink ref="B345" r:id="rId1305"/>
+    <hyperlink ref="B346" r:id="rId1306"/>
+    <hyperlink ref="B347" r:id="rId1307"/>
+    <hyperlink ref="B348" r:id="rId1308"/>
+    <hyperlink ref="B349" r:id="rId1309"/>
+    <hyperlink ref="B350" r:id="rId1310"/>
+    <hyperlink ref="B351" r:id="rId1311"/>
+    <hyperlink ref="B352" r:id="rId1312"/>
+    <hyperlink ref="B353" r:id="rId1313"/>
+    <hyperlink ref="B354" r:id="rId1314"/>
+    <hyperlink ref="B355" r:id="rId1315"/>
+    <hyperlink ref="B356" r:id="rId1316"/>
+    <hyperlink ref="B357" r:id="rId1317"/>
+    <hyperlink ref="B358" r:id="rId1318"/>
+    <hyperlink ref="B359" r:id="rId1319"/>
+    <hyperlink ref="B360" r:id="rId1320"/>
+    <hyperlink ref="B361" r:id="rId1321"/>
+    <hyperlink ref="B362" r:id="rId1322"/>
+    <hyperlink ref="B363" r:id="rId1323"/>
+    <hyperlink ref="B364" r:id="rId1324"/>
+    <hyperlink ref="B365" r:id="rId1325"/>
+    <hyperlink ref="B366" r:id="rId1326"/>
+    <hyperlink ref="B367" r:id="rId1327"/>
+    <hyperlink ref="B368" r:id="rId1328"/>
+    <hyperlink ref="B369" r:id="rId1329"/>
+    <hyperlink ref="B370" r:id="rId1330"/>
+    <hyperlink ref="B371" r:id="rId1331"/>
+    <hyperlink ref="B372" r:id="rId1332"/>
+    <hyperlink ref="B373" r:id="rId1333"/>
+    <hyperlink ref="B374" r:id="rId1334"/>
+    <hyperlink ref="B375" r:id="rId1335"/>
+    <hyperlink ref="B376" r:id="rId1336"/>
+    <hyperlink ref="B377" r:id="rId1337"/>
+    <hyperlink ref="B378" r:id="rId1338"/>
+    <hyperlink ref="B379" r:id="rId1339"/>
+    <hyperlink ref="B380" r:id="rId1340"/>
+    <hyperlink ref="B381" r:id="rId1341"/>
+    <hyperlink ref="B382" r:id="rId1342"/>
+    <hyperlink ref="B383" r:id="rId1343"/>
+    <hyperlink ref="B384" r:id="rId1344"/>
+    <hyperlink ref="B385" r:id="rId1345"/>
+    <hyperlink ref="B386" r:id="rId1346"/>
+    <hyperlink ref="B387" r:id="rId1347"/>
+    <hyperlink ref="B388" r:id="rId1348"/>
+    <hyperlink ref="B389" r:id="rId1349"/>
+    <hyperlink ref="B390" r:id="rId1350"/>
+    <hyperlink ref="B391" r:id="rId1351"/>
+    <hyperlink ref="B392" r:id="rId1352"/>
+    <hyperlink ref="B393" r:id="rId1353"/>
+    <hyperlink ref="B394" r:id="rId1354"/>
+    <hyperlink ref="B395" r:id="rId1355"/>
+    <hyperlink ref="B396" r:id="rId1356"/>
+    <hyperlink ref="B397" r:id="rId1357"/>
+    <hyperlink ref="B398" r:id="rId1358"/>
+    <hyperlink ref="B399" r:id="rId1359"/>
+    <hyperlink ref="B400" r:id="rId1360"/>
+    <hyperlink ref="B401" r:id="rId1361"/>
+    <hyperlink ref="B402" r:id="rId1362"/>
+    <hyperlink ref="B403" r:id="rId1363"/>
+    <hyperlink ref="B404" r:id="rId1364"/>
+    <hyperlink ref="B405" r:id="rId1365"/>
+    <hyperlink ref="B406" r:id="rId1366"/>
+    <hyperlink ref="B407" r:id="rId1367"/>
+    <hyperlink ref="B408" r:id="rId1368"/>
+    <hyperlink ref="B409" r:id="rId1369"/>
+    <hyperlink ref="B410" r:id="rId1370"/>
+    <hyperlink ref="B411" r:id="rId1371"/>
+    <hyperlink ref="B412" r:id="rId1372"/>
+    <hyperlink ref="B413" r:id="rId1373"/>
+    <hyperlink ref="B414" r:id="rId1374"/>
+    <hyperlink ref="B415" r:id="rId1375"/>
+    <hyperlink ref="B416" r:id="rId1376"/>
+    <hyperlink ref="B417" r:id="rId1377"/>
+    <hyperlink ref="B418" r:id="rId1378"/>
+    <hyperlink ref="B419" r:id="rId1379"/>
+    <hyperlink ref="B420" r:id="rId1380"/>
+    <hyperlink ref="B421" r:id="rId1381"/>
+    <hyperlink ref="B422" r:id="rId1382"/>
+    <hyperlink ref="B423" r:id="rId1383"/>
+    <hyperlink ref="B424" r:id="rId1384"/>
+    <hyperlink ref="B425" r:id="rId1385"/>
+    <hyperlink ref="B426" r:id="rId1386"/>
+    <hyperlink ref="B427" r:id="rId1387"/>
+    <hyperlink ref="B428" r:id="rId1388"/>
+    <hyperlink ref="B429" r:id="rId1389"/>
+    <hyperlink ref="B430" r:id="rId1390"/>
+    <hyperlink ref="B431" r:id="rId1391"/>
+    <hyperlink ref="B432" r:id="rId1392"/>
+    <hyperlink ref="B433" r:id="rId1393"/>
+    <hyperlink ref="B434" r:id="rId1394"/>
+    <hyperlink ref="B435" r:id="rId1395"/>
+    <hyperlink ref="B436" r:id="rId1396"/>
+    <hyperlink ref="B437" r:id="rId1397"/>
+    <hyperlink ref="B438" r:id="rId1398"/>
+    <hyperlink ref="B439" r:id="rId1399"/>
+    <hyperlink ref="B440" r:id="rId1400"/>
+    <hyperlink ref="B441" r:id="rId1401"/>
+    <hyperlink ref="B442" r:id="rId1402"/>
+    <hyperlink ref="B443" r:id="rId1403"/>
+    <hyperlink ref="B444" r:id="rId1404"/>
+    <hyperlink ref="B445" r:id="rId1405"/>
+    <hyperlink ref="B446" r:id="rId1406"/>
+    <hyperlink ref="B447" r:id="rId1407"/>
+    <hyperlink ref="B448" r:id="rId1408"/>
+    <hyperlink ref="B449" r:id="rId1409"/>
+    <hyperlink ref="B450" r:id="rId1410"/>
+    <hyperlink ref="B451" r:id="rId1411"/>
+    <hyperlink ref="B452" r:id="rId1412"/>
+    <hyperlink ref="B453" r:id="rId1413"/>
+    <hyperlink ref="B454" r:id="rId1414"/>
+    <hyperlink ref="B455" r:id="rId1415"/>
+    <hyperlink ref="B456" r:id="rId1416"/>
+    <hyperlink ref="B457" r:id="rId1417"/>
+    <hyperlink ref="B458" r:id="rId1418"/>
+    <hyperlink ref="B459" r:id="rId1419"/>
+    <hyperlink ref="B460" r:id="rId1420"/>
+    <hyperlink ref="B461" r:id="rId1421"/>
+    <hyperlink ref="B462" r:id="rId1422"/>
+    <hyperlink ref="B463" r:id="rId1423"/>
+    <hyperlink ref="B464" r:id="rId1424"/>
+    <hyperlink ref="B465" r:id="rId1425"/>
+    <hyperlink ref="B466" r:id="rId1426"/>
+    <hyperlink ref="B467" r:id="rId1427"/>
+    <hyperlink ref="B468" r:id="rId1428"/>
+    <hyperlink ref="B469" r:id="rId1429"/>
+    <hyperlink ref="B470" r:id="rId1430"/>
+    <hyperlink ref="B471" r:id="rId1431"/>
+    <hyperlink ref="B472" r:id="rId1432"/>
+    <hyperlink ref="B473" r:id="rId1433"/>
+    <hyperlink ref="B474" r:id="rId1434"/>
+    <hyperlink ref="B475" r:id="rId1435"/>
+    <hyperlink ref="B476" r:id="rId1436"/>
+    <hyperlink ref="B477" r:id="rId1437"/>
+    <hyperlink ref="B478" r:id="rId1438"/>
+    <hyperlink ref="B479" r:id="rId1439"/>
+    <hyperlink ref="B480" r:id="rId1440"/>
+    <hyperlink ref="B481" r:id="rId1441"/>
+    <hyperlink ref="B482" r:id="rId1442"/>
+    <hyperlink ref="B483" r:id="rId1443"/>
+    <hyperlink ref="B484" r:id="rId1444"/>
+    <hyperlink ref="B485" r:id="rId1445"/>
+    <hyperlink ref="B486" r:id="rId1446"/>
+    <hyperlink ref="B487" r:id="rId1447"/>
+    <hyperlink ref="B488" r:id="rId1448"/>
+    <hyperlink ref="B489" r:id="rId1449"/>
+    <hyperlink ref="B490" r:id="rId1450"/>
+    <hyperlink ref="B491" r:id="rId1451"/>
+    <hyperlink ref="B492" r:id="rId1452"/>
+    <hyperlink ref="B493" r:id="rId1453"/>
+    <hyperlink ref="B494" r:id="rId1454"/>
+    <hyperlink ref="B495" r:id="rId1455"/>
+    <hyperlink ref="B496" r:id="rId1456"/>
+    <hyperlink ref="B497" r:id="rId1457"/>
+    <hyperlink ref="B498" r:id="rId1458"/>
+    <hyperlink ref="B499" r:id="rId1459"/>
+    <hyperlink ref="B500" r:id="rId1460"/>
+    <hyperlink ref="B501" r:id="rId1461"/>
+    <hyperlink ref="B502" r:id="rId1462"/>
+    <hyperlink ref="B503" r:id="rId1463"/>
+    <hyperlink ref="B504" r:id="rId1464"/>
+    <hyperlink ref="B505" r:id="rId1465"/>
+    <hyperlink ref="B506" r:id="rId1466"/>
+    <hyperlink ref="B507" r:id="rId1467"/>
+    <hyperlink ref="B508" r:id="rId1468"/>
+    <hyperlink ref="B509" r:id="rId1469"/>
+    <hyperlink ref="B510" r:id="rId1470"/>
+    <hyperlink ref="B511" r:id="rId1471"/>
+    <hyperlink ref="B512" r:id="rId1472"/>
+    <hyperlink ref="B513" r:id="rId1473"/>
+    <hyperlink ref="B514" r:id="rId1474"/>
+    <hyperlink ref="B515" r:id="rId1475"/>
+    <hyperlink ref="B516" r:id="rId1476"/>
+    <hyperlink ref="B517" r:id="rId1477"/>
+    <hyperlink ref="B518" r:id="rId1478"/>
+    <hyperlink ref="B519" r:id="rId1479"/>
+    <hyperlink ref="B520" r:id="rId1480"/>
+    <hyperlink ref="B521" r:id="rId1481"/>
+    <hyperlink ref="B522" r:id="rId1482"/>
+    <hyperlink ref="B523" r:id="rId1483"/>
+    <hyperlink ref="B524" r:id="rId1484"/>
+    <hyperlink ref="B525" r:id="rId1485"/>
+    <hyperlink ref="B526" r:id="rId1486"/>
+    <hyperlink ref="B527" r:id="rId1487"/>
+    <hyperlink ref="B528" r:id="rId1488"/>
+    <hyperlink ref="B529" r:id="rId1489"/>
+    <hyperlink ref="B530" r:id="rId1490"/>
+    <hyperlink ref="B531" r:id="rId1491"/>
+    <hyperlink ref="B532" r:id="rId1492"/>
+    <hyperlink ref="B533" r:id="rId1493"/>
+    <hyperlink ref="B534" r:id="rId1494"/>
+    <hyperlink ref="B535" r:id="rId1495"/>
+    <hyperlink ref="B536" r:id="rId1496"/>
+    <hyperlink ref="B537" r:id="rId1497"/>
+    <hyperlink ref="B538" r:id="rId1498"/>
+    <hyperlink ref="B539" r:id="rId1499"/>
+    <hyperlink ref="B540" r:id="rId1500"/>
+    <hyperlink ref="B541" r:id="rId1501"/>
+    <hyperlink ref="B542" r:id="rId1502"/>
+    <hyperlink ref="B543" r:id="rId1503"/>
+    <hyperlink ref="B544" r:id="rId1504"/>
+    <hyperlink ref="B545" r:id="rId1505"/>
+    <hyperlink ref="B546" r:id="rId1506"/>
+    <hyperlink ref="B547" r:id="rId1507"/>
+    <hyperlink ref="B548" r:id="rId1508"/>
+    <hyperlink ref="B549" r:id="rId1509"/>
+    <hyperlink ref="B550" r:id="rId1510"/>
+    <hyperlink ref="B551" r:id="rId1511"/>
+    <hyperlink ref="B552" r:id="rId1512"/>
+    <hyperlink ref="B553" r:id="rId1513"/>
+    <hyperlink ref="B554" r:id="rId1514"/>
+    <hyperlink ref="B555" r:id="rId1515"/>
+    <hyperlink ref="B556" r:id="rId1516"/>
+    <hyperlink ref="B557" r:id="rId1517"/>
+    <hyperlink ref="B558" r:id="rId1518"/>
+    <hyperlink ref="B559" r:id="rId1519"/>
+    <hyperlink ref="B560" r:id="rId1520"/>
+    <hyperlink ref="B561" r:id="rId1521"/>
+    <hyperlink ref="B562" r:id="rId1522"/>
+    <hyperlink ref="B563" r:id="rId1523"/>
+    <hyperlink ref="B564" r:id="rId1524"/>
+    <hyperlink ref="B565" r:id="rId1525"/>
+    <hyperlink ref="B566" r:id="rId1526"/>
+    <hyperlink ref="B567" r:id="rId1527"/>
+    <hyperlink ref="B568" r:id="rId1528"/>
+    <hyperlink ref="B569" r:id="rId1529"/>
+    <hyperlink ref="B570" r:id="rId1530"/>
+    <hyperlink ref="B571" r:id="rId1531"/>
+    <hyperlink ref="B572" r:id="rId1532"/>
+    <hyperlink ref="B573" r:id="rId1533"/>
+    <hyperlink ref="B574" r:id="rId1534"/>
+    <hyperlink ref="B575" r:id="rId1535"/>
+    <hyperlink ref="B576" r:id="rId1536"/>
+    <hyperlink ref="B577" r:id="rId1537"/>
+    <hyperlink ref="B578" r:id="rId1538"/>
+    <hyperlink ref="B579" r:id="rId1539"/>
+    <hyperlink ref="B580" r:id="rId1540"/>
+    <hyperlink ref="B581" r:id="rId1541"/>
+    <hyperlink ref="B582" r:id="rId1542"/>
+    <hyperlink ref="B583" r:id="rId1543"/>
+    <hyperlink ref="B584" r:id="rId1544"/>
+    <hyperlink ref="B585" r:id="rId1545"/>
+    <hyperlink ref="B586" r:id="rId1546"/>
+    <hyperlink ref="B587" r:id="rId1547"/>
+    <hyperlink ref="B588" r:id="rId1548"/>
+    <hyperlink ref="B589" r:id="rId1549"/>
+    <hyperlink ref="B590" r:id="rId1550"/>
+    <hyperlink ref="B591" r:id="rId1551"/>
+    <hyperlink ref="B592" r:id="rId1552"/>
+    <hyperlink ref="B593" r:id="rId1553"/>
+    <hyperlink ref="B594" r:id="rId1554"/>
+    <hyperlink ref="B595" r:id="rId1555"/>
+    <hyperlink ref="B596" r:id="rId1556"/>
+    <hyperlink ref="B597" r:id="rId1557"/>
+    <hyperlink ref="B598" r:id="rId1558"/>
+    <hyperlink ref="B599" r:id="rId1559"/>
+    <hyperlink ref="B600" r:id="rId1560"/>
+    <hyperlink ref="B601" r:id="rId1561"/>
+    <hyperlink ref="B602" r:id="rId1562"/>
+    <hyperlink ref="B603" r:id="rId1563"/>
+    <hyperlink ref="B604" r:id="rId1564"/>
+    <hyperlink ref="B605" r:id="rId1565"/>
+    <hyperlink ref="B606" r:id="rId1566"/>
+    <hyperlink ref="B607" r:id="rId1567"/>
+    <hyperlink ref="B608" r:id="rId1568"/>
+    <hyperlink ref="B609" r:id="rId1569"/>
+    <hyperlink ref="B610" r:id="rId1570"/>
+    <hyperlink ref="B611" r:id="rId1571"/>
+    <hyperlink ref="B612" r:id="rId1572"/>
+    <hyperlink ref="B613" r:id="rId1573"/>
+    <hyperlink ref="B614" r:id="rId1574"/>
+    <hyperlink ref="B615" r:id="rId1575"/>
+    <hyperlink ref="B616" r:id="rId1576"/>
+    <hyperlink ref="B617" r:id="rId1577"/>
+    <hyperlink ref="B618" r:id="rId1578"/>
+    <hyperlink ref="B619" r:id="rId1579"/>
+    <hyperlink ref="B620" r:id="rId1580"/>
+    <hyperlink ref="B621" r:id="rId1581"/>
+    <hyperlink ref="B622" r:id="rId1582"/>
+    <hyperlink ref="B623" r:id="rId1583"/>
+    <hyperlink ref="B624" r:id="rId1584"/>
+    <hyperlink ref="B625" r:id="rId1585"/>
+    <hyperlink ref="B626" r:id="rId1586"/>
+    <hyperlink ref="B627" r:id="rId1587"/>
+    <hyperlink ref="B628" r:id="rId1588"/>
+    <hyperlink ref="B629" r:id="rId1589"/>
+    <hyperlink ref="B630" r:id="rId1590"/>
+    <hyperlink ref="B631" r:id="rId1591"/>
+    <hyperlink ref="B632" r:id="rId1592"/>
+    <hyperlink ref="B633" r:id="rId1593"/>
+    <hyperlink ref="B634" r:id="rId1594"/>
+    <hyperlink ref="B635" r:id="rId1595"/>
+    <hyperlink ref="B636" r:id="rId1596"/>
+    <hyperlink ref="B637" r:id="rId1597"/>
+    <hyperlink ref="B638" r:id="rId1598"/>
+    <hyperlink ref="B639" r:id="rId1599"/>
+    <hyperlink ref="B640" r:id="rId1600"/>
+    <hyperlink ref="B641" r:id="rId1601"/>
+    <hyperlink ref="B642" r:id="rId1602"/>
+    <hyperlink ref="B643" r:id="rId1603"/>
+    <hyperlink ref="B644" r:id="rId1604"/>
+    <hyperlink ref="B645" r:id="rId1605"/>
+    <hyperlink ref="B646" r:id="rId1606"/>
+    <hyperlink ref="B647" r:id="rId1607"/>
+    <hyperlink ref="B648" r:id="rId1608"/>
+    <hyperlink ref="B649" r:id="rId1609"/>
+    <hyperlink ref="B650" r:id="rId1610"/>
+    <hyperlink ref="B651" r:id="rId1611"/>
+    <hyperlink ref="B652" r:id="rId1612"/>
+    <hyperlink ref="B653" r:id="rId1613"/>
+    <hyperlink ref="B654" r:id="rId1614"/>
+    <hyperlink ref="B655" r:id="rId1615"/>
+    <hyperlink ref="B656" r:id="rId1616"/>
+    <hyperlink ref="B657" r:id="rId1617"/>
+    <hyperlink ref="B658" r:id="rId1618"/>
+    <hyperlink ref="B659" r:id="rId1619"/>
+    <hyperlink ref="B660" r:id="rId1620"/>
+    <hyperlink ref="B661" r:id="rId1621"/>
+    <hyperlink ref="B662" r:id="rId1622"/>
+    <hyperlink ref="B663" r:id="rId1623"/>
+    <hyperlink ref="B664" r:id="rId1624"/>
+    <hyperlink ref="B665" r:id="rId1625"/>
+    <hyperlink ref="B666" r:id="rId1626"/>
+    <hyperlink ref="B667" r:id="rId1627"/>
+    <hyperlink ref="B668" r:id="rId1628"/>
+    <hyperlink ref="B669" r:id="rId1629"/>
+    <hyperlink ref="B670" r:id="rId1630"/>
+    <hyperlink ref="B671" r:id="rId1631"/>
+    <hyperlink ref="B672" r:id="rId1632"/>
+    <hyperlink ref="B673" r:id="rId1633"/>
+    <hyperlink ref="B674" r:id="rId1634"/>
+    <hyperlink ref="B675" r:id="rId1635"/>
+    <hyperlink ref="B676" r:id="rId1636"/>
+    <hyperlink ref="B677" r:id="rId1637"/>
+    <hyperlink ref="B678" r:id="rId1638"/>
+    <hyperlink ref="B679" r:id="rId1639"/>
+    <hyperlink ref="B680" r:id="rId1640"/>
+    <hyperlink ref="B681" r:id="rId1641"/>
+    <hyperlink ref="B682" r:id="rId1642"/>
+    <hyperlink ref="B683" r:id="rId1643"/>
+    <hyperlink ref="B684" r:id="rId1644"/>
+    <hyperlink ref="B685" r:id="rId1645"/>
+    <hyperlink ref="B686" r:id="rId1646"/>
+    <hyperlink ref="B687" r:id="rId1647"/>
+    <hyperlink ref="B688" r:id="rId1648"/>
+    <hyperlink ref="B689" r:id="rId1649"/>
+    <hyperlink ref="B690" r:id="rId1650"/>
+    <hyperlink ref="B691" r:id="rId1651"/>
+    <hyperlink ref="B692" r:id="rId1652"/>
+    <hyperlink ref="B693" r:id="rId1653"/>
+    <hyperlink ref="B694" r:id="rId1654"/>
+    <hyperlink ref="B695" r:id="rId1655"/>
+    <hyperlink ref="B696" r:id="rId1656"/>
+    <hyperlink ref="B697" r:id="rId1657"/>
+    <hyperlink ref="B698" r:id="rId1658"/>
+    <hyperlink ref="B699" r:id="rId1659"/>
+    <hyperlink ref="B700" r:id="rId1660"/>
+    <hyperlink ref="B701" r:id="rId1661"/>
+    <hyperlink ref="B702" r:id="rId1662"/>
+    <hyperlink ref="B703" r:id="rId1663"/>
+    <hyperlink ref="B704" r:id="rId1664"/>
+    <hyperlink ref="B705" r:id="rId1665"/>
+    <hyperlink ref="B706" r:id="rId1666"/>
+    <hyperlink ref="B707" r:id="rId1667"/>
+    <hyperlink ref="B708" r:id="rId1668"/>
+    <hyperlink ref="B709" r:id="rId1669"/>
+    <hyperlink ref="B710" r:id="rId1670"/>
+    <hyperlink ref="B711" r:id="rId1671"/>
+    <hyperlink ref="B712" r:id="rId1672"/>
+    <hyperlink ref="B713" r:id="rId1673"/>
+    <hyperlink ref="B714" r:id="rId1674"/>
+    <hyperlink ref="B715" r:id="rId1675"/>
+    <hyperlink ref="B716" r:id="rId1676"/>
+    <hyperlink ref="B717" r:id="rId1677"/>
+    <hyperlink ref="B718" r:id="rId1678"/>
+    <hyperlink ref="B719" r:id="rId1679"/>
+    <hyperlink ref="B720" r:id="rId1680"/>
+    <hyperlink ref="B721" r:id="rId1681"/>
+    <hyperlink ref="B722" r:id="rId1682"/>
+    <hyperlink ref="B723" r:id="rId1683"/>
+    <hyperlink ref="B724" r:id="rId1684"/>
+    <hyperlink ref="B725" r:id="rId1685"/>
+    <hyperlink ref="B726" r:id="rId1686"/>
+    <hyperlink ref="B727" r:id="rId1687"/>
+    <hyperlink ref="B728" r:id="rId1688"/>
+    <hyperlink ref="B729" r:id="rId1689"/>
+    <hyperlink ref="B730" r:id="rId1690"/>
+    <hyperlink ref="B731" r:id="rId1691"/>
+    <hyperlink ref="B732" r:id="rId1692"/>
+    <hyperlink ref="B733" r:id="rId1693"/>
+    <hyperlink ref="B734" r:id="rId1694"/>
+    <hyperlink ref="B735" r:id="rId1695"/>
+    <hyperlink ref="B736" r:id="rId1696"/>
+    <hyperlink ref="B737" r:id="rId1697"/>
+    <hyperlink ref="B738" r:id="rId1698"/>
+    <hyperlink ref="B739" r:id="rId1699"/>
+    <hyperlink ref="B740" r:id="rId1700"/>
+    <hyperlink ref="B741" r:id="rId1701"/>
+    <hyperlink ref="B742" r:id="rId1702"/>
+    <hyperlink ref="B743" r:id="rId1703"/>
+    <hyperlink ref="B744" r:id="rId1704"/>
+    <hyperlink ref="B745" r:id="rId1705"/>
+    <hyperlink ref="B746" r:id="rId1706"/>
+    <hyperlink ref="B747" r:id="rId1707"/>
+    <hyperlink ref="B748" r:id="rId1708"/>
+    <hyperlink ref="B749" r:id="rId1709"/>
+    <hyperlink ref="B750" r:id="rId1710"/>
+    <hyperlink ref="B751" r:id="rId1711"/>
+    <hyperlink ref="B752" r:id="rId1712"/>
+    <hyperlink ref="B753" r:id="rId1713"/>
+    <hyperlink ref="B754" r:id="rId1714"/>
+    <hyperlink ref="B755" r:id="rId1715"/>
+    <hyperlink ref="B756" r:id="rId1716"/>
+    <hyperlink ref="B757" r:id="rId1717"/>
+    <hyperlink ref="B758" r:id="rId1718"/>
+    <hyperlink ref="B759" r:id="rId1719"/>
+    <hyperlink ref="B760" r:id="rId1720"/>
+    <hyperlink ref="B761" r:id="rId1721"/>
+    <hyperlink ref="B762" r:id="rId1722"/>
+    <hyperlink ref="B763" r:id="rId1723"/>
+    <hyperlink ref="B764" r:id="rId1724"/>
+    <hyperlink ref="B765" r:id="rId1725"/>
+    <hyperlink ref="B766" r:id="rId1726"/>
+    <hyperlink ref="B767" r:id="rId1727"/>
+    <hyperlink ref="B768" r:id="rId1728"/>
+    <hyperlink ref="B769" r:id="rId1729"/>
+    <hyperlink ref="B770" r:id="rId1730"/>
+    <hyperlink ref="B771" r:id="rId1731"/>
+    <hyperlink ref="B772" r:id="rId1732"/>
+    <hyperlink ref="B773" r:id="rId1733"/>
+    <hyperlink ref="B774" r:id="rId1734"/>
+    <hyperlink ref="B775" r:id="rId1735"/>
+    <hyperlink ref="B776" r:id="rId1736"/>
+    <hyperlink ref="B777" r:id="rId1737"/>
+    <hyperlink ref="B778" r:id="rId1738"/>
+    <hyperlink ref="B779" r:id="rId1739"/>
+    <hyperlink ref="B780" r:id="rId1740"/>
+    <hyperlink ref="B781" r:id="rId1741"/>
+    <hyperlink ref="B782" r:id="rId1742"/>
+    <hyperlink ref="B783" r:id="rId1743"/>
+    <hyperlink ref="B784" r:id="rId1744"/>
+    <hyperlink ref="B785" r:id="rId1745"/>
+    <hyperlink ref="B786" r:id="rId1746"/>
+    <hyperlink ref="B787" r:id="rId1747"/>
+    <hyperlink ref="B788" r:id="rId1748"/>
+    <hyperlink ref="B789" r:id="rId1749"/>
+    <hyperlink ref="B790" r:id="rId1750"/>
+    <hyperlink ref="B791" r:id="rId1751"/>
+    <hyperlink ref="B792" r:id="rId1752"/>
+    <hyperlink ref="B793" r:id="rId1753"/>
+    <hyperlink ref="B794" r:id="rId1754"/>
+    <hyperlink ref="B795" r:id="rId1755"/>
+    <hyperlink ref="B796" r:id="rId1756"/>
+    <hyperlink ref="B797" r:id="rId1757"/>
+    <hyperlink ref="B798" r:id="rId1758"/>
+    <hyperlink ref="B799" r:id="rId1759"/>
+    <hyperlink ref="B800" r:id="rId1760"/>
+    <hyperlink ref="B801" r:id="rId1761"/>
+    <hyperlink ref="B802" r:id="rId1762"/>
+    <hyperlink ref="B803" r:id="rId1763"/>
+    <hyperlink ref="B804" r:id="rId1764"/>
+    <hyperlink ref="B805" r:id="rId1765"/>
+    <hyperlink ref="B806" r:id="rId1766"/>
+    <hyperlink ref="B807" r:id="rId1767"/>
+    <hyperlink ref="B808" r:id="rId1768"/>
+    <hyperlink ref="B809" r:id="rId1769"/>
+    <hyperlink ref="B810" r:id="rId1770"/>
+    <hyperlink ref="B811" r:id="rId1771"/>
+    <hyperlink ref="B812" r:id="rId1772"/>
+    <hyperlink ref="B813" r:id="rId1773"/>
+    <hyperlink ref="B814" r:id="rId1774"/>
+    <hyperlink ref="B815" r:id="rId1775"/>
+    <hyperlink ref="B816" r:id="rId1776"/>
+    <hyperlink ref="B817" r:id="rId1777"/>
+    <hyperlink ref="B818" r:id="rId1778"/>
+    <hyperlink ref="B819" r:id="rId1779"/>
+    <hyperlink ref="B820" r:id="rId1780"/>
+    <hyperlink ref="B821" r:id="rId1781"/>
+    <hyperlink ref="B822" r:id="rId1782"/>
+    <hyperlink ref="B823" r:id="rId1783"/>
+    <hyperlink ref="B824" r:id="rId1784"/>
+    <hyperlink ref="B825" r:id="rId1785"/>
+    <hyperlink ref="B826" r:id="rId1786"/>
+    <hyperlink ref="B827" r:id="rId1787"/>
+    <hyperlink ref="B828" r:id="rId1788"/>
+    <hyperlink ref="B829" r:id="rId1789"/>
+    <hyperlink ref="B830" r:id="rId1790"/>
+    <hyperlink ref="B831" r:id="rId1791"/>
+    <hyperlink ref="B832" r:id="rId1792"/>
+    <hyperlink ref="B833" r:id="rId1793"/>
+    <hyperlink ref="B834" r:id="rId1794"/>
+    <hyperlink ref="B835" r:id="rId1795"/>
+    <hyperlink ref="B836" r:id="rId1796"/>
+    <hyperlink ref="B837" r:id="rId1797"/>
+    <hyperlink ref="B838" r:id="rId1798"/>
+    <hyperlink ref="B839" r:id="rId1799"/>
+    <hyperlink ref="B840" r:id="rId1800"/>
+    <hyperlink ref="B841" r:id="rId1801"/>
+    <hyperlink ref="B842" r:id="rId1802"/>
+    <hyperlink ref="B843" r:id="rId1803"/>
+    <hyperlink ref="B844" r:id="rId1804"/>
+    <hyperlink ref="B845" r:id="rId1805"/>
+    <hyperlink ref="B846" r:id="rId1806"/>
+    <hyperlink ref="B847" r:id="rId1807"/>
+    <hyperlink ref="B848" r:id="rId1808"/>
+    <hyperlink ref="B849" r:id="rId1809"/>
+    <hyperlink ref="B850" r:id="rId1810"/>
+    <hyperlink ref="B851" r:id="rId1811"/>
+    <hyperlink ref="B852" r:id="rId1812"/>
+    <hyperlink ref="B853" r:id="rId1813"/>
+    <hyperlink ref="B854" r:id="rId1814"/>
+    <hyperlink ref="B855" r:id="rId1815"/>
+    <hyperlink ref="B856" r:id="rId1816"/>
+    <hyperlink ref="B857" r:id="rId1817"/>
+    <hyperlink ref="B858" r:id="rId1818"/>
+    <hyperlink ref="B859" r:id="rId1819"/>
+    <hyperlink ref="B860" r:id="rId1820"/>
+    <hyperlink ref="B861" r:id="rId1821"/>
+    <hyperlink ref="B862" r:id="rId1822"/>
+    <hyperlink ref="B863" r:id="rId1823"/>
+    <hyperlink ref="B864" r:id="rId1824"/>
+    <hyperlink ref="B865" r:id="rId1825"/>
+    <hyperlink ref="B866" r:id="rId1826"/>
+    <hyperlink ref="B867" r:id="rId1827"/>
+    <hyperlink ref="B868" r:id="rId1828"/>
+    <hyperlink ref="B869" r:id="rId1829"/>
+    <hyperlink ref="B870" r:id="rId1830"/>
+    <hyperlink ref="B871" r:id="rId1831"/>
+    <hyperlink ref="B872" r:id="rId1832"/>
+    <hyperlink ref="B873" r:id="rId1833"/>
+    <hyperlink ref="B874" r:id="rId1834"/>
+    <hyperlink ref="B875" r:id="rId1835"/>
+    <hyperlink ref="B876" r:id="rId1836"/>
+    <hyperlink ref="B877" r:id="rId1837"/>
+    <hyperlink ref="B878" r:id="rId1838"/>
+    <hyperlink ref="B879" r:id="rId1839"/>
+    <hyperlink ref="B880" r:id="rId1840"/>
+    <hyperlink ref="B881" r:id="rId1841"/>
+    <hyperlink ref="B882" r:id="rId1842"/>
+    <hyperlink ref="B883" r:id="rId1843"/>
+    <hyperlink ref="B884" r:id="rId1844"/>
+    <hyperlink ref="B885" r:id="rId1845"/>
+    <hyperlink ref="B886" r:id="rId1846"/>
+    <hyperlink ref="B887" r:id="rId1847"/>
+    <hyperlink ref="B888" r:id="rId1848"/>
+    <hyperlink ref="B889" r:id="rId1849"/>
+    <hyperlink ref="B890" r:id="rId1850"/>
+    <hyperlink ref="B891" r:id="rId1851"/>
+    <hyperlink ref="B892" r:id="rId1852"/>
+    <hyperlink ref="B893" r:id="rId1853"/>
+    <hyperlink ref="B894" r:id="rId1854"/>
+    <hyperlink ref="B895" r:id="rId1855"/>
+    <hyperlink ref="B896" r:id="rId1856"/>
+    <hyperlink ref="B897" r:id="rId1857"/>
+    <hyperlink ref="B898" r:id="rId1858"/>
+    <hyperlink ref="B899" r:id="rId1859"/>
+    <hyperlink ref="B900" r:id="rId1860"/>
+    <hyperlink ref="B901" r:id="rId1861"/>
+    <hyperlink ref="B902" r:id="rId1862"/>
+    <hyperlink ref="B903" r:id="rId1863"/>
+    <hyperlink ref="B904" r:id="rId1864"/>
+    <hyperlink ref="B905" r:id="rId1865"/>
+    <hyperlink ref="B906" r:id="rId1866"/>
+    <hyperlink ref="B907" r:id="rId1867"/>
+    <hyperlink ref="B908" r:id="rId1868"/>
+    <hyperlink ref="B909" r:id="rId1869"/>
+    <hyperlink ref="B910" r:id="rId1870"/>
+    <hyperlink ref="B911" r:id="rId1871"/>
+    <hyperlink ref="B912" r:id="rId1872"/>
+    <hyperlink ref="B913" r:id="rId1873"/>
+    <hyperlink ref="B914" r:id="rId1874"/>
+    <hyperlink ref="B915" r:id="rId1875"/>
+    <hyperlink ref="B916" r:id="rId1876"/>
+    <hyperlink ref="B917" r:id="rId1877"/>
+    <hyperlink ref="B918" r:id="rId1878"/>
+    <hyperlink ref="B919" r:id="rId1879"/>
+    <hyperlink ref="B920" r:id="rId1880"/>
+    <hyperlink ref="B921" r:id="rId1881"/>
+    <hyperlink ref="B922" r:id="rId1882"/>
+    <hyperlink ref="B923" r:id="rId1883"/>
+    <hyperlink ref="B924" r:id="rId1884"/>
+    <hyperlink ref="B925" r:id="rId1885"/>
+    <hyperlink ref="B926" r:id="rId1886"/>
+    <hyperlink ref="B927" r:id="rId1887"/>
+    <hyperlink ref="B928" r:id="rId1888"/>
+    <hyperlink ref="B929" r:id="rId1889"/>
+    <hyperlink ref="B930" r:id="rId1890"/>
+    <hyperlink ref="B931" r:id="rId1891"/>
+    <hyperlink ref="B932" r:id="rId1892"/>
+    <hyperlink ref="B933" r:id="rId1893"/>
+    <hyperlink ref="B934" r:id="rId1894"/>
+    <hyperlink ref="B935" r:id="rId1895"/>
+    <hyperlink ref="B936" r:id="rId1896"/>
+    <hyperlink ref="B937" r:id="rId1897"/>
+    <hyperlink ref="B938" r:id="rId1898"/>
+    <hyperlink ref="B939" r:id="rId1899"/>
+    <hyperlink ref="B940" r:id="rId1900"/>
+    <hyperlink ref="B941" r:id="rId1901"/>
+    <hyperlink ref="B942" r:id="rId1902"/>
+    <hyperlink ref="B943" r:id="rId1903"/>
+    <hyperlink ref="B944" r:id="rId1904"/>
+    <hyperlink ref="B945" r:id="rId1905"/>
+    <hyperlink ref="B946" r:id="rId1906"/>
+    <hyperlink ref="B947" r:id="rId1907"/>
+    <hyperlink ref="B948" r:id="rId1908"/>
+    <hyperlink ref="B949" r:id="rId1909"/>
+    <hyperlink ref="B950" r:id="rId1910"/>
+    <hyperlink ref="B951" r:id="rId1911"/>
+    <hyperlink ref="B952" r:id="rId1912"/>
+    <hyperlink ref="B953" r:id="rId1913"/>
+    <hyperlink ref="B954" r:id="rId1914"/>
+    <hyperlink ref="B955" r:id="rId1915"/>
+    <hyperlink ref="B956" r:id="rId1916"/>
+    <hyperlink ref="B957" r:id="rId1917"/>
+    <hyperlink ref="B958" r:id="rId1918"/>
+    <hyperlink ref="B959" r:id="rId1919"/>
+    <hyperlink ref="B960" r:id="rId1920"/>
+    <hyperlink ref="B961" r:id="rId1921"/>
+    <hyperlink ref="B962" r:id="rId1922"/>
+    <hyperlink ref="B963" r:id="rId1923"/>
+    <hyperlink ref="B964" r:id="rId1924"/>
+    <hyperlink ref="B965" r:id="rId1925"/>
+    <hyperlink ref="B966" r:id="rId1926"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update: Add Dr. Bronner's with Leaping Bunny certification
</commit_message>
<xml_diff>
--- a/comprehensive_grocery_certifications_COMPLETE.xlsx
+++ b/comprehensive_grocery_certifications_COMPLETE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StardogChampion\TBL-Grocery-Scanner---DEVELOPMENT-VERSION-Active-development-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C78270-3243-4FCA-A3A5-DD37D0D566B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E18E20F-DFCB-4B77-833A-56CE8C156C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3618,10 +3618,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15098,8 +15099,11 @@
       <c r="I384" t="b">
         <v>0</v>
       </c>
-      <c r="K384" t="s">
-        <v>18</v>
+      <c r="J384" s="3">
+        <v>46229</v>
+      </c>
+      <c r="K384" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="385" spans="1:11">

</xml_diff>

<commit_message>
Update grocery certifications - all categories refined and 629 B Corp brands identified
</commit_message>
<xml_diff>
--- a/comprehensive_grocery_certifications_COMPLETE.xlsx
+++ b/comprehensive_grocery_certifications_COMPLETE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StardogChampion\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C9683DFD-4CEE-41A6-80C8-ECDD498BFA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{42C19749-577C-465E-8EC3-24F740B52F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{19469BE1-8F8D-4AFA-93D0-D5949C9BE75B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{68D0211E-86CB-4046-B700-CDB6DE671534}"/>
   </bookViews>
   <sheets>
     <sheet name="comprehensive_grocery_certifica" sheetId="1" r:id="rId1"/>
@@ -3046,10 +3046,10 @@
     <t>Sandwich bags, Food storage bags, Compostable food storage bags, Compostable trash bags, Compostable drawstring bags, Compostable bags with handles, Storage bags, Gloves</t>
   </si>
   <si>
+    <t>Annie's Homegrown</t>
+  </si>
+  <si>
     <t>en:foods</t>
-  </si>
-  <si>
-    <t>Annie's Homegrown</t>
   </si>
   <si>
     <t>Pasta, Sauces, Snacks</t>
@@ -6158,14 +6158,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{503DEF07-E9B0-477B-B1DF-394F132BDC32}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B836EE20-1FD5-4D07-9567-DC501BE74B76}">
   <dimension ref="A1:K1541"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="29.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="67.21875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -19562,7 +19557,7 @@
         <v>577</v>
       </c>
       <c r="B462" t="s">
-        <v>530</v>
+        <v>127</v>
       </c>
       <c r="D462" t="b">
         <v>1</v>
@@ -19707,7 +19702,7 @@
         <v>584</v>
       </c>
       <c r="B467" t="s">
-        <v>530</v>
+        <v>127</v>
       </c>
       <c r="D467" t="b">
         <v>1</v>
@@ -20374,7 +20369,7 @@
         <v>605</v>
       </c>
       <c r="B490" t="s">
-        <v>530</v>
+        <v>127</v>
       </c>
       <c r="D490" t="b">
         <v>1</v>
@@ -26798,7 +26793,7 @@
         <v>876</v>
       </c>
       <c r="B711" t="s">
-        <v>871</v>
+        <v>804</v>
       </c>
       <c r="D711" t="b">
         <v>1</v>
@@ -29855,7 +29850,7 @@
         <v>873</v>
       </c>
       <c r="B816" t="s">
-        <v>1008</v>
+        <v>871</v>
       </c>
       <c r="D816" t="b">
         <v>1</v>
@@ -29881,10 +29876,10 @@
     </row>
     <row r="817" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A817" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B817" t="s">
         <v>1009</v>
-      </c>
-      <c r="B817" t="s">
-        <v>1008</v>
       </c>
       <c r="D817" t="b">
         <v>0</v>
@@ -30029,7 +30024,7 @@
         <v>285</v>
       </c>
       <c r="B822" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D822" t="b">
         <v>0</v>
@@ -30174,7 +30169,7 @@
         <v>427</v>
       </c>
       <c r="B827" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D827" t="b">
         <v>0</v>
@@ -30319,7 +30314,7 @@
         <v>35</v>
       </c>
       <c r="B832" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D832" t="b">
         <v>0</v>
@@ -30348,7 +30343,7 @@
         <v>1024</v>
       </c>
       <c r="B833" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D833" t="b">
         <v>0</v>
@@ -30522,7 +30517,7 @@
         <v>1031</v>
       </c>
       <c r="B839" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D839" t="b">
         <v>0</v>
@@ -30580,7 +30575,7 @@
         <v>1032</v>
       </c>
       <c r="B841" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D841" t="b">
         <v>0</v>
@@ -30638,7 +30633,7 @@
         <v>845</v>
       </c>
       <c r="B843" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D843" t="b">
         <v>0</v>
@@ -30696,7 +30691,7 @@
         <v>1034</v>
       </c>
       <c r="B845" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D845" t="b">
         <v>0</v>
@@ -30783,7 +30778,7 @@
         <v>658</v>
       </c>
       <c r="B848" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D848" t="b">
         <v>0</v>
@@ -30841,7 +30836,7 @@
         <v>1036</v>
       </c>
       <c r="B850" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D850" t="b">
         <v>0</v>
@@ -30902,7 +30897,7 @@
         <v>1038</v>
       </c>
       <c r="B852" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D852" t="b">
         <v>0</v>
@@ -31047,7 +31042,7 @@
         <v>1041</v>
       </c>
       <c r="B857" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D857" t="b">
         <v>0</v>
@@ -31076,7 +31071,7 @@
         <v>56</v>
       </c>
       <c r="B858" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D858" t="b">
         <v>0</v>
@@ -31192,7 +31187,7 @@
         <v>1043</v>
       </c>
       <c r="B862" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D862" t="b">
         <v>0</v>
@@ -31250,7 +31245,7 @@
         <v>15</v>
       </c>
       <c r="B864" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D864" t="b">
         <v>0</v>
@@ -34252,7 +34247,7 @@
         <v>1186</v>
       </c>
       <c r="B967" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D967" t="b">
         <v>1</v>
@@ -34292,7 +34287,7 @@
         <v>1190</v>
       </c>
       <c r="B969" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D969" t="b">
         <v>1</v>
@@ -34332,7 +34327,7 @@
         <v>1192</v>
       </c>
       <c r="B971" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D971" t="b">
         <v>1</v>
@@ -34392,7 +34387,7 @@
         <v>1196</v>
       </c>
       <c r="B974" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D974" t="b">
         <v>1</v>
@@ -34432,7 +34427,7 @@
         <v>1198</v>
       </c>
       <c r="B976" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D976" t="b">
         <v>1</v>
@@ -34452,7 +34447,7 @@
         <v>1199</v>
       </c>
       <c r="B977" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D977" t="b">
         <v>1</v>
@@ -34472,7 +34467,7 @@
         <v>1200</v>
       </c>
       <c r="B978" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D978" t="b">
         <v>1</v>
@@ -34512,7 +34507,7 @@
         <v>1202</v>
       </c>
       <c r="B980" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D980" t="b">
         <v>1</v>
@@ -34532,7 +34527,7 @@
         <v>1203</v>
       </c>
       <c r="B981" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D981" t="b">
         <v>1</v>
@@ -34632,7 +34627,7 @@
         <v>1209</v>
       </c>
       <c r="B986" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D986" t="b">
         <v>1</v>
@@ -34652,7 +34647,7 @@
         <v>1210</v>
       </c>
       <c r="B987" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D987" t="b">
         <v>1</v>
@@ -34692,7 +34687,7 @@
         <v>1212</v>
       </c>
       <c r="B989" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D989" t="b">
         <v>1</v>
@@ -34732,7 +34727,7 @@
         <v>1214</v>
       </c>
       <c r="B991" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D991" t="b">
         <v>1</v>
@@ -34752,7 +34747,7 @@
         <v>1215</v>
       </c>
       <c r="B992" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D992" t="b">
         <v>1</v>
@@ -34792,7 +34787,7 @@
         <v>1217</v>
       </c>
       <c r="B994" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D994" t="b">
         <v>1</v>
@@ -34812,7 +34807,7 @@
         <v>1218</v>
       </c>
       <c r="B995" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D995" t="b">
         <v>1</v>
@@ -34832,7 +34827,7 @@
         <v>1219</v>
       </c>
       <c r="B996" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D996" t="b">
         <v>1</v>
@@ -34992,7 +34987,7 @@
         <v>1227</v>
       </c>
       <c r="B1004" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1004" t="b">
         <v>1</v>
@@ -35052,7 +35047,7 @@
         <v>1230</v>
       </c>
       <c r="B1007" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1007" t="b">
         <v>1</v>
@@ -35092,7 +35087,7 @@
         <v>1232</v>
       </c>
       <c r="B1009" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1009" t="b">
         <v>1</v>
@@ -35112,7 +35107,7 @@
         <v>1233</v>
       </c>
       <c r="B1010" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1010" t="b">
         <v>1</v>
@@ -35192,7 +35187,7 @@
         <v>1237</v>
       </c>
       <c r="B1014" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1014" t="b">
         <v>1</v>
@@ -35212,7 +35207,7 @@
         <v>1238</v>
       </c>
       <c r="B1015" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1015" t="b">
         <v>1</v>
@@ -35252,7 +35247,7 @@
         <v>1240</v>
       </c>
       <c r="B1017" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1017" t="b">
         <v>1</v>
@@ -35572,7 +35567,7 @@
         <v>1256</v>
       </c>
       <c r="B1033" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1033" t="b">
         <v>1</v>
@@ -35592,7 +35587,7 @@
         <v>1257</v>
       </c>
       <c r="B1034" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1034" t="b">
         <v>1</v>
@@ -35612,7 +35607,7 @@
         <v>1258</v>
       </c>
       <c r="B1035" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1035" t="b">
         <v>1</v>
@@ -35692,7 +35687,7 @@
         <v>1262</v>
       </c>
       <c r="B1039" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1039" t="b">
         <v>1</v>
@@ -35712,7 +35707,7 @@
         <v>1263</v>
       </c>
       <c r="B1040" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1040" t="b">
         <v>1</v>
@@ -35752,7 +35747,7 @@
         <v>1265</v>
       </c>
       <c r="B1042" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1042" t="b">
         <v>1</v>
@@ -35872,7 +35867,7 @@
         <v>1271</v>
       </c>
       <c r="B1048" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1048" t="b">
         <v>1</v>
@@ -35892,7 +35887,7 @@
         <v>1272</v>
       </c>
       <c r="B1049" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1049" t="b">
         <v>1</v>
@@ -35932,7 +35927,7 @@
         <v>1274</v>
       </c>
       <c r="B1051" t="s">
-        <v>1008</v>
+        <v>218</v>
       </c>
       <c r="D1051" t="b">
         <v>1</v>
@@ -35952,7 +35947,7 @@
         <v>1275</v>
       </c>
       <c r="B1052" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1052" t="b">
         <v>1</v>
@@ -35972,7 +35967,7 @@
         <v>1276</v>
       </c>
       <c r="B1053" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1053" t="b">
         <v>1</v>
@@ -35992,7 +35987,7 @@
         <v>1277</v>
       </c>
       <c r="B1054" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1054" t="b">
         <v>1</v>
@@ -36052,7 +36047,7 @@
         <v>1280</v>
       </c>
       <c r="B1057" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1057" t="b">
         <v>1</v>
@@ -36092,7 +36087,7 @@
         <v>1282</v>
       </c>
       <c r="B1059" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1059" t="b">
         <v>1</v>
@@ -36132,7 +36127,7 @@
         <v>1284</v>
       </c>
       <c r="B1061" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1061" t="b">
         <v>1</v>
@@ -36152,7 +36147,7 @@
         <v>1285</v>
       </c>
       <c r="B1062" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1062" t="b">
         <v>1</v>
@@ -36192,7 +36187,7 @@
         <v>1287</v>
       </c>
       <c r="B1064" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1064" t="b">
         <v>1</v>
@@ -36232,7 +36227,7 @@
         <v>1289</v>
       </c>
       <c r="B1066" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1066" t="b">
         <v>1</v>
@@ -36252,7 +36247,7 @@
         <v>1290</v>
       </c>
       <c r="B1067" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1067" t="b">
         <v>1</v>
@@ -36272,7 +36267,7 @@
         <v>1291</v>
       </c>
       <c r="B1068" t="s">
-        <v>1008</v>
+        <v>871</v>
       </c>
       <c r="D1068" t="b">
         <v>1</v>
@@ -36312,7 +36307,7 @@
         <v>1293</v>
       </c>
       <c r="B1070" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1070" t="b">
         <v>1</v>
@@ -36352,7 +36347,7 @@
         <v>1295</v>
       </c>
       <c r="B1072" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1072" t="b">
         <v>1</v>
@@ -36372,7 +36367,7 @@
         <v>1296</v>
       </c>
       <c r="B1073" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1073" t="b">
         <v>1</v>
@@ -36452,7 +36447,7 @@
         <v>1300</v>
       </c>
       <c r="B1077" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1077" t="b">
         <v>1</v>
@@ -36492,7 +36487,7 @@
         <v>1302</v>
       </c>
       <c r="B1079" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1079" t="b">
         <v>1</v>
@@ -36572,7 +36567,7 @@
         <v>1307</v>
       </c>
       <c r="B1083" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1083" t="b">
         <v>1</v>
@@ -36592,7 +36587,7 @@
         <v>1308</v>
       </c>
       <c r="B1084" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1084" t="b">
         <v>1</v>
@@ -36632,7 +36627,7 @@
         <v>1310</v>
       </c>
       <c r="B1086" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1086" t="b">
         <v>1</v>
@@ -36692,7 +36687,7 @@
         <v>1313</v>
       </c>
       <c r="B1089" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1089" t="b">
         <v>1</v>
@@ -36712,7 +36707,7 @@
         <v>1314</v>
       </c>
       <c r="B1090" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1090" t="b">
         <v>1</v>
@@ -36832,7 +36827,7 @@
         <v>1320</v>
       </c>
       <c r="B1096" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1096" t="b">
         <v>1</v>
@@ -36872,7 +36867,7 @@
         <v>1322</v>
       </c>
       <c r="B1098" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1098" t="b">
         <v>1</v>
@@ -36912,7 +36907,7 @@
         <v>1324</v>
       </c>
       <c r="B1100" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1100" t="b">
         <v>1</v>
@@ -36932,7 +36927,7 @@
         <v>1325</v>
       </c>
       <c r="B1101" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1101" t="b">
         <v>1</v>
@@ -36952,7 +36947,7 @@
         <v>1326</v>
       </c>
       <c r="B1102" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1102" t="b">
         <v>1</v>
@@ -36992,7 +36987,7 @@
         <v>1328</v>
       </c>
       <c r="B1104" t="s">
-        <v>730</v>
+        <v>1052</v>
       </c>
       <c r="D1104" t="b">
         <v>1</v>
@@ -37052,7 +37047,7 @@
         <v>1331</v>
       </c>
       <c r="B1107" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1107" t="b">
         <v>1</v>
@@ -37072,7 +37067,7 @@
         <v>1332</v>
       </c>
       <c r="B1108" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1108" t="b">
         <v>1</v>
@@ -37192,7 +37187,7 @@
         <v>1338</v>
       </c>
       <c r="B1114" t="s">
-        <v>1008</v>
+        <v>871</v>
       </c>
       <c r="D1114" t="b">
         <v>1</v>
@@ -37272,7 +37267,7 @@
         <v>1342</v>
       </c>
       <c r="B1118" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1118" t="b">
         <v>1</v>
@@ -37312,7 +37307,7 @@
         <v>1344</v>
       </c>
       <c r="B1120" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1120" t="b">
         <v>1</v>
@@ -37352,7 +37347,7 @@
         <v>1346</v>
       </c>
       <c r="B1122" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1122" t="b">
         <v>1</v>
@@ -37392,7 +37387,7 @@
         <v>1348</v>
       </c>
       <c r="B1124" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1124" t="b">
         <v>1</v>
@@ -37412,7 +37407,7 @@
         <v>1349</v>
       </c>
       <c r="B1125" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1125" t="b">
         <v>1</v>
@@ -37512,7 +37507,7 @@
         <v>1354</v>
       </c>
       <c r="B1130" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1130" t="b">
         <v>1</v>
@@ -37532,7 +37527,7 @@
         <v>1355</v>
       </c>
       <c r="B1131" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1131" t="b">
         <v>1</v>
@@ -37612,7 +37607,7 @@
         <v>1359</v>
       </c>
       <c r="B1135" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1135" t="b">
         <v>1</v>
@@ -37672,7 +37667,7 @@
         <v>1362</v>
       </c>
       <c r="B1138" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1138" t="b">
         <v>1</v>
@@ -37712,7 +37707,7 @@
         <v>1364</v>
       </c>
       <c r="B1140" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1140" t="b">
         <v>1</v>
@@ -37772,7 +37767,7 @@
         <v>1367</v>
       </c>
       <c r="B1143" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1143" t="b">
         <v>1</v>
@@ -37852,7 +37847,7 @@
         <v>1371</v>
       </c>
       <c r="B1147" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1147" t="b">
         <v>1</v>
@@ -37872,7 +37867,7 @@
         <v>1372</v>
       </c>
       <c r="B1148" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1148" t="b">
         <v>1</v>
@@ -37992,7 +37987,7 @@
         <v>1378</v>
       </c>
       <c r="B1154" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1154" t="b">
         <v>1</v>
@@ -38012,7 +38007,7 @@
         <v>1379</v>
       </c>
       <c r="B1155" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1155" t="b">
         <v>1</v>
@@ -38092,7 +38087,7 @@
         <v>1383</v>
       </c>
       <c r="B1159" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1159" t="b">
         <v>1</v>
@@ -38212,7 +38207,7 @@
         <v>1389</v>
       </c>
       <c r="B1165" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1165" t="b">
         <v>1</v>
@@ -38252,7 +38247,7 @@
         <v>1391</v>
       </c>
       <c r="B1167" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1167" t="b">
         <v>1</v>
@@ -38272,7 +38267,7 @@
         <v>1392</v>
       </c>
       <c r="B1168" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1168" t="b">
         <v>1</v>
@@ -38352,7 +38347,7 @@
         <v>1396</v>
       </c>
       <c r="B1172" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1172" t="b">
         <v>1</v>
@@ -38372,7 +38367,7 @@
         <v>1397</v>
       </c>
       <c r="B1173" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1173" t="b">
         <v>1</v>
@@ -38392,7 +38387,7 @@
         <v>1398</v>
       </c>
       <c r="B1174" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1174" t="b">
         <v>1</v>
@@ -38452,7 +38447,7 @@
         <v>1401</v>
       </c>
       <c r="B1177" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1177" t="b">
         <v>1</v>
@@ -38552,7 +38547,7 @@
         <v>1406</v>
       </c>
       <c r="B1182" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1182" t="b">
         <v>1</v>
@@ -38612,7 +38607,7 @@
         <v>1409</v>
       </c>
       <c r="B1185" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1185" t="b">
         <v>1</v>
@@ -38672,7 +38667,7 @@
         <v>1412</v>
       </c>
       <c r="B1188" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1188" t="b">
         <v>1</v>
@@ -38692,7 +38687,7 @@
         <v>1413</v>
       </c>
       <c r="B1189" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1189" t="b">
         <v>1</v>
@@ -38812,7 +38807,7 @@
         <v>1419</v>
       </c>
       <c r="B1195" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1195" t="b">
         <v>1</v>
@@ -38852,7 +38847,7 @@
         <v>1421</v>
       </c>
       <c r="B1197" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1197" t="b">
         <v>1</v>
@@ -38872,7 +38867,7 @@
         <v>1422</v>
       </c>
       <c r="B1198" t="s">
-        <v>730</v>
+        <v>63</v>
       </c>
       <c r="D1198" t="b">
         <v>1</v>
@@ -38892,7 +38887,7 @@
         <v>1423</v>
       </c>
       <c r="B1199" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1199" t="b">
         <v>1</v>
@@ -38912,7 +38907,7 @@
         <v>1424</v>
       </c>
       <c r="B1200" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1200" t="b">
         <v>1</v>
@@ -38932,7 +38927,7 @@
         <v>1425</v>
       </c>
       <c r="B1201" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1201" t="b">
         <v>1</v>
@@ -38952,7 +38947,7 @@
         <v>1426</v>
       </c>
       <c r="B1202" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1202" t="b">
         <v>1</v>
@@ -39012,7 +39007,7 @@
         <v>1429</v>
       </c>
       <c r="B1205" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1205" t="b">
         <v>1</v>
@@ -39032,7 +39027,7 @@
         <v>1430</v>
       </c>
       <c r="B1206" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1206" t="b">
         <v>1</v>
@@ -39052,7 +39047,7 @@
         <v>1431</v>
       </c>
       <c r="B1207" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1207" t="b">
         <v>1</v>
@@ -39072,7 +39067,7 @@
         <v>1432</v>
       </c>
       <c r="B1208" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1208" t="b">
         <v>1</v>
@@ -39092,7 +39087,7 @@
         <v>1433</v>
       </c>
       <c r="B1209" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1209" t="b">
         <v>1</v>
@@ -39132,7 +39127,7 @@
         <v>1435</v>
       </c>
       <c r="B1211" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1211" t="b">
         <v>1</v>
@@ -39172,7 +39167,7 @@
         <v>1437</v>
       </c>
       <c r="B1213" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1213" t="b">
         <v>1</v>
@@ -39192,7 +39187,7 @@
         <v>1438</v>
       </c>
       <c r="B1214" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1214" t="b">
         <v>1</v>
@@ -39212,7 +39207,7 @@
         <v>1439</v>
       </c>
       <c r="B1215" t="s">
-        <v>1008</v>
+        <v>871</v>
       </c>
       <c r="D1215" t="b">
         <v>1</v>
@@ -39252,7 +39247,7 @@
         <v>1441</v>
       </c>
       <c r="B1217" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1217" t="b">
         <v>1</v>
@@ -39272,7 +39267,7 @@
         <v>1442</v>
       </c>
       <c r="B1218" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1218" t="b">
         <v>1</v>
@@ -39372,7 +39367,7 @@
         <v>1447</v>
       </c>
       <c r="B1223" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1223" t="b">
         <v>1</v>
@@ -39392,7 +39387,7 @@
         <v>1448</v>
       </c>
       <c r="B1224" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1224" t="b">
         <v>1</v>
@@ -39432,7 +39427,7 @@
         <v>1450</v>
       </c>
       <c r="B1226" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1226" t="b">
         <v>1</v>
@@ -39452,7 +39447,7 @@
         <v>1451</v>
       </c>
       <c r="B1227" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1227" t="b">
         <v>1</v>
@@ -39492,7 +39487,7 @@
         <v>1453</v>
       </c>
       <c r="B1229" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1229" t="b">
         <v>1</v>
@@ -39512,7 +39507,7 @@
         <v>1454</v>
       </c>
       <c r="B1230" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1230" t="b">
         <v>1</v>
@@ -39552,7 +39547,7 @@
         <v>1456</v>
       </c>
       <c r="B1232" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1232" t="b">
         <v>1</v>
@@ -39572,7 +39567,7 @@
         <v>1457</v>
       </c>
       <c r="B1233" t="s">
-        <v>1008</v>
+        <v>218</v>
       </c>
       <c r="D1233" t="b">
         <v>1</v>
@@ -39632,7 +39627,7 @@
         <v>1460</v>
       </c>
       <c r="B1236" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1236" t="b">
         <v>1</v>
@@ -39652,7 +39647,7 @@
         <v>1461</v>
       </c>
       <c r="B1237" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1237" t="b">
         <v>1</v>
@@ -39672,7 +39667,7 @@
         <v>1462</v>
       </c>
       <c r="B1238" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1238" t="b">
         <v>1</v>
@@ -39772,7 +39767,7 @@
         <v>1467</v>
       </c>
       <c r="B1243" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1243" t="b">
         <v>1</v>
@@ -39872,7 +39867,7 @@
         <v>1472</v>
       </c>
       <c r="B1248" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1248" t="b">
         <v>1</v>
@@ -39992,7 +39987,7 @@
         <v>1478</v>
       </c>
       <c r="B1254" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1254" t="b">
         <v>1</v>
@@ -40032,7 +40027,7 @@
         <v>1480</v>
       </c>
       <c r="B1256" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1256" t="b">
         <v>1</v>
@@ -40052,7 +40047,7 @@
         <v>1481</v>
       </c>
       <c r="B1257" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1257" t="b">
         <v>1</v>
@@ -40092,7 +40087,7 @@
         <v>1483</v>
       </c>
       <c r="B1259" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1259" t="b">
         <v>1</v>
@@ -40112,7 +40107,7 @@
         <v>1484</v>
       </c>
       <c r="B1260" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1260" t="b">
         <v>1</v>
@@ -40152,7 +40147,7 @@
         <v>1486</v>
       </c>
       <c r="B1262" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1262" t="b">
         <v>1</v>
@@ -40172,7 +40167,7 @@
         <v>1487</v>
       </c>
       <c r="B1263" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1263" t="b">
         <v>1</v>
@@ -40212,7 +40207,7 @@
         <v>1489</v>
       </c>
       <c r="B1265" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1265" t="b">
         <v>1</v>
@@ -40292,7 +40287,7 @@
         <v>1493</v>
       </c>
       <c r="B1269" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1269" t="b">
         <v>1</v>
@@ -40392,7 +40387,7 @@
         <v>1498</v>
       </c>
       <c r="B1274" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1274" t="b">
         <v>1</v>
@@ -40612,7 +40607,7 @@
         <v>1509</v>
       </c>
       <c r="B1285" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1285" t="b">
         <v>1</v>
@@ -40632,7 +40627,7 @@
         <v>1510</v>
       </c>
       <c r="B1286" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1286" t="b">
         <v>1</v>
@@ -40652,7 +40647,7 @@
         <v>1511</v>
       </c>
       <c r="B1287" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1287" t="b">
         <v>1</v>
@@ -40712,7 +40707,7 @@
         <v>1514</v>
       </c>
       <c r="B1290" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1290" t="b">
         <v>1</v>
@@ -40812,7 +40807,7 @@
         <v>1519</v>
       </c>
       <c r="B1295" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1295" t="b">
         <v>1</v>
@@ -40852,7 +40847,7 @@
         <v>1521</v>
       </c>
       <c r="B1297" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1297" t="b">
         <v>1</v>
@@ -41012,7 +41007,7 @@
         <v>1529</v>
       </c>
       <c r="B1305" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1305" t="b">
         <v>1</v>
@@ -41052,7 +41047,7 @@
         <v>1531</v>
       </c>
       <c r="B1307" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1307" t="b">
         <v>1</v>
@@ -41072,7 +41067,7 @@
         <v>1532</v>
       </c>
       <c r="B1308" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1308" t="b">
         <v>1</v>
@@ -41112,7 +41107,7 @@
         <v>1534</v>
       </c>
       <c r="B1310" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1310" t="b">
         <v>1</v>
@@ -41132,7 +41127,7 @@
         <v>1535</v>
       </c>
       <c r="B1311" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1311" t="b">
         <v>1</v>
@@ -41172,7 +41167,7 @@
         <v>1537</v>
       </c>
       <c r="B1313" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1313" t="b">
         <v>1</v>
@@ -41192,7 +41187,7 @@
         <v>1538</v>
       </c>
       <c r="B1314" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1314" t="b">
         <v>1</v>
@@ -41232,7 +41227,7 @@
         <v>1540</v>
       </c>
       <c r="B1316" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1316" t="b">
         <v>1</v>
@@ -41272,7 +41267,7 @@
         <v>1542</v>
       </c>
       <c r="B1318" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1318" t="b">
         <v>1</v>
@@ -41312,7 +41307,7 @@
         <v>1544</v>
       </c>
       <c r="B1320" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1320" t="b">
         <v>1</v>
@@ -41332,7 +41327,7 @@
         <v>1545</v>
       </c>
       <c r="B1321" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1321" t="b">
         <v>1</v>
@@ -41372,7 +41367,7 @@
         <v>1547</v>
       </c>
       <c r="B1323" t="s">
-        <v>1008</v>
+        <v>871</v>
       </c>
       <c r="D1323" t="b">
         <v>1</v>
@@ -41392,7 +41387,7 @@
         <v>1548</v>
       </c>
       <c r="B1324" t="s">
-        <v>1008</v>
+        <v>402</v>
       </c>
       <c r="D1324" t="b">
         <v>1</v>
@@ -41412,7 +41407,7 @@
         <v>1549</v>
       </c>
       <c r="B1325" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1325" t="b">
         <v>1</v>
@@ -41432,7 +41427,7 @@
         <v>1550</v>
       </c>
       <c r="B1326" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1326" t="b">
         <v>1</v>
@@ -41512,7 +41507,7 @@
         <v>1554</v>
       </c>
       <c r="B1330" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1330" t="b">
         <v>1</v>
@@ -41532,7 +41527,7 @@
         <v>1555</v>
       </c>
       <c r="B1331" t="s">
-        <v>730</v>
+        <v>218</v>
       </c>
       <c r="D1331" t="b">
         <v>1</v>
@@ -41552,7 +41547,7 @@
         <v>1556</v>
       </c>
       <c r="B1332" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1332" t="b">
         <v>1</v>
@@ -41592,7 +41587,7 @@
         <v>1558</v>
       </c>
       <c r="B1334" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1334" t="b">
         <v>1</v>
@@ -41612,7 +41607,7 @@
         <v>1559</v>
       </c>
       <c r="B1335" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="D1335" t="b">
         <v>1</v>
@@ -41632,7 +41627,7 @@
         <v>1560</v>
       </c>
       <c r="B1336" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1336" t="b">
         <v>1</v>
@@ -41672,7 +41667,7 @@
         <v>1562</v>
       </c>
       <c r="B1338" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1338" t="b">
         <v>1</v>
@@ -41772,7 +41767,7 @@
         <v>1567</v>
       </c>
       <c r="B1343" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1343" t="b">
         <v>1</v>
@@ -41792,7 +41787,7 @@
         <v>1568</v>
       </c>
       <c r="B1344" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1344" t="b">
         <v>1</v>
@@ -41832,7 +41827,7 @@
         <v>1570</v>
       </c>
       <c r="B1346" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1346" t="b">
         <v>1</v>
@@ -41852,7 +41847,7 @@
         <v>1571</v>
       </c>
       <c r="B1347" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1347" t="b">
         <v>1</v>
@@ -41872,7 +41867,7 @@
         <v>1572</v>
       </c>
       <c r="B1348" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1348" t="b">
         <v>1</v>
@@ -41892,7 +41887,7 @@
         <v>1573</v>
       </c>
       <c r="B1349" t="s">
-        <v>730</v>
+        <v>336</v>
       </c>
       <c r="D1349" t="b">
         <v>1</v>
@@ -41952,7 +41947,7 @@
         <v>1576</v>
       </c>
       <c r="B1352" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1352" t="b">
         <v>1</v>
@@ -42052,7 +42047,7 @@
         <v>1581</v>
       </c>
       <c r="B1357" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1357" t="b">
         <v>1</v>
@@ -42072,7 +42067,7 @@
         <v>1582</v>
       </c>
       <c r="B1358" t="s">
-        <v>1008</v>
+        <v>218</v>
       </c>
       <c r="D1358" t="b">
         <v>1</v>
@@ -42112,7 +42107,7 @@
         <v>1584</v>
       </c>
       <c r="B1360" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1360" t="b">
         <v>1</v>
@@ -42192,7 +42187,7 @@
         <v>1588</v>
       </c>
       <c r="B1364" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1364" t="b">
         <v>1</v>
@@ -42312,7 +42307,7 @@
         <v>1594</v>
       </c>
       <c r="B1370" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1370" t="b">
         <v>1</v>
@@ -42332,7 +42327,7 @@
         <v>1595</v>
       </c>
       <c r="B1371" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1371" t="b">
         <v>1</v>
@@ -42392,7 +42387,7 @@
         <v>1598</v>
       </c>
       <c r="B1374" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1374" t="b">
         <v>1</v>
@@ -42412,7 +42407,7 @@
         <v>1599</v>
       </c>
       <c r="B1375" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1375" t="b">
         <v>1</v>
@@ -42472,7 +42467,7 @@
         <v>1602</v>
       </c>
       <c r="B1378" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1378" t="b">
         <v>1</v>
@@ -42512,7 +42507,7 @@
         <v>1604</v>
       </c>
       <c r="B1380" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1380" t="b">
         <v>1</v>
@@ -42532,7 +42527,7 @@
         <v>1605</v>
       </c>
       <c r="B1381" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1381" t="b">
         <v>1</v>
@@ -42552,7 +42547,7 @@
         <v>1606</v>
       </c>
       <c r="B1382" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1382" t="b">
         <v>1</v>
@@ -42572,7 +42567,7 @@
         <v>1607</v>
       </c>
       <c r="B1383" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1383" t="b">
         <v>1</v>
@@ -42632,7 +42627,7 @@
         <v>1610</v>
       </c>
       <c r="B1386" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1386" t="b">
         <v>1</v>
@@ -42672,7 +42667,7 @@
         <v>1612</v>
       </c>
       <c r="B1388" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1388" t="b">
         <v>1</v>
@@ -42692,7 +42687,7 @@
         <v>1613</v>
       </c>
       <c r="B1389" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1389" t="b">
         <v>1</v>
@@ -42732,7 +42727,7 @@
         <v>1615</v>
       </c>
       <c r="B1391" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1391" t="b">
         <v>1</v>
@@ -42752,7 +42747,7 @@
         <v>1616</v>
       </c>
       <c r="B1392" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1392" t="b">
         <v>1</v>
@@ -42832,7 +42827,7 @@
         <v>1620</v>
       </c>
       <c r="B1396" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1396" t="b">
         <v>1</v>
@@ -42892,7 +42887,7 @@
         <v>1623</v>
       </c>
       <c r="B1399" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1399" t="b">
         <v>1</v>
@@ -42912,7 +42907,7 @@
         <v>1624</v>
       </c>
       <c r="B1400" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1400" t="b">
         <v>1</v>
@@ -42932,7 +42927,7 @@
         <v>1625</v>
       </c>
       <c r="B1401" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1401" t="b">
         <v>1</v>
@@ -42952,7 +42947,7 @@
         <v>1626</v>
       </c>
       <c r="B1402" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="D1402" t="b">
         <v>1</v>
@@ -42972,7 +42967,7 @@
         <v>1627</v>
       </c>
       <c r="B1403" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1403" t="b">
         <v>1</v>
@@ -42992,7 +42987,7 @@
         <v>1628</v>
       </c>
       <c r="B1404" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1404" t="b">
         <v>1</v>
@@ -43012,7 +43007,7 @@
         <v>1629</v>
       </c>
       <c r="B1405" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1405" t="b">
         <v>1</v>
@@ -43052,7 +43047,7 @@
         <v>1631</v>
       </c>
       <c r="B1407" t="s">
-        <v>1008</v>
+        <v>614</v>
       </c>
       <c r="D1407" t="b">
         <v>1</v>
@@ -43072,7 +43067,7 @@
         <v>1632</v>
       </c>
       <c r="B1408" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1408" t="b">
         <v>1</v>
@@ -43092,7 +43087,7 @@
         <v>1633</v>
       </c>
       <c r="B1409" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1409" t="b">
         <v>1</v>
@@ -43112,7 +43107,7 @@
         <v>1634</v>
       </c>
       <c r="B1410" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1410" t="b">
         <v>1</v>
@@ -43172,7 +43167,7 @@
         <v>1637</v>
       </c>
       <c r="B1413" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1413" t="b">
         <v>1</v>
@@ -43212,7 +43207,7 @@
         <v>1639</v>
       </c>
       <c r="B1415" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1415" t="b">
         <v>1</v>
@@ -43252,7 +43247,7 @@
         <v>1641</v>
       </c>
       <c r="B1417" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1417" t="b">
         <v>1</v>
@@ -43332,7 +43327,7 @@
         <v>1645</v>
       </c>
       <c r="B1421" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1421" t="b">
         <v>1</v>
@@ -43352,7 +43347,7 @@
         <v>1646</v>
       </c>
       <c r="B1422" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1422" t="b">
         <v>1</v>
@@ -43372,7 +43367,7 @@
         <v>1647</v>
       </c>
       <c r="B1423" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1423" t="b">
         <v>1</v>
@@ -43432,7 +43427,7 @@
         <v>1650</v>
       </c>
       <c r="B1426" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1426" t="b">
         <v>1</v>
@@ -43452,7 +43447,7 @@
         <v>1651</v>
       </c>
       <c r="B1427" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1427" t="b">
         <v>1</v>
@@ -43472,7 +43467,7 @@
         <v>1652</v>
       </c>
       <c r="B1428" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1428" t="b">
         <v>1</v>
@@ -43532,7 +43527,7 @@
         <v>1655</v>
       </c>
       <c r="B1431" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1431" t="b">
         <v>1</v>
@@ -43592,7 +43587,7 @@
         <v>1658</v>
       </c>
       <c r="B1434" t="s">
-        <v>730</v>
+        <v>218</v>
       </c>
       <c r="D1434" t="b">
         <v>1</v>
@@ -43632,7 +43627,7 @@
         <v>1660</v>
       </c>
       <c r="B1436" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1436" t="b">
         <v>1</v>
@@ -43692,7 +43687,7 @@
         <v>1663</v>
       </c>
       <c r="B1439" t="s">
-        <v>1008</v>
+        <v>218</v>
       </c>
       <c r="D1439" t="b">
         <v>1</v>
@@ -43712,7 +43707,7 @@
         <v>1664</v>
       </c>
       <c r="B1440" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1440" t="b">
         <v>1</v>
@@ -43732,7 +43727,7 @@
         <v>1665</v>
       </c>
       <c r="B1441" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1441" t="b">
         <v>1</v>
@@ -43752,7 +43747,7 @@
         <v>1666</v>
       </c>
       <c r="B1442" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1442" t="b">
         <v>1</v>
@@ -43772,7 +43767,7 @@
         <v>1667</v>
       </c>
       <c r="B1443" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1443" t="b">
         <v>1</v>
@@ -43812,7 +43807,7 @@
         <v>1669</v>
       </c>
       <c r="B1445" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1445" t="b">
         <v>1</v>
@@ -43832,7 +43827,7 @@
         <v>1670</v>
       </c>
       <c r="B1446" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1446" t="b">
         <v>1</v>
@@ -43852,7 +43847,7 @@
         <v>1671</v>
       </c>
       <c r="B1447" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1447" t="b">
         <v>1</v>
@@ -43872,7 +43867,7 @@
         <v>1672</v>
       </c>
       <c r="B1448" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1448" t="b">
         <v>1</v>
@@ -43892,7 +43887,7 @@
         <v>1673</v>
       </c>
       <c r="B1449" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1449" t="b">
         <v>1</v>
@@ -43932,7 +43927,7 @@
         <v>1675</v>
       </c>
       <c r="B1451" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1451" t="b">
         <v>1</v>
@@ -43952,7 +43947,7 @@
         <v>1676</v>
       </c>
       <c r="B1452" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1452" t="b">
         <v>1</v>
@@ -44032,7 +44027,7 @@
         <v>1680</v>
       </c>
       <c r="B1456" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1456" t="b">
         <v>1</v>
@@ -44052,7 +44047,7 @@
         <v>1681</v>
       </c>
       <c r="B1457" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="D1457" t="b">
         <v>1</v>
@@ -44072,7 +44067,7 @@
         <v>1682</v>
       </c>
       <c r="B1458" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1458" t="b">
         <v>1</v>
@@ -44092,7 +44087,7 @@
         <v>1683</v>
       </c>
       <c r="B1459" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1459" t="b">
         <v>1</v>
@@ -44112,7 +44107,7 @@
         <v>1684</v>
       </c>
       <c r="B1460" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1460" t="b">
         <v>1</v>
@@ -44132,7 +44127,7 @@
         <v>1685</v>
       </c>
       <c r="B1461" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1461" t="b">
         <v>1</v>
@@ -44172,7 +44167,7 @@
         <v>1687</v>
       </c>
       <c r="B1463" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1463" t="b">
         <v>1</v>
@@ -44232,7 +44227,7 @@
         <v>1690</v>
       </c>
       <c r="B1466" t="s">
-        <v>1008</v>
+        <v>402</v>
       </c>
       <c r="D1466" t="b">
         <v>1</v>
@@ -44312,7 +44307,7 @@
         <v>1694</v>
       </c>
       <c r="B1470" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1470" t="b">
         <v>1</v>
@@ -44372,7 +44367,7 @@
         <v>1697</v>
       </c>
       <c r="B1473" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1473" t="b">
         <v>1</v>
@@ -44412,7 +44407,7 @@
         <v>1699</v>
       </c>
       <c r="B1475" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1475" t="b">
         <v>1</v>
@@ -44452,7 +44447,7 @@
         <v>1701</v>
       </c>
       <c r="B1477" t="s">
-        <v>1008</v>
+        <v>1111</v>
       </c>
       <c r="D1477" t="b">
         <v>1</v>
@@ -44492,7 +44487,7 @@
         <v>1703</v>
       </c>
       <c r="B1479" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1479" t="b">
         <v>1</v>
@@ -44552,7 +44547,7 @@
         <v>1706</v>
       </c>
       <c r="B1482" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1482" t="b">
         <v>1</v>
@@ -44612,7 +44607,7 @@
         <v>1709</v>
       </c>
       <c r="B1485" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1485" t="b">
         <v>1</v>
@@ -44632,7 +44627,7 @@
         <v>1710</v>
       </c>
       <c r="B1486" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1486" t="b">
         <v>1</v>
@@ -44672,7 +44667,7 @@
         <v>1712</v>
       </c>
       <c r="B1488" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1488" t="b">
         <v>1</v>
@@ -44732,7 +44727,7 @@
         <v>1715</v>
       </c>
       <c r="B1491" t="s">
-        <v>730</v>
+        <v>218</v>
       </c>
       <c r="D1491" t="b">
         <v>1</v>
@@ -44772,7 +44767,7 @@
         <v>1717</v>
       </c>
       <c r="B1493" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1493" t="b">
         <v>1</v>
@@ -44832,7 +44827,7 @@
         <v>1720</v>
       </c>
       <c r="B1496" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1496" t="b">
         <v>1</v>
@@ -44932,7 +44927,7 @@
         <v>1725</v>
       </c>
       <c r="B1501" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1501" t="b">
         <v>1</v>
@@ -44952,7 +44947,7 @@
         <v>1726</v>
       </c>
       <c r="B1502" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1502" t="b">
         <v>1</v>
@@ -44992,7 +44987,7 @@
         <v>1728</v>
       </c>
       <c r="B1504" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1504" t="b">
         <v>1</v>
@@ -45012,7 +45007,7 @@
         <v>1729</v>
       </c>
       <c r="B1505" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1505" t="b">
         <v>1</v>
@@ -45072,7 +45067,7 @@
         <v>1732</v>
       </c>
       <c r="B1508" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1508" t="b">
         <v>1</v>
@@ -45092,7 +45087,7 @@
         <v>1733</v>
       </c>
       <c r="B1509" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1509" t="b">
         <v>1</v>
@@ -45112,7 +45107,7 @@
         <v>1734</v>
       </c>
       <c r="B1510" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1510" t="b">
         <v>1</v>
@@ -45152,7 +45147,7 @@
         <v>1736</v>
       </c>
       <c r="B1512" t="s">
-        <v>730</v>
+        <v>1111</v>
       </c>
       <c r="D1512" t="b">
         <v>1</v>
@@ -45172,7 +45167,7 @@
         <v>1737</v>
       </c>
       <c r="B1513" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1513" t="b">
         <v>1</v>
@@ -45252,7 +45247,7 @@
         <v>1741</v>
       </c>
       <c r="B1517" t="s">
-        <v>730</v>
+        <v>941</v>
       </c>
       <c r="D1517" t="b">
         <v>1</v>
@@ -45272,7 +45267,7 @@
         <v>1742</v>
       </c>
       <c r="B1518" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1518" t="b">
         <v>1</v>
@@ -45292,7 +45287,7 @@
         <v>1743</v>
       </c>
       <c r="B1519" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1519" t="b">
         <v>1</v>
@@ -45352,7 +45347,7 @@
         <v>1746</v>
       </c>
       <c r="B1522" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1522" t="b">
         <v>1</v>
@@ -45392,7 +45387,7 @@
         <v>1748</v>
       </c>
       <c r="B1524" t="s">
-        <v>1008</v>
+        <v>127</v>
       </c>
       <c r="D1524" t="b">
         <v>1</v>
@@ -45412,7 +45407,7 @@
         <v>1749</v>
       </c>
       <c r="B1525" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="D1525" t="b">
         <v>1</v>
@@ -45432,7 +45427,7 @@
         <v>1750</v>
       </c>
       <c r="B1526" t="s">
-        <v>1008</v>
+        <v>12</v>
       </c>
       <c r="D1526" t="b">
         <v>1</v>
@@ -45472,7 +45467,7 @@
         <v>1752</v>
       </c>
       <c r="B1528" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1528" t="b">
         <v>1</v>
@@ -45532,7 +45527,7 @@
         <v>1755</v>
       </c>
       <c r="B1531" t="s">
-        <v>1008</v>
+        <v>941</v>
       </c>
       <c r="D1531" t="b">
         <v>1</v>
@@ -45572,7 +45567,7 @@
         <v>1757</v>
       </c>
       <c r="B1533" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1533" t="b">
         <v>1</v>
@@ -45592,7 +45587,7 @@
         <v>1758</v>
       </c>
       <c r="B1534" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1534" t="b">
         <v>1</v>
@@ -45612,7 +45607,7 @@
         <v>1759</v>
       </c>
       <c r="B1535" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="D1535" t="b">
         <v>1</v>
@@ -45632,7 +45627,7 @@
         <v>1760</v>
       </c>
       <c r="B1536" t="s">
-        <v>1008</v>
+        <v>336</v>
       </c>
       <c r="D1536" t="b">
         <v>1</v>
@@ -45652,7 +45647,7 @@
         <v>1761</v>
       </c>
       <c r="B1537" t="s">
-        <v>1008</v>
+        <v>804</v>
       </c>
       <c r="D1537" t="b">
         <v>1</v>
@@ -45692,7 +45687,7 @@
         <v>1763</v>
       </c>
       <c r="B1539" t="s">
-        <v>1008</v>
+        <v>1052</v>
       </c>
       <c r="D1539" t="b">
         <v>1</v>
@@ -45732,7 +45727,7 @@
         <v>1765</v>
       </c>
       <c r="B1541" t="s">
-        <v>1008</v>
+        <v>63</v>
       </c>
       <c r="D1541" t="b">
         <v>1</v>
@@ -45748,6 +45743,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>